<commit_message>
Utiliser le discriminator value/\$this plutôt que pattern/\$this
pattern et value sont tous deux déterminés via fixed[x]/pattern[x]
d'après la spec R4 (value accepte en plus le required binding) ;
value/\$this + patternCodeableConcept par slice est la convention
dominante dans l'écosystème ANS/FR-Core/IHE (ex. DiagnosticReport.category
dans ans.fhir.fr.document-core, AuditEvent.subtype dans les profils
IHE MHD), alors que pattern/\$this est plutôt l'usage observé côté IPS.
Alignement sur la convention du dépôt, sans changement de comportement. 6cae2fca49a9c47418f482aa9512581dca083f59
</commit_message>
<xml_diff>
--- a/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-06T13:28:00+00:00</t>
+    <t>2026-08-06T13:33:58+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1247,7 +1247,7 @@
     <t>Use of the Health Care Privacy/Security Classification (HCS) system of security-tag use is recommended.</t>
   </si>
   <si>
-    <t xml:space="preserve">pattern:$this}
+    <t xml:space="preserve">value:$this}
 </t>
   </si>
   <si>

</xml_diff>

<commit_message>
Retirer le pattern redondant sur confidentiality, MAJ description slicing
confidentiality est bindé (required) sur un ValueSet fermé/énuméré
(v3-ConfidentialityClassification, 6 codes), ce qui suffit à lui seul
comme mécanisme de discrimination pour le discriminator "value" au
sens de la spec R4 (fixed[x], pattern[x] ou required ValueSet
énuméré). Le patternCodeableConcept.coding.system devenait redondant.
Met à jour la description du slicing pour refléter que les deux
slices sont désormais discriminées par des mécanismes différents. 9095d3146e03a4c8d13133e1a7c9c14e0d0eaa04
</commit_message>
<xml_diff>
--- a/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4295" uniqueCount="777">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4295" uniqueCount="776">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-06T13:33:58+00:00</t>
+    <t>2026-08-06T13:37:30+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1251,7 +1251,7 @@
 </t>
   </si>
   <si>
-    <t>Slice sur securityLabel (pattern sur coding.system) pour distinguer le niveau de confidentialité (NRV) du statut de visibilité complémentaire (TRE A07)</t>
+    <t>Slice sur securityLabel pour distinguer le niveau de confidentialité (NRV) du statut de visibilité complémentaire (TRE A07) : confidentiality est discriminée par son required binding (ValueSet fermé v3-ConfidentialityClassification), visibilityStatus par un pattern sur coding.system (JDV_J110-StatutVisibiliteDocument-CISIS)</t>
   </si>
   <si>
     <t>niveauConfidentialite : [0..*] code</t>
@@ -1279,13 +1279,6 @@
   </si>
   <si>
     <t>Niveau de confidentialité standard du document (Normal, Restreint, Très restreint).</t>
-  </si>
-  <si>
-    <t>&lt;valueCodeableConcept xmlns="http://hl7.org/fhir"&gt;
-  &lt;coding&gt;
-    &lt;system value="http://terminology.hl7.org/CodeSystem/v3-Confidentiality"/&gt;
-  &lt;/coding&gt;
-&lt;/valueCodeableConcept&gt;</t>
   </si>
   <si>
     <t>http://terminology.hl7.org/ValueSet/v3-ConfidentialityClassification</t>
@@ -2794,7 +2787,7 @@
     <col min="26" max="26" width="102.93359375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="119.3046875" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="253.52734375" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="32" max="32" width="37.78125" customWidth="true" bestFit="true" hidden="true"/>
@@ -7885,7 +7878,7 @@
         <v>82</v>
       </c>
       <c r="S40" t="s" s="2">
-        <v>403</v>
+        <v>82</v>
       </c>
       <c r="T40" t="s" s="2">
         <v>82</v>
@@ -7904,7 +7897,7 @@
       </c>
       <c r="Y40" s="2"/>
       <c r="Z40" t="s" s="2">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="AA40" t="s" s="2">
         <v>82</v>
@@ -7966,13 +7959,13 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B41" t="s" s="2">
         <v>387</v>
       </c>
       <c r="C41" t="s" s="2">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D41" t="s" s="2">
         <v>82</v>
@@ -7997,7 +7990,7 @@
         <v>259</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="M41" t="s" s="2">
         <v>389</v>
@@ -8016,7 +8009,7 @@
         <v>82</v>
       </c>
       <c r="S41" t="s" s="2">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="T41" t="s" s="2">
         <v>82</v>
@@ -8035,7 +8028,7 @@
       </c>
       <c r="Y41" s="2"/>
       <c r="Z41" t="s" s="2">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="AA41" t="s" s="2">
         <v>82</v>
@@ -8097,10 +8090,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -8126,10 +8119,10 @@
         <v>341</v>
       </c>
       <c r="L42" t="s" s="2">
+        <v>410</v>
+      </c>
+      <c r="M42" t="s" s="2">
         <v>411</v>
-      </c>
-      <c r="M42" t="s" s="2">
-        <v>412</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -8180,7 +8173,7 @@
         <v>82</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>97</v>
@@ -8204,10 +8197,10 @@
         <v>82</v>
       </c>
       <c r="AN42" t="s" s="2">
+        <v>412</v>
+      </c>
+      <c r="AO42" t="s" s="2">
         <v>413</v>
-      </c>
-      <c r="AO42" t="s" s="2">
-        <v>414</v>
       </c>
       <c r="AP42" t="s" s="2">
         <v>82</v>
@@ -8224,10 +8217,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -8351,10 +8344,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -8480,10 +8473,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -8611,10 +8604,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -8637,13 +8630,13 @@
         <v>98</v>
       </c>
       <c r="K46" t="s" s="2">
+        <v>418</v>
+      </c>
+      <c r="L46" t="s" s="2">
         <v>419</v>
       </c>
-      <c r="L46" t="s" s="2">
+      <c r="M46" t="s" s="2">
         <v>420</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>421</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -8694,7 +8687,7 @@
         <v>82</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>97</v>
@@ -8718,30 +8711,30 @@
         <v>82</v>
       </c>
       <c r="AN46" t="s" s="2">
+        <v>421</v>
+      </c>
+      <c r="AO46" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="AP46" t="s" s="2">
         <v>422</v>
       </c>
-      <c r="AO46" t="s" s="2">
-        <v>414</v>
-      </c>
-      <c r="AP46" t="s" s="2">
+      <c r="AQ46" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR46" t="s" s="2">
         <v>423</v>
       </c>
-      <c r="AQ46" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR46" t="s" s="2">
+      <c r="AS46" t="s" s="2">
         <v>424</v>
-      </c>
-      <c r="AS46" t="s" s="2">
-        <v>425</v>
       </c>
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -8865,10 +8858,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -8994,10 +8987,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -9023,14 +9016,14 @@
         <v>175</v>
       </c>
       <c r="L49" t="s" s="2">
+        <v>428</v>
+      </c>
+      <c r="M49" t="s" s="2">
         <v>429</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>430</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" t="s" s="2">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="P49" t="s" s="2">
         <v>82</v>
@@ -9043,7 +9036,7 @@
         <v>82</v>
       </c>
       <c r="T49" t="s" s="2">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="U49" t="s" s="2">
         <v>82</v>
@@ -9058,28 +9051,28 @@
         <v>242</v>
       </c>
       <c r="Y49" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="Z49" t="s" s="2">
         <v>433</v>
       </c>
-      <c r="Z49" t="s" s="2">
+      <c r="AA49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF49" t="s" s="2">
         <v>434</v>
-      </c>
-      <c r="AA49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF49" t="s" s="2">
-        <v>435</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>83</v>
@@ -9097,25 +9090,25 @@
         <v>82</v>
       </c>
       <c r="AL49" t="s" s="2">
+        <v>435</v>
+      </c>
+      <c r="AM49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO49" t="s" s="2">
         <v>436</v>
       </c>
-      <c r="AM49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO49" t="s" s="2">
+      <c r="AP49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR49" t="s" s="2">
         <v>437</v>
-      </c>
-      <c r="AP49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR49" t="s" s="2">
-        <v>438</v>
       </c>
       <c r="AS49" t="s" s="2">
         <v>82</v>
@@ -9123,10 +9116,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -9152,14 +9145,14 @@
         <v>175</v>
       </c>
       <c r="L50" t="s" s="2">
+        <v>439</v>
+      </c>
+      <c r="M50" t="s" s="2">
         <v>440</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>441</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" t="s" s="2">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="P50" t="s" s="2">
         <v>82</v>
@@ -9172,7 +9165,7 @@
         <v>82</v>
       </c>
       <c r="T50" t="s" s="2">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="U50" t="s" s="2">
         <v>82</v>
@@ -9208,7 +9201,7 @@
         <v>82</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>83</v>
@@ -9223,19 +9216,19 @@
         <v>109</v>
       </c>
       <c r="AK50" t="s" s="2">
+        <v>444</v>
+      </c>
+      <c r="AL50" t="s" s="2">
         <v>445</v>
       </c>
-      <c r="AL50" t="s" s="2">
+      <c r="AM50" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN50" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO50" t="s" s="2">
         <v>446</v>
-      </c>
-      <c r="AM50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO50" t="s" s="2">
-        <v>447</v>
       </c>
       <c r="AP50" t="s" s="2">
         <v>82</v>
@@ -9252,10 +9245,10 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -9278,19 +9271,19 @@
         <v>82</v>
       </c>
       <c r="K51" t="s" s="2">
+        <v>448</v>
+      </c>
+      <c r="L51" t="s" s="2">
         <v>449</v>
       </c>
-      <c r="L51" t="s" s="2">
+      <c r="M51" t="s" s="2">
         <v>450</v>
       </c>
-      <c r="M51" t="s" s="2">
+      <c r="N51" t="s" s="2">
         <v>451</v>
       </c>
-      <c r="N51" t="s" s="2">
+      <c r="O51" t="s" s="2">
         <v>452</v>
-      </c>
-      <c r="O51" t="s" s="2">
-        <v>453</v>
       </c>
       <c r="P51" t="s" s="2">
         <v>82</v>
@@ -9339,7 +9332,7 @@
         <v>82</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>83</v>
@@ -9366,16 +9359,16 @@
         <v>82</v>
       </c>
       <c r="AO51" t="s" s="2">
+        <v>454</v>
+      </c>
+      <c r="AP51" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ51" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR51" t="s" s="2">
         <v>455</v>
-      </c>
-      <c r="AP51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR51" t="s" s="2">
-        <v>456</v>
       </c>
       <c r="AS51" t="s" s="2">
         <v>82</v>
@@ -9383,10 +9376,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -9409,19 +9402,19 @@
         <v>98</v>
       </c>
       <c r="K52" t="s" s="2">
+        <v>457</v>
+      </c>
+      <c r="L52" t="s" s="2">
         <v>458</v>
       </c>
-      <c r="L52" t="s" s="2">
+      <c r="M52" t="s" s="2">
         <v>459</v>
       </c>
-      <c r="M52" t="s" s="2">
+      <c r="N52" t="s" s="2">
         <v>460</v>
       </c>
-      <c r="N52" t="s" s="2">
+      <c r="O52" t="s" s="2">
         <v>461</v>
-      </c>
-      <c r="O52" t="s" s="2">
-        <v>462</v>
       </c>
       <c r="P52" t="s" s="2">
         <v>82</v>
@@ -9434,79 +9427,79 @@
         <v>82</v>
       </c>
       <c r="T52" t="s" s="2">
+        <v>462</v>
+      </c>
+      <c r="U52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF52" t="s" s="2">
         <v>463</v>
       </c>
-      <c r="U52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF52" t="s" s="2">
+      <c r="AG52" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH52" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ52" t="s" s="2">
         <v>464</v>
       </c>
-      <c r="AG52" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH52" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ52" t="s" s="2">
+      <c r="AK52" t="s" s="2">
         <v>465</v>
       </c>
-      <c r="AK52" t="s" s="2">
+      <c r="AL52" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="AL52" t="s" s="2">
+      <c r="AM52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO52" t="s" s="2">
         <v>467</v>
       </c>
-      <c r="AM52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO52" t="s" s="2">
+      <c r="AP52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR52" t="s" s="2">
         <v>468</v>
-      </c>
-      <c r="AP52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR52" t="s" s="2">
-        <v>469</v>
       </c>
       <c r="AS52" t="s" s="2">
         <v>82</v>
@@ -9514,10 +9507,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -9540,19 +9533,19 @@
         <v>98</v>
       </c>
       <c r="K53" t="s" s="2">
+        <v>470</v>
+      </c>
+      <c r="L53" t="s" s="2">
         <v>471</v>
       </c>
-      <c r="L53" t="s" s="2">
+      <c r="M53" t="s" s="2">
         <v>472</v>
       </c>
-      <c r="M53" t="s" s="2">
+      <c r="N53" t="s" s="2">
         <v>473</v>
       </c>
-      <c r="N53" t="s" s="2">
+      <c r="O53" t="s" s="2">
         <v>474</v>
-      </c>
-      <c r="O53" t="s" s="2">
-        <v>475</v>
       </c>
       <c r="P53" t="s" s="2">
         <v>82</v>
@@ -9601,7 +9594,7 @@
         <v>82</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>83</v>
@@ -9619,16 +9612,16 @@
         <v>82</v>
       </c>
       <c r="AL53" t="s" s="2">
+        <v>476</v>
+      </c>
+      <c r="AM53" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN53" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO53" t="s" s="2">
         <v>477</v>
-      </c>
-      <c r="AM53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO53" t="s" s="2">
-        <v>478</v>
       </c>
       <c r="AP53" t="s" s="2">
         <v>82</v>
@@ -9645,10 +9638,10 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -9671,19 +9664,19 @@
         <v>98</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="L54" t="s" s="2">
+        <v>479</v>
+      </c>
+      <c r="M54" t="s" s="2">
         <v>480</v>
       </c>
-      <c r="M54" t="s" s="2">
+      <c r="N54" t="s" s="2">
         <v>481</v>
       </c>
-      <c r="N54" t="s" s="2">
+      <c r="O54" t="s" s="2">
         <v>482</v>
-      </c>
-      <c r="O54" t="s" s="2">
-        <v>483</v>
       </c>
       <c r="P54" t="s" s="2">
         <v>82</v>
@@ -9732,7 +9725,7 @@
         <v>82</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>83</v>
@@ -9750,16 +9743,16 @@
         <v>82</v>
       </c>
       <c r="AL54" t="s" s="2">
+        <v>484</v>
+      </c>
+      <c r="AM54" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN54" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO54" t="s" s="2">
         <v>485</v>
-      </c>
-      <c r="AM54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO54" t="s" s="2">
-        <v>486</v>
       </c>
       <c r="AP54" t="s" s="2">
         <v>82</v>
@@ -9776,10 +9769,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -9805,14 +9798,14 @@
         <v>111</v>
       </c>
       <c r="L55" t="s" s="2">
+        <v>487</v>
+      </c>
+      <c r="M55" t="s" s="2">
         <v>488</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>489</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" t="s" s="2">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="P55" t="s" s="2">
         <v>82</v>
@@ -9825,43 +9818,43 @@
         <v>82</v>
       </c>
       <c r="T55" t="s" s="2">
+        <v>490</v>
+      </c>
+      <c r="U55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF55" t="s" s="2">
         <v>491</v>
-      </c>
-      <c r="U55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF55" t="s" s="2">
-        <v>492</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>83</v>
@@ -9876,19 +9869,19 @@
         <v>109</v>
       </c>
       <c r="AK55" t="s" s="2">
+        <v>492</v>
+      </c>
+      <c r="AL55" t="s" s="2">
         <v>493</v>
       </c>
-      <c r="AL55" t="s" s="2">
+      <c r="AM55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO55" t="s" s="2">
         <v>494</v>
-      </c>
-      <c r="AM55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO55" t="s" s="2">
-        <v>495</v>
       </c>
       <c r="AP55" t="s" s="2">
         <v>82</v>
@@ -9905,10 +9898,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -9931,17 +9924,17 @@
         <v>98</v>
       </c>
       <c r="K56" t="s" s="2">
+        <v>496</v>
+      </c>
+      <c r="L56" t="s" s="2">
         <v>497</v>
       </c>
-      <c r="L56" t="s" s="2">
+      <c r="M56" t="s" s="2">
         <v>498</v>
-      </c>
-      <c r="M56" t="s" s="2">
-        <v>499</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" t="s" s="2">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="P56" t="s" s="2">
         <v>82</v>
@@ -9990,7 +9983,7 @@
         <v>82</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>83</v>
@@ -10005,11 +9998,11 @@
         <v>109</v>
       </c>
       <c r="AK56" t="s" s="2">
+        <v>501</v>
+      </c>
+      <c r="AL56" t="s" s="2">
         <v>502</v>
       </c>
-      <c r="AL56" t="s" s="2">
-        <v>503</v>
-      </c>
       <c r="AM56" t="s" s="2">
         <v>82</v>
       </c>
@@ -10017,7 +10010,7 @@
         <v>82</v>
       </c>
       <c r="AO56" t="s" s="2">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="AP56" t="s" s="2">
         <v>82</v>
@@ -10034,10 +10027,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -10063,13 +10056,13 @@
         <v>153</v>
       </c>
       <c r="L57" t="s" s="2">
+        <v>504</v>
+      </c>
+      <c r="M57" t="s" s="2">
         <v>505</v>
       </c>
-      <c r="M57" t="s" s="2">
+      <c r="N57" t="s" s="2">
         <v>506</v>
-      </c>
-      <c r="N57" t="s" s="2">
-        <v>507</v>
       </c>
       <c r="O57" s="2"/>
       <c r="P57" t="s" s="2">
@@ -10099,56 +10092,56 @@
       </c>
       <c r="Y57" s="2"/>
       <c r="Z57" t="s" s="2">
+        <v>507</v>
+      </c>
+      <c r="AA57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF57" t="s" s="2">
+        <v>503</v>
+      </c>
+      <c r="AG57" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH57" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ57" t="s" s="2">
         <v>508</v>
       </c>
-      <c r="AA57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF57" t="s" s="2">
-        <v>504</v>
-      </c>
-      <c r="AG57" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH57" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ57" t="s" s="2">
+      <c r="AK57" t="s" s="2">
         <v>509</v>
       </c>
-      <c r="AK57" t="s" s="2">
+      <c r="AL57" t="s" s="2">
         <v>510</v>
       </c>
-      <c r="AL57" t="s" s="2">
+      <c r="AM57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN57" t="s" s="2">
         <v>511</v>
       </c>
-      <c r="AM57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN57" t="s" s="2">
+      <c r="AO57" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="AP57" t="s" s="2">
         <v>512</v>
       </c>
-      <c r="AO57" t="s" s="2">
-        <v>414</v>
-      </c>
-      <c r="AP57" t="s" s="2">
-        <v>513</v>
-      </c>
       <c r="AQ57" t="s" s="2">
         <v>82</v>
       </c>
@@ -10156,15 +10149,15 @@
         <v>82</v>
       </c>
       <c r="AS57" t="s" s="2">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -10190,13 +10183,13 @@
         <v>341</v>
       </c>
       <c r="L58" t="s" s="2">
+        <v>514</v>
+      </c>
+      <c r="M58" t="s" s="2">
         <v>515</v>
       </c>
-      <c r="M58" t="s" s="2">
+      <c r="N58" t="s" s="2">
         <v>516</v>
-      </c>
-      <c r="N58" t="s" s="2">
-        <v>517</v>
       </c>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
@@ -10246,7 +10239,7 @@
         <v>82</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>83</v>
@@ -10273,7 +10266,7 @@
         <v>82</v>
       </c>
       <c r="AO58" t="s" s="2">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="AP58" t="s" s="2">
         <v>82</v>
@@ -10290,10 +10283,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -10417,10 +10410,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -10546,10 +10539,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -10677,10 +10670,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -10703,13 +10696,13 @@
         <v>82</v>
       </c>
       <c r="K62" t="s" s="2">
+        <v>522</v>
+      </c>
+      <c r="L62" t="s" s="2">
         <v>523</v>
       </c>
-      <c r="L62" t="s" s="2">
+      <c r="M62" t="s" s="2">
         <v>524</v>
-      </c>
-      <c r="M62" t="s" s="2">
-        <v>525</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -10760,7 +10753,7 @@
         <v>82</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>83</v>
@@ -10778,22 +10771,22 @@
         <v>82</v>
       </c>
       <c r="AL62" t="s" s="2">
+        <v>525</v>
+      </c>
+      <c r="AM62" t="s" s="2">
         <v>526</v>
       </c>
-      <c r="AM62" t="s" s="2">
+      <c r="AN62" t="s" s="2">
         <v>527</v>
       </c>
-      <c r="AN62" t="s" s="2">
+      <c r="AO62" t="s" s="2">
         <v>528</v>
       </c>
-      <c r="AO62" t="s" s="2">
+      <c r="AP62" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ62" t="s" s="2">
         <v>529</v>
-      </c>
-      <c r="AP62" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ62" t="s" s="2">
-        <v>530</v>
       </c>
       <c r="AR62" t="s" s="2">
         <v>82</v>
@@ -10804,10 +10797,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -10833,13 +10826,13 @@
         <v>259</v>
       </c>
       <c r="L63" t="s" s="2">
+        <v>531</v>
+      </c>
+      <c r="M63" t="s" s="2">
         <v>532</v>
       </c>
-      <c r="M63" t="s" s="2">
+      <c r="N63" t="s" s="2">
         <v>533</v>
-      </c>
-      <c r="N63" t="s" s="2">
-        <v>534</v>
       </c>
       <c r="O63" s="2"/>
       <c r="P63" t="s" s="2">
@@ -10868,11 +10861,11 @@
         <v>165</v>
       </c>
       <c r="Y63" t="s" s="2">
+        <v>534</v>
+      </c>
+      <c r="Z63" t="s" s="2">
         <v>535</v>
       </c>
-      <c r="Z63" t="s" s="2">
-        <v>536</v>
-      </c>
       <c r="AA63" t="s" s="2">
         <v>82</v>
       </c>
@@ -10889,7 +10882,7 @@
         <v>82</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>83</v>
@@ -10901,23 +10894,23 @@
         <v>82</v>
       </c>
       <c r="AJ63" t="s" s="2">
+        <v>536</v>
+      </c>
+      <c r="AK63" t="s" s="2">
         <v>537</v>
       </c>
-      <c r="AK63" t="s" s="2">
+      <c r="AL63" t="s" s="2">
         <v>538</v>
       </c>
-      <c r="AL63" t="s" s="2">
+      <c r="AM63" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN63" t="s" s="2">
         <v>539</v>
       </c>
-      <c r="AM63" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN63" t="s" s="2">
+      <c r="AO63" t="s" s="2">
         <v>540</v>
       </c>
-      <c r="AO63" t="s" s="2">
-        <v>541</v>
-      </c>
       <c r="AP63" t="s" s="2">
         <v>82</v>
       </c>
@@ -10928,15 +10921,15 @@
         <v>82</v>
       </c>
       <c r="AS63" t="s" s="2">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -10959,13 +10952,13 @@
         <v>98</v>
       </c>
       <c r="K64" t="s" s="2">
+        <v>542</v>
+      </c>
+      <c r="L64" t="s" s="2">
         <v>543</v>
       </c>
-      <c r="L64" t="s" s="2">
+      <c r="M64" t="s" s="2">
         <v>544</v>
-      </c>
-      <c r="M64" t="s" s="2">
-        <v>545</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
@@ -11016,7 +11009,7 @@
         <v>82</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>83</v>
@@ -11040,30 +11033,30 @@
         <v>82</v>
       </c>
       <c r="AN64" t="s" s="2">
+        <v>545</v>
+      </c>
+      <c r="AO64" t="s" s="2">
         <v>546</v>
       </c>
-      <c r="AO64" t="s" s="2">
+      <c r="AP64" t="s" s="2">
         <v>547</v>
       </c>
-      <c r="AP64" t="s" s="2">
+      <c r="AQ64" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR64" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AS64" t="s" s="2">
         <v>548</v>
-      </c>
-      <c r="AQ64" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR64" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AS64" t="s" s="2">
-        <v>549</v>
       </c>
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -11187,10 +11180,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -11316,10 +11309,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -11342,16 +11335,16 @@
         <v>98</v>
       </c>
       <c r="K67" t="s" s="2">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="L67" t="s" s="2">
+        <v>552</v>
+      </c>
+      <c r="M67" t="s" s="2">
         <v>553</v>
       </c>
-      <c r="M67" t="s" s="2">
+      <c r="N67" t="s" s="2">
         <v>554</v>
-      </c>
-      <c r="N67" t="s" s="2">
-        <v>555</v>
       </c>
       <c r="O67" s="2"/>
       <c r="P67" t="s" s="2">
@@ -11401,43 +11394,43 @@
         <v>82</v>
       </c>
       <c r="AF67" t="s" s="2">
+        <v>555</v>
+      </c>
+      <c r="AG67" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH67" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI67" t="s" s="2">
         <v>556</v>
-      </c>
-      <c r="AG67" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH67" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI67" t="s" s="2">
-        <v>557</v>
       </c>
       <c r="AJ67" t="s" s="2">
         <v>109</v>
       </c>
       <c r="AK67" t="s" s="2">
+        <v>557</v>
+      </c>
+      <c r="AL67" t="s" s="2">
         <v>558</v>
       </c>
-      <c r="AL67" t="s" s="2">
+      <c r="AM67" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN67" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO67" t="s" s="2">
         <v>559</v>
       </c>
-      <c r="AM67" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN67" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO67" t="s" s="2">
+      <c r="AP67" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ67" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR67" t="s" s="2">
         <v>560</v>
-      </c>
-      <c r="AP67" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ67" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR67" t="s" s="2">
-        <v>561</v>
       </c>
       <c r="AS67" t="s" s="2">
         <v>82</v>
@@ -11445,10 +11438,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -11471,69 +11464,69 @@
         <v>98</v>
       </c>
       <c r="K68" t="s" s="2">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="L68" t="s" s="2">
+        <v>562</v>
+      </c>
+      <c r="M68" t="s" s="2">
         <v>563</v>
       </c>
-      <c r="M68" t="s" s="2">
+      <c r="N68" t="s" s="2">
         <v>564</v>
-      </c>
-      <c r="N68" t="s" s="2">
-        <v>565</v>
       </c>
       <c r="O68" s="2"/>
       <c r="P68" t="s" s="2">
         <v>82</v>
       </c>
       <c r="Q68" t="s" s="2">
+        <v>565</v>
+      </c>
+      <c r="R68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF68" t="s" s="2">
         <v>566</v>
       </c>
-      <c r="R68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF68" t="s" s="2">
-        <v>567</v>
-      </c>
       <c r="AG68" t="s" s="2">
         <v>83</v>
       </c>
@@ -11541,34 +11534,34 @@
         <v>97</v>
       </c>
       <c r="AI68" t="s" s="2">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="AJ68" t="s" s="2">
         <v>109</v>
       </c>
       <c r="AK68" t="s" s="2">
+        <v>567</v>
+      </c>
+      <c r="AL68" t="s" s="2">
         <v>568</v>
       </c>
-      <c r="AL68" t="s" s="2">
+      <c r="AM68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO68" t="s" s="2">
         <v>569</v>
       </c>
-      <c r="AM68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO68" t="s" s="2">
+      <c r="AP68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR68" t="s" s="2">
         <v>570</v>
-      </c>
-      <c r="AP68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR68" t="s" s="2">
-        <v>571</v>
       </c>
       <c r="AS68" t="s" s="2">
         <v>82</v>
@@ -11576,10 +11569,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -11605,10 +11598,10 @@
         <v>259</v>
       </c>
       <c r="L69" t="s" s="2">
+        <v>572</v>
+      </c>
+      <c r="M69" t="s" s="2">
         <v>573</v>
-      </c>
-      <c r="M69" t="s" s="2">
-        <v>574</v>
       </c>
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
@@ -11639,56 +11632,56 @@
       </c>
       <c r="Y69" s="2"/>
       <c r="Z69" t="s" s="2">
+        <v>574</v>
+      </c>
+      <c r="AA69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF69" t="s" s="2">
+        <v>571</v>
+      </c>
+      <c r="AG69" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH69" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ69" t="s" s="2">
         <v>575</v>
       </c>
-      <c r="AA69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF69" t="s" s="2">
-        <v>572</v>
-      </c>
-      <c r="AG69" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH69" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ69" t="s" s="2">
+      <c r="AK69" t="s" s="2">
         <v>576</v>
       </c>
-      <c r="AK69" t="s" s="2">
+      <c r="AL69" t="s" s="2">
         <v>577</v>
       </c>
-      <c r="AL69" t="s" s="2">
+      <c r="AM69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN69" t="s" s="2">
         <v>578</v>
       </c>
-      <c r="AM69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN69" t="s" s="2">
+      <c r="AO69" t="s" s="2">
         <v>579</v>
       </c>
-      <c r="AO69" t="s" s="2">
+      <c r="AP69" t="s" s="2">
         <v>580</v>
       </c>
-      <c r="AP69" t="s" s="2">
-        <v>581</v>
-      </c>
       <c r="AQ69" t="s" s="2">
         <v>82</v>
       </c>
@@ -11696,15 +11689,15 @@
         <v>82</v>
       </c>
       <c r="AS69" t="s" s="2">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -11730,16 +11723,16 @@
         <v>259</v>
       </c>
       <c r="L70" t="s" s="2">
+        <v>582</v>
+      </c>
+      <c r="M70" t="s" s="2">
         <v>583</v>
       </c>
-      <c r="M70" t="s" s="2">
+      <c r="N70" t="s" s="2">
         <v>584</v>
       </c>
-      <c r="N70" t="s" s="2">
+      <c r="O70" t="s" s="2">
         <v>585</v>
-      </c>
-      <c r="O70" t="s" s="2">
-        <v>586</v>
       </c>
       <c r="P70" t="s" s="2">
         <v>82</v>
@@ -11768,55 +11761,55 @@
       </c>
       <c r="Y70" s="2"/>
       <c r="Z70" t="s" s="2">
+        <v>586</v>
+      </c>
+      <c r="AA70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF70" t="s" s="2">
+        <v>581</v>
+      </c>
+      <c r="AG70" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH70" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ70" t="s" s="2">
+        <v>575</v>
+      </c>
+      <c r="AK70" t="s" s="2">
         <v>587</v>
       </c>
-      <c r="AA70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF70" t="s" s="2">
-        <v>582</v>
-      </c>
-      <c r="AG70" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH70" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ70" t="s" s="2">
-        <v>576</v>
-      </c>
-      <c r="AK70" t="s" s="2">
+      <c r="AL70" t="s" s="2">
         <v>588</v>
       </c>
-      <c r="AL70" t="s" s="2">
-        <v>589</v>
-      </c>
       <c r="AM70" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN70" t="s" s="2">
+        <v>578</v>
+      </c>
+      <c r="AO70" t="s" s="2">
         <v>579</v>
       </c>
-      <c r="AO70" t="s" s="2">
-        <v>580</v>
-      </c>
       <c r="AP70" t="s" s="2">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="AQ70" t="s" s="2">
         <v>82</v>
@@ -11825,15 +11818,15 @@
         <v>82</v>
       </c>
       <c r="AS70" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -11856,13 +11849,13 @@
         <v>82</v>
       </c>
       <c r="K71" t="s" s="2">
+        <v>590</v>
+      </c>
+      <c r="L71" t="s" s="2">
         <v>591</v>
       </c>
-      <c r="L71" t="s" s="2">
+      <c r="M71" t="s" s="2">
         <v>592</v>
-      </c>
-      <c r="M71" t="s" s="2">
-        <v>593</v>
       </c>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
@@ -11913,7 +11906,7 @@
         <v>82</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>83</v>
@@ -11952,15 +11945,15 @@
         <v>82</v>
       </c>
       <c r="AS71" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -12084,10 +12077,10 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -12213,10 +12206,10 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -12242,13 +12235,13 @@
         <v>111</v>
       </c>
       <c r="L74" t="s" s="2">
+        <v>597</v>
+      </c>
+      <c r="M74" t="s" s="2">
         <v>598</v>
       </c>
-      <c r="M74" t="s" s="2">
+      <c r="N74" t="s" s="2">
         <v>599</v>
-      </c>
-      <c r="N74" t="s" s="2">
-        <v>600</v>
       </c>
       <c r="O74" s="2"/>
       <c r="P74" t="s" s="2">
@@ -12298,16 +12291,16 @@
         <v>82</v>
       </c>
       <c r="AF74" t="s" s="2">
+        <v>600</v>
+      </c>
+      <c r="AG74" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH74" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI74" t="s" s="2">
         <v>601</v>
-      </c>
-      <c r="AG74" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH74" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI74" t="s" s="2">
-        <v>602</v>
       </c>
       <c r="AJ74" t="s" s="2">
         <v>109</v>
@@ -12316,7 +12309,7 @@
         <v>82</v>
       </c>
       <c r="AL74" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="AM74" t="s" s="2">
         <v>82</v>
@@ -12342,10 +12335,10 @@
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -12371,13 +12364,13 @@
         <v>140</v>
       </c>
       <c r="L75" t="s" s="2">
+        <v>604</v>
+      </c>
+      <c r="M75" t="s" s="2">
         <v>605</v>
       </c>
-      <c r="M75" t="s" s="2">
+      <c r="N75" t="s" s="2">
         <v>606</v>
-      </c>
-      <c r="N75" t="s" s="2">
-        <v>607</v>
       </c>
       <c r="O75" s="2"/>
       <c r="P75" t="s" s="2">
@@ -12406,28 +12399,28 @@
         <v>157</v>
       </c>
       <c r="Y75" t="s" s="2">
+        <v>607</v>
+      </c>
+      <c r="Z75" t="s" s="2">
         <v>608</v>
       </c>
-      <c r="Z75" t="s" s="2">
+      <c r="AA75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF75" t="s" s="2">
         <v>609</v>
-      </c>
-      <c r="AA75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF75" t="s" s="2">
-        <v>610</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>83</v>
@@ -12471,10 +12464,10 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -12500,13 +12493,13 @@
         <v>227</v>
       </c>
       <c r="L76" t="s" s="2">
+        <v>611</v>
+      </c>
+      <c r="M76" t="s" s="2">
         <v>612</v>
       </c>
-      <c r="M76" t="s" s="2">
+      <c r="N76" t="s" s="2">
         <v>613</v>
-      </c>
-      <c r="N76" t="s" s="2">
-        <v>614</v>
       </c>
       <c r="O76" s="2"/>
       <c r="P76" t="s" s="2">
@@ -12556,7 +12549,7 @@
         <v>82</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>83</v>
@@ -12574,16 +12567,16 @@
         <v>82</v>
       </c>
       <c r="AL76" t="s" s="2">
+        <v>615</v>
+      </c>
+      <c r="AM76" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN76" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO76" t="s" s="2">
         <v>616</v>
-      </c>
-      <c r="AM76" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN76" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO76" t="s" s="2">
-        <v>617</v>
       </c>
       <c r="AP76" t="s" s="2">
         <v>82</v>
@@ -12600,10 +12593,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -12629,13 +12622,13 @@
         <v>111</v>
       </c>
       <c r="L77" t="s" s="2">
+        <v>618</v>
+      </c>
+      <c r="M77" t="s" s="2">
         <v>619</v>
       </c>
-      <c r="M77" t="s" s="2">
+      <c r="N77" t="s" s="2">
         <v>620</v>
-      </c>
-      <c r="N77" t="s" s="2">
-        <v>621</v>
       </c>
       <c r="O77" s="2"/>
       <c r="P77" t="s" s="2">
@@ -12685,7 +12678,7 @@
         <v>82</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>83</v>
@@ -12729,10 +12722,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -12755,16 +12748,16 @@
         <v>82</v>
       </c>
       <c r="K78" t="s" s="2">
+        <v>623</v>
+      </c>
+      <c r="L78" t="s" s="2">
         <v>624</v>
       </c>
-      <c r="L78" t="s" s="2">
+      <c r="M78" t="s" s="2">
         <v>625</v>
       </c>
-      <c r="M78" t="s" s="2">
+      <c r="N78" t="s" s="2">
         <v>626</v>
-      </c>
-      <c r="N78" t="s" s="2">
-        <v>627</v>
       </c>
       <c r="O78" s="2"/>
       <c r="P78" t="s" s="2">
@@ -12802,10 +12795,10 @@
         <v>82</v>
       </c>
       <c r="AB78" t="s" s="2">
+        <v>627</v>
+      </c>
+      <c r="AC78" t="s" s="2">
         <v>628</v>
-      </c>
-      <c r="AC78" t="s" s="2">
-        <v>629</v>
       </c>
       <c r="AD78" t="s" s="2">
         <v>82</v>
@@ -12814,7 +12807,7 @@
         <v>124</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>83</v>
@@ -12832,39 +12825,39 @@
         <v>82</v>
       </c>
       <c r="AL78" t="s" s="2">
+        <v>629</v>
+      </c>
+      <c r="AM78" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN78" t="s" s="2">
         <v>630</v>
       </c>
-      <c r="AM78" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN78" t="s" s="2">
+      <c r="AO78" t="s" s="2">
         <v>631</v>
       </c>
-      <c r="AO78" t="s" s="2">
+      <c r="AP78" t="s" s="2">
         <v>632</v>
       </c>
-      <c r="AP78" t="s" s="2">
+      <c r="AQ78" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR78" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AS78" t="s" s="2">
         <v>633</v>
-      </c>
-      <c r="AQ78" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR78" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AS78" t="s" s="2">
-        <v>634</v>
       </c>
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
+        <v>634</v>
+      </c>
+      <c r="B79" t="s" s="2">
+        <v>622</v>
+      </c>
+      <c r="C79" t="s" s="2">
         <v>635</v>
-      </c>
-      <c r="B79" t="s" s="2">
-        <v>623</v>
-      </c>
-      <c r="C79" t="s" s="2">
-        <v>636</v>
       </c>
       <c r="D79" t="s" s="2">
         <v>82</v>
@@ -12886,16 +12879,16 @@
         <v>82</v>
       </c>
       <c r="K79" t="s" s="2">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="M79" t="s" s="2">
+        <v>625</v>
+      </c>
+      <c r="N79" t="s" s="2">
         <v>626</v>
-      </c>
-      <c r="N79" t="s" s="2">
-        <v>627</v>
       </c>
       <c r="O79" s="2"/>
       <c r="P79" t="s" s="2">
@@ -12945,7 +12938,7 @@
         <v>82</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>83</v>
@@ -12963,36 +12956,36 @@
         <v>82</v>
       </c>
       <c r="AL79" t="s" s="2">
+        <v>629</v>
+      </c>
+      <c r="AM79" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN79" t="s" s="2">
         <v>630</v>
       </c>
-      <c r="AM79" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN79" t="s" s="2">
+      <c r="AO79" t="s" s="2">
         <v>631</v>
       </c>
-      <c r="AO79" t="s" s="2">
+      <c r="AP79" t="s" s="2">
         <v>632</v>
       </c>
-      <c r="AP79" t="s" s="2">
+      <c r="AQ79" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR79" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AS79" t="s" s="2">
         <v>633</v>
-      </c>
-      <c r="AQ79" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR79" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AS79" t="s" s="2">
-        <v>634</v>
       </c>
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
+        <v>637</v>
+      </c>
+      <c r="B80" t="s" s="2">
         <v>638</v>
-      </c>
-      <c r="B80" t="s" s="2">
-        <v>639</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -13116,10 +13109,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
+        <v>639</v>
+      </c>
+      <c r="B81" t="s" s="2">
         <v>640</v>
-      </c>
-      <c r="B81" t="s" s="2">
-        <v>641</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -13245,10 +13238,10 @@
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
+        <v>641</v>
+      </c>
+      <c r="B82" t="s" s="2">
         <v>642</v>
-      </c>
-      <c r="B82" t="s" s="2">
-        <v>643</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -13274,13 +13267,13 @@
         <v>111</v>
       </c>
       <c r="L82" t="s" s="2">
+        <v>597</v>
+      </c>
+      <c r="M82" t="s" s="2">
         <v>598</v>
       </c>
-      <c r="M82" t="s" s="2">
+      <c r="N82" t="s" s="2">
         <v>599</v>
-      </c>
-      <c r="N82" t="s" s="2">
-        <v>600</v>
       </c>
       <c r="O82" s="2"/>
       <c r="P82" t="s" s="2">
@@ -13330,16 +13323,16 @@
         <v>82</v>
       </c>
       <c r="AF82" t="s" s="2">
+        <v>600</v>
+      </c>
+      <c r="AG82" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH82" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI82" t="s" s="2">
         <v>601</v>
-      </c>
-      <c r="AG82" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH82" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI82" t="s" s="2">
-        <v>602</v>
       </c>
       <c r="AJ82" t="s" s="2">
         <v>109</v>
@@ -13374,10 +13367,10 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
+        <v>643</v>
+      </c>
+      <c r="B83" t="s" s="2">
         <v>644</v>
-      </c>
-      <c r="B83" t="s" s="2">
-        <v>645</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -13403,13 +13396,13 @@
         <v>140</v>
       </c>
       <c r="L83" t="s" s="2">
+        <v>604</v>
+      </c>
+      <c r="M83" t="s" s="2">
         <v>605</v>
       </c>
-      <c r="M83" t="s" s="2">
+      <c r="N83" t="s" s="2">
         <v>606</v>
-      </c>
-      <c r="N83" t="s" s="2">
-        <v>607</v>
       </c>
       <c r="O83" s="2"/>
       <c r="P83" t="s" s="2">
@@ -13438,28 +13431,28 @@
         <v>157</v>
       </c>
       <c r="Y83" t="s" s="2">
+        <v>607</v>
+      </c>
+      <c r="Z83" t="s" s="2">
         <v>608</v>
       </c>
-      <c r="Z83" t="s" s="2">
+      <c r="AA83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF83" t="s" s="2">
         <v>609</v>
-      </c>
-      <c r="AA83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF83" t="s" s="2">
-        <v>610</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>83</v>
@@ -13503,10 +13496,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
+        <v>645</v>
+      </c>
+      <c r="B84" t="s" s="2">
         <v>646</v>
-      </c>
-      <c r="B84" t="s" s="2">
-        <v>647</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -13532,13 +13525,13 @@
         <v>227</v>
       </c>
       <c r="L84" t="s" s="2">
+        <v>611</v>
+      </c>
+      <c r="M84" t="s" s="2">
         <v>612</v>
       </c>
-      <c r="M84" t="s" s="2">
+      <c r="N84" t="s" s="2">
         <v>613</v>
-      </c>
-      <c r="N84" t="s" s="2">
-        <v>614</v>
       </c>
       <c r="O84" s="2"/>
       <c r="P84" t="s" s="2">
@@ -13588,7 +13581,7 @@
         <v>82</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>83</v>
@@ -13615,7 +13608,7 @@
         <v>82</v>
       </c>
       <c r="AO84" t="s" s="2">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="AP84" t="s" s="2">
         <v>82</v>
@@ -13632,10 +13625,10 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
+        <v>647</v>
+      </c>
+      <c r="B85" t="s" s="2">
         <v>648</v>
-      </c>
-      <c r="B85" t="s" s="2">
-        <v>649</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -13759,10 +13752,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
+        <v>649</v>
+      </c>
+      <c r="B86" t="s" s="2">
         <v>650</v>
-      </c>
-      <c r="B86" t="s" s="2">
-        <v>651</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -13888,10 +13881,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
+        <v>651</v>
+      </c>
+      <c r="B87" t="s" s="2">
         <v>652</v>
-      </c>
-      <c r="B87" t="s" s="2">
-        <v>653</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -13917,16 +13910,16 @@
         <v>175</v>
       </c>
       <c r="L87" t="s" s="2">
+        <v>653</v>
+      </c>
+      <c r="M87" t="s" s="2">
         <v>654</v>
       </c>
-      <c r="M87" t="s" s="2">
+      <c r="N87" t="s" s="2">
         <v>655</v>
       </c>
-      <c r="N87" t="s" s="2">
+      <c r="O87" t="s" s="2">
         <v>656</v>
-      </c>
-      <c r="O87" t="s" s="2">
-        <v>657</v>
       </c>
       <c r="P87" t="s" s="2">
         <v>82</v>
@@ -13954,28 +13947,28 @@
         <v>242</v>
       </c>
       <c r="Y87" t="s" s="2">
+        <v>657</v>
+      </c>
+      <c r="Z87" t="s" s="2">
         <v>658</v>
       </c>
-      <c r="Z87" t="s" s="2">
+      <c r="AA87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF87" t="s" s="2">
         <v>659</v>
-      </c>
-      <c r="AA87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF87" t="s" s="2">
-        <v>660</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>83</v>
@@ -14002,7 +13995,7 @@
         <v>82</v>
       </c>
       <c r="AO87" t="s" s="2">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="AP87" t="s" s="2">
         <v>82</v>
@@ -14019,10 +14012,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
+        <v>661</v>
+      </c>
+      <c r="B88" t="s" s="2">
         <v>662</v>
-      </c>
-      <c r="B88" t="s" s="2">
-        <v>663</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -14048,16 +14041,16 @@
         <v>259</v>
       </c>
       <c r="L88" t="s" s="2">
+        <v>663</v>
+      </c>
+      <c r="M88" t="s" s="2">
         <v>664</v>
       </c>
-      <c r="M88" t="s" s="2">
+      <c r="N88" t="s" s="2">
         <v>665</v>
       </c>
-      <c r="N88" t="s" s="2">
+      <c r="O88" t="s" s="2">
         <v>666</v>
-      </c>
-      <c r="O88" t="s" s="2">
-        <v>667</v>
       </c>
       <c r="P88" t="s" s="2">
         <v>82</v>
@@ -14085,28 +14078,28 @@
         <v>157</v>
       </c>
       <c r="Y88" t="s" s="2">
+        <v>667</v>
+      </c>
+      <c r="Z88" t="s" s="2">
         <v>668</v>
       </c>
-      <c r="Z88" t="s" s="2">
+      <c r="AA88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF88" t="s" s="2">
         <v>669</v>
-      </c>
-      <c r="AA88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF88" t="s" s="2">
-        <v>670</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>83</v>
@@ -14133,7 +14126,7 @@
         <v>82</v>
       </c>
       <c r="AO88" t="s" s="2">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="AP88" t="s" s="2">
         <v>82</v>
@@ -14142,7 +14135,7 @@
         <v>82</v>
       </c>
       <c r="AR88" t="s" s="2">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="AS88" t="s" s="2">
         <v>82</v>
@@ -14150,10 +14143,10 @@
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
+        <v>671</v>
+      </c>
+      <c r="B89" t="s" s="2">
         <v>672</v>
-      </c>
-      <c r="B89" t="s" s="2">
-        <v>673</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -14277,10 +14270,10 @@
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
+        <v>673</v>
+      </c>
+      <c r="B90" t="s" s="2">
         <v>674</v>
-      </c>
-      <c r="B90" t="s" s="2">
-        <v>675</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -14406,10 +14399,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
+        <v>675</v>
+      </c>
+      <c r="B91" t="s" s="2">
         <v>676</v>
-      </c>
-      <c r="B91" t="s" s="2">
-        <v>677</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -14435,16 +14428,16 @@
         <v>153</v>
       </c>
       <c r="L91" t="s" s="2">
+        <v>677</v>
+      </c>
+      <c r="M91" t="s" s="2">
         <v>678</v>
       </c>
-      <c r="M91" t="s" s="2">
+      <c r="N91" t="s" s="2">
         <v>679</v>
       </c>
-      <c r="N91" t="s" s="2">
+      <c r="O91" t="s" s="2">
         <v>680</v>
-      </c>
-      <c r="O91" t="s" s="2">
-        <v>681</v>
       </c>
       <c r="P91" t="s" s="2">
         <v>82</v>
@@ -14493,7 +14486,7 @@
         <v>82</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>83</v>
@@ -14520,16 +14513,16 @@
         <v>82</v>
       </c>
       <c r="AO91" t="s" s="2">
+        <v>682</v>
+      </c>
+      <c r="AP91" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ91" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR91" t="s" s="2">
         <v>683</v>
-      </c>
-      <c r="AP91" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ91" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR91" t="s" s="2">
-        <v>684</v>
       </c>
       <c r="AS91" t="s" s="2">
         <v>82</v>
@@ -14537,10 +14530,10 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
+        <v>684</v>
+      </c>
+      <c r="B92" t="s" s="2">
         <v>685</v>
-      </c>
-      <c r="B92" t="s" s="2">
-        <v>686</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -14664,10 +14657,10 @@
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
+        <v>686</v>
+      </c>
+      <c r="B93" t="s" s="2">
         <v>687</v>
-      </c>
-      <c r="B93" t="s" s="2">
-        <v>688</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -14793,10 +14786,10 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
+        <v>688</v>
+      </c>
+      <c r="B94" t="s" s="2">
         <v>689</v>
-      </c>
-      <c r="B94" t="s" s="2">
-        <v>690</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -14822,16 +14815,16 @@
         <v>140</v>
       </c>
       <c r="L94" t="s" s="2">
+        <v>690</v>
+      </c>
+      <c r="M94" t="s" s="2">
         <v>691</v>
       </c>
-      <c r="M94" t="s" s="2">
+      <c r="N94" t="s" s="2">
         <v>692</v>
       </c>
-      <c r="N94" t="s" s="2">
+      <c r="O94" t="s" s="2">
         <v>693</v>
-      </c>
-      <c r="O94" t="s" s="2">
-        <v>694</v>
       </c>
       <c r="P94" t="s" s="2">
         <v>82</v>
@@ -14841,46 +14834,46 @@
         <v>82</v>
       </c>
       <c r="S94" t="s" s="2">
+        <v>694</v>
+      </c>
+      <c r="T94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF94" t="s" s="2">
         <v>695</v>
-      </c>
-      <c r="T94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF94" t="s" s="2">
-        <v>696</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>83</v>
@@ -14907,16 +14900,16 @@
         <v>82</v>
       </c>
       <c r="AO94" t="s" s="2">
+        <v>696</v>
+      </c>
+      <c r="AP94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR94" t="s" s="2">
         <v>697</v>
-      </c>
-      <c r="AP94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR94" t="s" s="2">
-        <v>698</v>
       </c>
       <c r="AS94" t="s" s="2">
         <v>82</v>
@@ -14924,10 +14917,10 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
+        <v>698</v>
+      </c>
+      <c r="B95" t="s" s="2">
         <v>699</v>
-      </c>
-      <c r="B95" t="s" s="2">
-        <v>700</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -14953,13 +14946,13 @@
         <v>111</v>
       </c>
       <c r="L95" t="s" s="2">
+        <v>700</v>
+      </c>
+      <c r="M95" t="s" s="2">
         <v>701</v>
       </c>
-      <c r="M95" t="s" s="2">
+      <c r="N95" t="s" s="2">
         <v>702</v>
-      </c>
-      <c r="N95" t="s" s="2">
-        <v>703</v>
       </c>
       <c r="O95" s="2"/>
       <c r="P95" t="s" s="2">
@@ -15009,7 +15002,7 @@
         <v>82</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>83</v>
@@ -15036,16 +15029,16 @@
         <v>82</v>
       </c>
       <c r="AO95" t="s" s="2">
+        <v>704</v>
+      </c>
+      <c r="AP95" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ95" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR95" t="s" s="2">
         <v>705</v>
-      </c>
-      <c r="AP95" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ95" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR95" t="s" s="2">
-        <v>706</v>
       </c>
       <c r="AS95" t="s" s="2">
         <v>82</v>
@@ -15053,10 +15046,10 @@
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
+        <v>706</v>
+      </c>
+      <c r="B96" t="s" s="2">
         <v>707</v>
-      </c>
-      <c r="B96" t="s" s="2">
-        <v>708</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -15082,14 +15075,14 @@
         <v>175</v>
       </c>
       <c r="L96" t="s" s="2">
+        <v>708</v>
+      </c>
+      <c r="M96" t="s" s="2">
         <v>709</v>
-      </c>
-      <c r="M96" t="s" s="2">
-        <v>710</v>
       </c>
       <c r="N96" s="2"/>
       <c r="O96" t="s" s="2">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="P96" t="s" s="2">
         <v>82</v>
@@ -15138,7 +15131,7 @@
         <v>82</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>83</v>
@@ -15174,7 +15167,7 @@
         <v>82</v>
       </c>
       <c r="AR96" t="s" s="2">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="AS96" t="s" s="2">
         <v>82</v>
@@ -15182,10 +15175,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
+        <v>713</v>
+      </c>
+      <c r="B97" t="s" s="2">
         <v>714</v>
-      </c>
-      <c r="B97" t="s" s="2">
-        <v>715</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -15211,14 +15204,14 @@
         <v>111</v>
       </c>
       <c r="L97" t="s" s="2">
+        <v>715</v>
+      </c>
+      <c r="M97" t="s" s="2">
         <v>716</v>
-      </c>
-      <c r="M97" t="s" s="2">
-        <v>717</v>
       </c>
       <c r="N97" s="2"/>
       <c r="O97" t="s" s="2">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="P97" t="s" s="2">
         <v>82</v>
@@ -15267,7 +15260,7 @@
         <v>82</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>83</v>
@@ -15294,16 +15287,16 @@
         <v>82</v>
       </c>
       <c r="AO97" t="s" s="2">
+        <v>719</v>
+      </c>
+      <c r="AP97" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ97" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR97" t="s" s="2">
         <v>720</v>
-      </c>
-      <c r="AP97" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ97" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR97" t="s" s="2">
-        <v>721</v>
       </c>
       <c r="AS97" t="s" s="2">
         <v>82</v>
@@ -15311,10 +15304,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
+        <v>721</v>
+      </c>
+      <c r="B98" t="s" s="2">
         <v>722</v>
-      </c>
-      <c r="B98" t="s" s="2">
-        <v>723</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -15337,19 +15330,19 @@
         <v>98</v>
       </c>
       <c r="K98" t="s" s="2">
+        <v>723</v>
+      </c>
+      <c r="L98" t="s" s="2">
         <v>724</v>
       </c>
-      <c r="L98" t="s" s="2">
+      <c r="M98" t="s" s="2">
         <v>725</v>
       </c>
-      <c r="M98" t="s" s="2">
+      <c r="N98" t="s" s="2">
         <v>726</v>
       </c>
-      <c r="N98" t="s" s="2">
+      <c r="O98" t="s" s="2">
         <v>727</v>
-      </c>
-      <c r="O98" t="s" s="2">
-        <v>728</v>
       </c>
       <c r="P98" t="s" s="2">
         <v>82</v>
@@ -15398,7 +15391,7 @@
         <v>82</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>83</v>
@@ -15425,16 +15418,16 @@
         <v>82</v>
       </c>
       <c r="AO98" t="s" s="2">
+        <v>729</v>
+      </c>
+      <c r="AP98" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ98" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR98" t="s" s="2">
         <v>730</v>
-      </c>
-      <c r="AP98" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ98" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR98" t="s" s="2">
-        <v>731</v>
       </c>
       <c r="AS98" t="s" s="2">
         <v>82</v>
@@ -15442,10 +15435,10 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
+        <v>731</v>
+      </c>
+      <c r="B99" t="s" s="2">
         <v>732</v>
-      </c>
-      <c r="B99" t="s" s="2">
-        <v>733</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -15471,16 +15464,16 @@
         <v>111</v>
       </c>
       <c r="L99" t="s" s="2">
+        <v>733</v>
+      </c>
+      <c r="M99" t="s" s="2">
         <v>734</v>
       </c>
-      <c r="M99" t="s" s="2">
+      <c r="N99" t="s" s="2">
         <v>735</v>
       </c>
-      <c r="N99" t="s" s="2">
+      <c r="O99" t="s" s="2">
         <v>736</v>
-      </c>
-      <c r="O99" t="s" s="2">
-        <v>737</v>
       </c>
       <c r="P99" t="s" s="2">
         <v>82</v>
@@ -15529,7 +15522,7 @@
         <v>82</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>83</v>
@@ -15556,16 +15549,16 @@
         <v>82</v>
       </c>
       <c r="AO99" t="s" s="2">
+        <v>738</v>
+      </c>
+      <c r="AP99" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ99" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR99" t="s" s="2">
         <v>739</v>
-      </c>
-      <c r="AP99" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ99" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR99" t="s" s="2">
-        <v>740</v>
       </c>
       <c r="AS99" t="s" s="2">
         <v>82</v>
@@ -15573,10 +15566,10 @@
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
+        <v>740</v>
+      </c>
+      <c r="B100" t="s" s="2">
         <v>741</v>
-      </c>
-      <c r="B100" t="s" s="2">
-        <v>742</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -15602,16 +15595,16 @@
         <v>140</v>
       </c>
       <c r="L100" t="s" s="2">
+        <v>742</v>
+      </c>
+      <c r="M100" t="s" s="2">
         <v>743</v>
       </c>
-      <c r="M100" t="s" s="2">
+      <c r="N100" t="s" s="2">
         <v>744</v>
       </c>
-      <c r="N100" t="s" s="2">
+      <c r="O100" t="s" s="2">
         <v>745</v>
-      </c>
-      <c r="O100" t="s" s="2">
-        <v>746</v>
       </c>
       <c r="P100" t="s" s="2">
         <v>82</v>
@@ -15624,43 +15617,43 @@
         <v>82</v>
       </c>
       <c r="T100" t="s" s="2">
+        <v>746</v>
+      </c>
+      <c r="U100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF100" t="s" s="2">
         <v>747</v>
-      </c>
-      <c r="U100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF100" t="s" s="2">
-        <v>748</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>83</v>
@@ -15687,16 +15680,16 @@
         <v>82</v>
       </c>
       <c r="AO100" t="s" s="2">
+        <v>748</v>
+      </c>
+      <c r="AP100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR100" t="s" s="2">
         <v>749</v>
-      </c>
-      <c r="AP100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR100" t="s" s="2">
-        <v>750</v>
       </c>
       <c r="AS100" t="s" s="2">
         <v>82</v>
@@ -15704,10 +15697,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
+        <v>750</v>
+      </c>
+      <c r="B101" t="s" s="2">
         <v>751</v>
-      </c>
-      <c r="B101" t="s" s="2">
-        <v>752</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -15733,13 +15726,13 @@
         <v>111</v>
       </c>
       <c r="L101" t="s" s="2">
+        <v>752</v>
+      </c>
+      <c r="M101" t="s" s="2">
         <v>753</v>
       </c>
-      <c r="M101" t="s" s="2">
+      <c r="N101" t="s" s="2">
         <v>754</v>
-      </c>
-      <c r="N101" t="s" s="2">
-        <v>755</v>
       </c>
       <c r="O101" s="2"/>
       <c r="P101" t="s" s="2">
@@ -15753,43 +15746,43 @@
         <v>82</v>
       </c>
       <c r="T101" t="s" s="2">
+        <v>755</v>
+      </c>
+      <c r="U101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF101" t="s" s="2">
         <v>756</v>
-      </c>
-      <c r="U101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF101" t="s" s="2">
-        <v>757</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>83</v>
@@ -15816,16 +15809,16 @@
         <v>82</v>
       </c>
       <c r="AO101" t="s" s="2">
+        <v>757</v>
+      </c>
+      <c r="AP101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR101" t="s" s="2">
         <v>758</v>
-      </c>
-      <c r="AP101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR101" t="s" s="2">
-        <v>759</v>
       </c>
       <c r="AS101" t="s" s="2">
         <v>82</v>
@@ -15833,10 +15826,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
+        <v>759</v>
+      </c>
+      <c r="B102" t="s" s="2">
         <v>760</v>
-      </c>
-      <c r="B102" t="s" s="2">
-        <v>761</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -15859,13 +15852,13 @@
         <v>98</v>
       </c>
       <c r="K102" t="s" s="2">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="L102" t="s" s="2">
+        <v>761</v>
+      </c>
+      <c r="M102" t="s" s="2">
         <v>762</v>
-      </c>
-      <c r="M102" t="s" s="2">
-        <v>763</v>
       </c>
       <c r="N102" s="2"/>
       <c r="O102" s="2"/>
@@ -15916,7 +15909,7 @@
         <v>82</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>83</v>
@@ -15943,16 +15936,16 @@
         <v>82</v>
       </c>
       <c r="AO102" t="s" s="2">
+        <v>764</v>
+      </c>
+      <c r="AP102" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ102" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR102" t="s" s="2">
         <v>765</v>
-      </c>
-      <c r="AP102" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ102" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR102" t="s" s="2">
-        <v>766</v>
       </c>
       <c r="AS102" t="s" s="2">
         <v>82</v>
@@ -15960,10 +15953,10 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
+        <v>766</v>
+      </c>
+      <c r="B103" t="s" s="2">
         <v>767</v>
-      </c>
-      <c r="B103" t="s" s="2">
-        <v>768</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -15989,13 +15982,13 @@
         <v>333</v>
       </c>
       <c r="L103" t="s" s="2">
+        <v>768</v>
+      </c>
+      <c r="M103" t="s" s="2">
         <v>769</v>
       </c>
-      <c r="M103" t="s" s="2">
+      <c r="N103" t="s" s="2">
         <v>770</v>
-      </c>
-      <c r="N103" t="s" s="2">
-        <v>771</v>
       </c>
       <c r="O103" s="2"/>
       <c r="P103" t="s" s="2">
@@ -16045,7 +16038,7 @@
         <v>82</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>83</v>
@@ -16072,16 +16065,16 @@
         <v>82</v>
       </c>
       <c r="AO103" t="s" s="2">
+        <v>772</v>
+      </c>
+      <c r="AP103" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ103" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR103" t="s" s="2">
         <v>773</v>
-      </c>
-      <c r="AP103" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ103" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR103" t="s" s="2">
-        <v>774</v>
       </c>
       <c r="AS103" t="s" s="2">
         <v>82</v>
@@ -16089,10 +16082,10 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
+        <v>774</v>
+      </c>
+      <c r="B104" t="s" s="2">
         <v>775</v>
-      </c>
-      <c r="B104" t="s" s="2">
-        <v>776</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -16118,13 +16111,13 @@
         <v>111</v>
       </c>
       <c r="L104" t="s" s="2">
+        <v>618</v>
+      </c>
+      <c r="M104" t="s" s="2">
         <v>619</v>
       </c>
-      <c r="M104" t="s" s="2">
+      <c r="N104" t="s" s="2">
         <v>620</v>
-      </c>
-      <c r="N104" t="s" s="2">
-        <v>621</v>
       </c>
       <c r="O104" s="2"/>
       <c r="P104" t="s" s="2">
@@ -16174,7 +16167,7 @@
         <v>82</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>83</v>

</xml_diff>

<commit_message>
Retirer le pattern redondant sur visibilityStatus
Même raisonnement que pour confidentiality : JDV_J110-StatutVisibiliteDocument-CISIS
est un ValueSet fermé/énuméré (5 codes), son required binding suffit
seul à discriminer la slice. Les deux slices reposent maintenant
uniquement sur leur required binding respectif. c50a069327db053650c699a7b6c9a243ef4011d1
</commit_message>
<xml_diff>
--- a/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4295" uniqueCount="776">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4295" uniqueCount="775">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-06T13:37:30+00:00</t>
+    <t>2026-08-06T13:40:23+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1251,7 +1251,7 @@
 </t>
   </si>
   <si>
-    <t>Slice sur securityLabel pour distinguer le niveau de confidentialité (NRV) du statut de visibilité complémentaire (TRE A07) : confidentiality est discriminée par son required binding (ValueSet fermé v3-ConfidentialityClassification), visibilityStatus par un pattern sur coding.system (JDV_J110-StatutVisibiliteDocument-CISIS)</t>
+    <t>Slice sur securityLabel pour distinguer le niveau de confidentialité (NRV) du statut de visibilité complémentaire (TRE A07) : chaque slice est discriminée par son required binding sur un ValueSet fermé (v3-ConfidentialityClassification pour confidentiality, JDV_J110-StatutVisibiliteDocument-CISIS pour visibilityStatus)</t>
   </si>
   <si>
     <t>niveauConfidentialite : [0..*] code</t>
@@ -1291,13 +1291,6 @@
   </si>
   <si>
     <t>Statut de visibilité complémentaire du document (motifs de masquage patient, représentants légaux, professionnels).</t>
-  </si>
-  <si>
-    <t>&lt;valueCodeableConcept xmlns="http://hl7.org/fhir"&gt;
-  &lt;coding&gt;
-    &lt;system value="https://mos.esante.gouv.fr/NOS/TRE_A07-StatutVisibiliteDocument/FHIR/TRE-A07-StatutVisibiliteDocument"/&gt;
-  &lt;/coding&gt;
-&lt;/valueCodeableConcept&gt;</t>
   </si>
   <si>
     <t>https://mos.esante.gouv.fr/NOS/JDV_J110-StatutVisibiliteDocument-CISIS/FHIR/JDV-J110-StatutVisibiliteDocument-CISIS</t>
@@ -2787,7 +2780,7 @@
     <col min="26" max="26" width="102.93359375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="253.52734375" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="249.46875" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="32" max="32" width="37.78125" customWidth="true" bestFit="true" hidden="true"/>
@@ -8009,7 +8002,7 @@
         <v>82</v>
       </c>
       <c r="S41" t="s" s="2">
-        <v>407</v>
+        <v>82</v>
       </c>
       <c r="T41" t="s" s="2">
         <v>82</v>
@@ -8028,7 +8021,7 @@
       </c>
       <c r="Y41" s="2"/>
       <c r="Z41" t="s" s="2">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="AA41" t="s" s="2">
         <v>82</v>
@@ -8090,10 +8083,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -8119,10 +8112,10 @@
         <v>341</v>
       </c>
       <c r="L42" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="M42" t="s" s="2">
         <v>410</v>
-      </c>
-      <c r="M42" t="s" s="2">
-        <v>411</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -8173,7 +8166,7 @@
         <v>82</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>97</v>
@@ -8197,10 +8190,10 @@
         <v>82</v>
       </c>
       <c r="AN42" t="s" s="2">
+        <v>411</v>
+      </c>
+      <c r="AO42" t="s" s="2">
         <v>412</v>
-      </c>
-      <c r="AO42" t="s" s="2">
-        <v>413</v>
       </c>
       <c r="AP42" t="s" s="2">
         <v>82</v>
@@ -8217,10 +8210,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -8344,10 +8337,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -8473,10 +8466,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -8604,10 +8597,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -8630,13 +8623,13 @@
         <v>98</v>
       </c>
       <c r="K46" t="s" s="2">
+        <v>417</v>
+      </c>
+      <c r="L46" t="s" s="2">
         <v>418</v>
       </c>
-      <c r="L46" t="s" s="2">
+      <c r="M46" t="s" s="2">
         <v>419</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>420</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -8687,7 +8680,7 @@
         <v>82</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>97</v>
@@ -8711,30 +8704,30 @@
         <v>82</v>
       </c>
       <c r="AN46" t="s" s="2">
+        <v>420</v>
+      </c>
+      <c r="AO46" t="s" s="2">
+        <v>412</v>
+      </c>
+      <c r="AP46" t="s" s="2">
         <v>421</v>
       </c>
-      <c r="AO46" t="s" s="2">
-        <v>413</v>
-      </c>
-      <c r="AP46" t="s" s="2">
+      <c r="AQ46" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR46" t="s" s="2">
         <v>422</v>
       </c>
-      <c r="AQ46" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR46" t="s" s="2">
+      <c r="AS46" t="s" s="2">
         <v>423</v>
-      </c>
-      <c r="AS46" t="s" s="2">
-        <v>424</v>
       </c>
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -8858,10 +8851,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -8987,10 +8980,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -9016,14 +9009,14 @@
         <v>175</v>
       </c>
       <c r="L49" t="s" s="2">
+        <v>427</v>
+      </c>
+      <c r="M49" t="s" s="2">
         <v>428</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>429</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" t="s" s="2">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="P49" t="s" s="2">
         <v>82</v>
@@ -9036,7 +9029,7 @@
         <v>82</v>
       </c>
       <c r="T49" t="s" s="2">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="U49" t="s" s="2">
         <v>82</v>
@@ -9051,28 +9044,28 @@
         <v>242</v>
       </c>
       <c r="Y49" t="s" s="2">
+        <v>431</v>
+      </c>
+      <c r="Z49" t="s" s="2">
         <v>432</v>
       </c>
-      <c r="Z49" t="s" s="2">
+      <c r="AA49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF49" t="s" s="2">
         <v>433</v>
-      </c>
-      <c r="AA49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF49" t="s" s="2">
-        <v>434</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>83</v>
@@ -9090,25 +9083,25 @@
         <v>82</v>
       </c>
       <c r="AL49" t="s" s="2">
+        <v>434</v>
+      </c>
+      <c r="AM49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO49" t="s" s="2">
         <v>435</v>
       </c>
-      <c r="AM49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO49" t="s" s="2">
+      <c r="AP49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR49" t="s" s="2">
         <v>436</v>
-      </c>
-      <c r="AP49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR49" t="s" s="2">
-        <v>437</v>
       </c>
       <c r="AS49" t="s" s="2">
         <v>82</v>
@@ -9116,10 +9109,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -9145,14 +9138,14 @@
         <v>175</v>
       </c>
       <c r="L50" t="s" s="2">
+        <v>438</v>
+      </c>
+      <c r="M50" t="s" s="2">
         <v>439</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>440</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" t="s" s="2">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="P50" t="s" s="2">
         <v>82</v>
@@ -9165,7 +9158,7 @@
         <v>82</v>
       </c>
       <c r="T50" t="s" s="2">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="U50" t="s" s="2">
         <v>82</v>
@@ -9201,7 +9194,7 @@
         <v>82</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>83</v>
@@ -9216,19 +9209,19 @@
         <v>109</v>
       </c>
       <c r="AK50" t="s" s="2">
+        <v>443</v>
+      </c>
+      <c r="AL50" t="s" s="2">
         <v>444</v>
       </c>
-      <c r="AL50" t="s" s="2">
+      <c r="AM50" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN50" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO50" t="s" s="2">
         <v>445</v>
-      </c>
-      <c r="AM50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO50" t="s" s="2">
-        <v>446</v>
       </c>
       <c r="AP50" t="s" s="2">
         <v>82</v>
@@ -9245,10 +9238,10 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -9271,19 +9264,19 @@
         <v>82</v>
       </c>
       <c r="K51" t="s" s="2">
+        <v>447</v>
+      </c>
+      <c r="L51" t="s" s="2">
         <v>448</v>
       </c>
-      <c r="L51" t="s" s="2">
+      <c r="M51" t="s" s="2">
         <v>449</v>
       </c>
-      <c r="M51" t="s" s="2">
+      <c r="N51" t="s" s="2">
         <v>450</v>
       </c>
-      <c r="N51" t="s" s="2">
+      <c r="O51" t="s" s="2">
         <v>451</v>
-      </c>
-      <c r="O51" t="s" s="2">
-        <v>452</v>
       </c>
       <c r="P51" t="s" s="2">
         <v>82</v>
@@ -9332,7 +9325,7 @@
         <v>82</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>83</v>
@@ -9359,16 +9352,16 @@
         <v>82</v>
       </c>
       <c r="AO51" t="s" s="2">
+        <v>453</v>
+      </c>
+      <c r="AP51" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ51" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR51" t="s" s="2">
         <v>454</v>
-      </c>
-      <c r="AP51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR51" t="s" s="2">
-        <v>455</v>
       </c>
       <c r="AS51" t="s" s="2">
         <v>82</v>
@@ -9376,10 +9369,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -9402,19 +9395,19 @@
         <v>98</v>
       </c>
       <c r="K52" t="s" s="2">
+        <v>456</v>
+      </c>
+      <c r="L52" t="s" s="2">
         <v>457</v>
       </c>
-      <c r="L52" t="s" s="2">
+      <c r="M52" t="s" s="2">
         <v>458</v>
       </c>
-      <c r="M52" t="s" s="2">
+      <c r="N52" t="s" s="2">
         <v>459</v>
       </c>
-      <c r="N52" t="s" s="2">
+      <c r="O52" t="s" s="2">
         <v>460</v>
-      </c>
-      <c r="O52" t="s" s="2">
-        <v>461</v>
       </c>
       <c r="P52" t="s" s="2">
         <v>82</v>
@@ -9427,79 +9420,79 @@
         <v>82</v>
       </c>
       <c r="T52" t="s" s="2">
+        <v>461</v>
+      </c>
+      <c r="U52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF52" t="s" s="2">
         <v>462</v>
       </c>
-      <c r="U52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF52" t="s" s="2">
+      <c r="AG52" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH52" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ52" t="s" s="2">
         <v>463</v>
       </c>
-      <c r="AG52" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH52" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ52" t="s" s="2">
+      <c r="AK52" t="s" s="2">
         <v>464</v>
       </c>
-      <c r="AK52" t="s" s="2">
+      <c r="AL52" t="s" s="2">
         <v>465</v>
       </c>
-      <c r="AL52" t="s" s="2">
+      <c r="AM52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO52" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="AM52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO52" t="s" s="2">
+      <c r="AP52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR52" t="s" s="2">
         <v>467</v>
-      </c>
-      <c r="AP52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR52" t="s" s="2">
-        <v>468</v>
       </c>
       <c r="AS52" t="s" s="2">
         <v>82</v>
@@ -9507,10 +9500,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -9533,19 +9526,19 @@
         <v>98</v>
       </c>
       <c r="K53" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="L53" t="s" s="2">
         <v>470</v>
       </c>
-      <c r="L53" t="s" s="2">
+      <c r="M53" t="s" s="2">
         <v>471</v>
       </c>
-      <c r="M53" t="s" s="2">
+      <c r="N53" t="s" s="2">
         <v>472</v>
       </c>
-      <c r="N53" t="s" s="2">
+      <c r="O53" t="s" s="2">
         <v>473</v>
-      </c>
-      <c r="O53" t="s" s="2">
-        <v>474</v>
       </c>
       <c r="P53" t="s" s="2">
         <v>82</v>
@@ -9594,7 +9587,7 @@
         <v>82</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>83</v>
@@ -9612,16 +9605,16 @@
         <v>82</v>
       </c>
       <c r="AL53" t="s" s="2">
+        <v>475</v>
+      </c>
+      <c r="AM53" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN53" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO53" t="s" s="2">
         <v>476</v>
-      </c>
-      <c r="AM53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO53" t="s" s="2">
-        <v>477</v>
       </c>
       <c r="AP53" t="s" s="2">
         <v>82</v>
@@ -9638,10 +9631,10 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -9664,19 +9657,19 @@
         <v>98</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="L54" t="s" s="2">
+        <v>478</v>
+      </c>
+      <c r="M54" t="s" s="2">
         <v>479</v>
       </c>
-      <c r="M54" t="s" s="2">
+      <c r="N54" t="s" s="2">
         <v>480</v>
       </c>
-      <c r="N54" t="s" s="2">
+      <c r="O54" t="s" s="2">
         <v>481</v>
-      </c>
-      <c r="O54" t="s" s="2">
-        <v>482</v>
       </c>
       <c r="P54" t="s" s="2">
         <v>82</v>
@@ -9725,7 +9718,7 @@
         <v>82</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>83</v>
@@ -9743,16 +9736,16 @@
         <v>82</v>
       </c>
       <c r="AL54" t="s" s="2">
+        <v>483</v>
+      </c>
+      <c r="AM54" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN54" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO54" t="s" s="2">
         <v>484</v>
-      </c>
-      <c r="AM54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO54" t="s" s="2">
-        <v>485</v>
       </c>
       <c r="AP54" t="s" s="2">
         <v>82</v>
@@ -9769,10 +9762,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -9798,14 +9791,14 @@
         <v>111</v>
       </c>
       <c r="L55" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="M55" t="s" s="2">
         <v>487</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>488</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" t="s" s="2">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="P55" t="s" s="2">
         <v>82</v>
@@ -9818,43 +9811,43 @@
         <v>82</v>
       </c>
       <c r="T55" t="s" s="2">
+        <v>489</v>
+      </c>
+      <c r="U55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF55" t="s" s="2">
         <v>490</v>
-      </c>
-      <c r="U55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF55" t="s" s="2">
-        <v>491</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>83</v>
@@ -9869,19 +9862,19 @@
         <v>109</v>
       </c>
       <c r="AK55" t="s" s="2">
+        <v>491</v>
+      </c>
+      <c r="AL55" t="s" s="2">
         <v>492</v>
       </c>
-      <c r="AL55" t="s" s="2">
+      <c r="AM55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO55" t="s" s="2">
         <v>493</v>
-      </c>
-      <c r="AM55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO55" t="s" s="2">
-        <v>494</v>
       </c>
       <c r="AP55" t="s" s="2">
         <v>82</v>
@@ -9898,10 +9891,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -9924,17 +9917,17 @@
         <v>98</v>
       </c>
       <c r="K56" t="s" s="2">
+        <v>495</v>
+      </c>
+      <c r="L56" t="s" s="2">
         <v>496</v>
       </c>
-      <c r="L56" t="s" s="2">
+      <c r="M56" t="s" s="2">
         <v>497</v>
-      </c>
-      <c r="M56" t="s" s="2">
-        <v>498</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" t="s" s="2">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="P56" t="s" s="2">
         <v>82</v>
@@ -9983,7 +9976,7 @@
         <v>82</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>83</v>
@@ -9998,11 +9991,11 @@
         <v>109</v>
       </c>
       <c r="AK56" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="AL56" t="s" s="2">
         <v>501</v>
       </c>
-      <c r="AL56" t="s" s="2">
-        <v>502</v>
-      </c>
       <c r="AM56" t="s" s="2">
         <v>82</v>
       </c>
@@ -10010,7 +10003,7 @@
         <v>82</v>
       </c>
       <c r="AO56" t="s" s="2">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="AP56" t="s" s="2">
         <v>82</v>
@@ -10027,10 +10020,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -10056,13 +10049,13 @@
         <v>153</v>
       </c>
       <c r="L57" t="s" s="2">
+        <v>503</v>
+      </c>
+      <c r="M57" t="s" s="2">
         <v>504</v>
       </c>
-      <c r="M57" t="s" s="2">
+      <c r="N57" t="s" s="2">
         <v>505</v>
-      </c>
-      <c r="N57" t="s" s="2">
-        <v>506</v>
       </c>
       <c r="O57" s="2"/>
       <c r="P57" t="s" s="2">
@@ -10092,56 +10085,56 @@
       </c>
       <c r="Y57" s="2"/>
       <c r="Z57" t="s" s="2">
+        <v>506</v>
+      </c>
+      <c r="AA57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF57" t="s" s="2">
+        <v>502</v>
+      </c>
+      <c r="AG57" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH57" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ57" t="s" s="2">
         <v>507</v>
       </c>
-      <c r="AA57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF57" t="s" s="2">
-        <v>503</v>
-      </c>
-      <c r="AG57" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH57" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ57" t="s" s="2">
+      <c r="AK57" t="s" s="2">
         <v>508</v>
       </c>
-      <c r="AK57" t="s" s="2">
+      <c r="AL57" t="s" s="2">
         <v>509</v>
       </c>
-      <c r="AL57" t="s" s="2">
+      <c r="AM57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN57" t="s" s="2">
         <v>510</v>
       </c>
-      <c r="AM57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN57" t="s" s="2">
+      <c r="AO57" t="s" s="2">
+        <v>412</v>
+      </c>
+      <c r="AP57" t="s" s="2">
         <v>511</v>
       </c>
-      <c r="AO57" t="s" s="2">
-        <v>413</v>
-      </c>
-      <c r="AP57" t="s" s="2">
-        <v>512</v>
-      </c>
       <c r="AQ57" t="s" s="2">
         <v>82</v>
       </c>
@@ -10149,15 +10142,15 @@
         <v>82</v>
       </c>
       <c r="AS57" t="s" s="2">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -10183,13 +10176,13 @@
         <v>341</v>
       </c>
       <c r="L58" t="s" s="2">
+        <v>513</v>
+      </c>
+      <c r="M58" t="s" s="2">
         <v>514</v>
       </c>
-      <c r="M58" t="s" s="2">
+      <c r="N58" t="s" s="2">
         <v>515</v>
-      </c>
-      <c r="N58" t="s" s="2">
-        <v>516</v>
       </c>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
@@ -10239,7 +10232,7 @@
         <v>82</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>83</v>
@@ -10266,7 +10259,7 @@
         <v>82</v>
       </c>
       <c r="AO58" t="s" s="2">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="AP58" t="s" s="2">
         <v>82</v>
@@ -10283,10 +10276,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -10410,10 +10403,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -10539,10 +10532,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -10670,10 +10663,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -10696,13 +10689,13 @@
         <v>82</v>
       </c>
       <c r="K62" t="s" s="2">
+        <v>521</v>
+      </c>
+      <c r="L62" t="s" s="2">
         <v>522</v>
       </c>
-      <c r="L62" t="s" s="2">
+      <c r="M62" t="s" s="2">
         <v>523</v>
-      </c>
-      <c r="M62" t="s" s="2">
-        <v>524</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -10753,7 +10746,7 @@
         <v>82</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>83</v>
@@ -10771,22 +10764,22 @@
         <v>82</v>
       </c>
       <c r="AL62" t="s" s="2">
+        <v>524</v>
+      </c>
+      <c r="AM62" t="s" s="2">
         <v>525</v>
       </c>
-      <c r="AM62" t="s" s="2">
+      <c r="AN62" t="s" s="2">
         <v>526</v>
       </c>
-      <c r="AN62" t="s" s="2">
+      <c r="AO62" t="s" s="2">
         <v>527</v>
       </c>
-      <c r="AO62" t="s" s="2">
+      <c r="AP62" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ62" t="s" s="2">
         <v>528</v>
-      </c>
-      <c r="AP62" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ62" t="s" s="2">
-        <v>529</v>
       </c>
       <c r="AR62" t="s" s="2">
         <v>82</v>
@@ -10797,10 +10790,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -10826,13 +10819,13 @@
         <v>259</v>
       </c>
       <c r="L63" t="s" s="2">
+        <v>530</v>
+      </c>
+      <c r="M63" t="s" s="2">
         <v>531</v>
       </c>
-      <c r="M63" t="s" s="2">
+      <c r="N63" t="s" s="2">
         <v>532</v>
-      </c>
-      <c r="N63" t="s" s="2">
-        <v>533</v>
       </c>
       <c r="O63" s="2"/>
       <c r="P63" t="s" s="2">
@@ -10861,11 +10854,11 @@
         <v>165</v>
       </c>
       <c r="Y63" t="s" s="2">
+        <v>533</v>
+      </c>
+      <c r="Z63" t="s" s="2">
         <v>534</v>
       </c>
-      <c r="Z63" t="s" s="2">
-        <v>535</v>
-      </c>
       <c r="AA63" t="s" s="2">
         <v>82</v>
       </c>
@@ -10882,7 +10875,7 @@
         <v>82</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>83</v>
@@ -10894,23 +10887,23 @@
         <v>82</v>
       </c>
       <c r="AJ63" t="s" s="2">
+        <v>535</v>
+      </c>
+      <c r="AK63" t="s" s="2">
         <v>536</v>
       </c>
-      <c r="AK63" t="s" s="2">
+      <c r="AL63" t="s" s="2">
         <v>537</v>
       </c>
-      <c r="AL63" t="s" s="2">
+      <c r="AM63" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN63" t="s" s="2">
         <v>538</v>
       </c>
-      <c r="AM63" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN63" t="s" s="2">
+      <c r="AO63" t="s" s="2">
         <v>539</v>
       </c>
-      <c r="AO63" t="s" s="2">
-        <v>540</v>
-      </c>
       <c r="AP63" t="s" s="2">
         <v>82</v>
       </c>
@@ -10921,15 +10914,15 @@
         <v>82</v>
       </c>
       <c r="AS63" t="s" s="2">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -10952,13 +10945,13 @@
         <v>98</v>
       </c>
       <c r="K64" t="s" s="2">
+        <v>541</v>
+      </c>
+      <c r="L64" t="s" s="2">
         <v>542</v>
       </c>
-      <c r="L64" t="s" s="2">
+      <c r="M64" t="s" s="2">
         <v>543</v>
-      </c>
-      <c r="M64" t="s" s="2">
-        <v>544</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
@@ -11009,7 +11002,7 @@
         <v>82</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>83</v>
@@ -11033,30 +11026,30 @@
         <v>82</v>
       </c>
       <c r="AN64" t="s" s="2">
+        <v>544</v>
+      </c>
+      <c r="AO64" t="s" s="2">
         <v>545</v>
       </c>
-      <c r="AO64" t="s" s="2">
+      <c r="AP64" t="s" s="2">
         <v>546</v>
       </c>
-      <c r="AP64" t="s" s="2">
+      <c r="AQ64" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR64" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AS64" t="s" s="2">
         <v>547</v>
-      </c>
-      <c r="AQ64" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR64" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AS64" t="s" s="2">
-        <v>548</v>
       </c>
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -11180,10 +11173,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -11309,10 +11302,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -11335,16 +11328,16 @@
         <v>98</v>
       </c>
       <c r="K67" t="s" s="2">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="L67" t="s" s="2">
+        <v>551</v>
+      </c>
+      <c r="M67" t="s" s="2">
         <v>552</v>
       </c>
-      <c r="M67" t="s" s="2">
+      <c r="N67" t="s" s="2">
         <v>553</v>
-      </c>
-      <c r="N67" t="s" s="2">
-        <v>554</v>
       </c>
       <c r="O67" s="2"/>
       <c r="P67" t="s" s="2">
@@ -11394,43 +11387,43 @@
         <v>82</v>
       </c>
       <c r="AF67" t="s" s="2">
+        <v>554</v>
+      </c>
+      <c r="AG67" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH67" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI67" t="s" s="2">
         <v>555</v>
-      </c>
-      <c r="AG67" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH67" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI67" t="s" s="2">
-        <v>556</v>
       </c>
       <c r="AJ67" t="s" s="2">
         <v>109</v>
       </c>
       <c r="AK67" t="s" s="2">
+        <v>556</v>
+      </c>
+      <c r="AL67" t="s" s="2">
         <v>557</v>
       </c>
-      <c r="AL67" t="s" s="2">
+      <c r="AM67" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN67" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO67" t="s" s="2">
         <v>558</v>
       </c>
-      <c r="AM67" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN67" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO67" t="s" s="2">
+      <c r="AP67" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ67" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR67" t="s" s="2">
         <v>559</v>
-      </c>
-      <c r="AP67" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ67" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR67" t="s" s="2">
-        <v>560</v>
       </c>
       <c r="AS67" t="s" s="2">
         <v>82</v>
@@ -11438,10 +11431,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -11464,69 +11457,69 @@
         <v>98</v>
       </c>
       <c r="K68" t="s" s="2">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="L68" t="s" s="2">
+        <v>561</v>
+      </c>
+      <c r="M68" t="s" s="2">
         <v>562</v>
       </c>
-      <c r="M68" t="s" s="2">
+      <c r="N68" t="s" s="2">
         <v>563</v>
-      </c>
-      <c r="N68" t="s" s="2">
-        <v>564</v>
       </c>
       <c r="O68" s="2"/>
       <c r="P68" t="s" s="2">
         <v>82</v>
       </c>
       <c r="Q68" t="s" s="2">
+        <v>564</v>
+      </c>
+      <c r="R68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF68" t="s" s="2">
         <v>565</v>
       </c>
-      <c r="R68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF68" t="s" s="2">
-        <v>566</v>
-      </c>
       <c r="AG68" t="s" s="2">
         <v>83</v>
       </c>
@@ -11534,34 +11527,34 @@
         <v>97</v>
       </c>
       <c r="AI68" t="s" s="2">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="AJ68" t="s" s="2">
         <v>109</v>
       </c>
       <c r="AK68" t="s" s="2">
+        <v>566</v>
+      </c>
+      <c r="AL68" t="s" s="2">
         <v>567</v>
       </c>
-      <c r="AL68" t="s" s="2">
+      <c r="AM68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO68" t="s" s="2">
         <v>568</v>
       </c>
-      <c r="AM68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO68" t="s" s="2">
+      <c r="AP68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR68" t="s" s="2">
         <v>569</v>
-      </c>
-      <c r="AP68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR68" t="s" s="2">
-        <v>570</v>
       </c>
       <c r="AS68" t="s" s="2">
         <v>82</v>
@@ -11569,10 +11562,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -11598,10 +11591,10 @@
         <v>259</v>
       </c>
       <c r="L69" t="s" s="2">
+        <v>571</v>
+      </c>
+      <c r="M69" t="s" s="2">
         <v>572</v>
-      </c>
-      <c r="M69" t="s" s="2">
-        <v>573</v>
       </c>
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
@@ -11632,56 +11625,56 @@
       </c>
       <c r="Y69" s="2"/>
       <c r="Z69" t="s" s="2">
+        <v>573</v>
+      </c>
+      <c r="AA69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF69" t="s" s="2">
+        <v>570</v>
+      </c>
+      <c r="AG69" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH69" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ69" t="s" s="2">
         <v>574</v>
       </c>
-      <c r="AA69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF69" t="s" s="2">
-        <v>571</v>
-      </c>
-      <c r="AG69" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH69" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ69" t="s" s="2">
+      <c r="AK69" t="s" s="2">
         <v>575</v>
       </c>
-      <c r="AK69" t="s" s="2">
+      <c r="AL69" t="s" s="2">
         <v>576</v>
       </c>
-      <c r="AL69" t="s" s="2">
+      <c r="AM69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN69" t="s" s="2">
         <v>577</v>
       </c>
-      <c r="AM69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN69" t="s" s="2">
+      <c r="AO69" t="s" s="2">
         <v>578</v>
       </c>
-      <c r="AO69" t="s" s="2">
+      <c r="AP69" t="s" s="2">
         <v>579</v>
       </c>
-      <c r="AP69" t="s" s="2">
-        <v>580</v>
-      </c>
       <c r="AQ69" t="s" s="2">
         <v>82</v>
       </c>
@@ -11689,15 +11682,15 @@
         <v>82</v>
       </c>
       <c r="AS69" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -11723,16 +11716,16 @@
         <v>259</v>
       </c>
       <c r="L70" t="s" s="2">
+        <v>581</v>
+      </c>
+      <c r="M70" t="s" s="2">
         <v>582</v>
       </c>
-      <c r="M70" t="s" s="2">
+      <c r="N70" t="s" s="2">
         <v>583</v>
       </c>
-      <c r="N70" t="s" s="2">
+      <c r="O70" t="s" s="2">
         <v>584</v>
-      </c>
-      <c r="O70" t="s" s="2">
-        <v>585</v>
       </c>
       <c r="P70" t="s" s="2">
         <v>82</v>
@@ -11761,55 +11754,55 @@
       </c>
       <c r="Y70" s="2"/>
       <c r="Z70" t="s" s="2">
+        <v>585</v>
+      </c>
+      <c r="AA70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF70" t="s" s="2">
+        <v>580</v>
+      </c>
+      <c r="AG70" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH70" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ70" t="s" s="2">
+        <v>574</v>
+      </c>
+      <c r="AK70" t="s" s="2">
         <v>586</v>
       </c>
-      <c r="AA70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF70" t="s" s="2">
-        <v>581</v>
-      </c>
-      <c r="AG70" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH70" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ70" t="s" s="2">
-        <v>575</v>
-      </c>
-      <c r="AK70" t="s" s="2">
+      <c r="AL70" t="s" s="2">
         <v>587</v>
       </c>
-      <c r="AL70" t="s" s="2">
-        <v>588</v>
-      </c>
       <c r="AM70" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN70" t="s" s="2">
+        <v>577</v>
+      </c>
+      <c r="AO70" t="s" s="2">
         <v>578</v>
       </c>
-      <c r="AO70" t="s" s="2">
-        <v>579</v>
-      </c>
       <c r="AP70" t="s" s="2">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AQ70" t="s" s="2">
         <v>82</v>
@@ -11818,15 +11811,15 @@
         <v>82</v>
       </c>
       <c r="AS70" t="s" s="2">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -11849,13 +11842,13 @@
         <v>82</v>
       </c>
       <c r="K71" t="s" s="2">
+        <v>589</v>
+      </c>
+      <c r="L71" t="s" s="2">
         <v>590</v>
       </c>
-      <c r="L71" t="s" s="2">
+      <c r="M71" t="s" s="2">
         <v>591</v>
-      </c>
-      <c r="M71" t="s" s="2">
-        <v>592</v>
       </c>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
@@ -11906,7 +11899,7 @@
         <v>82</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>83</v>
@@ -11945,15 +11938,15 @@
         <v>82</v>
       </c>
       <c r="AS71" t="s" s="2">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -12077,10 +12070,10 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -12206,10 +12199,10 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -12235,13 +12228,13 @@
         <v>111</v>
       </c>
       <c r="L74" t="s" s="2">
+        <v>596</v>
+      </c>
+      <c r="M74" t="s" s="2">
         <v>597</v>
       </c>
-      <c r="M74" t="s" s="2">
+      <c r="N74" t="s" s="2">
         <v>598</v>
-      </c>
-      <c r="N74" t="s" s="2">
-        <v>599</v>
       </c>
       <c r="O74" s="2"/>
       <c r="P74" t="s" s="2">
@@ -12291,16 +12284,16 @@
         <v>82</v>
       </c>
       <c r="AF74" t="s" s="2">
+        <v>599</v>
+      </c>
+      <c r="AG74" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH74" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI74" t="s" s="2">
         <v>600</v>
-      </c>
-      <c r="AG74" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH74" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI74" t="s" s="2">
-        <v>601</v>
       </c>
       <c r="AJ74" t="s" s="2">
         <v>109</v>
@@ -12309,7 +12302,7 @@
         <v>82</v>
       </c>
       <c r="AL74" t="s" s="2">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="AM74" t="s" s="2">
         <v>82</v>
@@ -12335,10 +12328,10 @@
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -12364,13 +12357,13 @@
         <v>140</v>
       </c>
       <c r="L75" t="s" s="2">
+        <v>603</v>
+      </c>
+      <c r="M75" t="s" s="2">
         <v>604</v>
       </c>
-      <c r="M75" t="s" s="2">
+      <c r="N75" t="s" s="2">
         <v>605</v>
-      </c>
-      <c r="N75" t="s" s="2">
-        <v>606</v>
       </c>
       <c r="O75" s="2"/>
       <c r="P75" t="s" s="2">
@@ -12399,28 +12392,28 @@
         <v>157</v>
       </c>
       <c r="Y75" t="s" s="2">
+        <v>606</v>
+      </c>
+      <c r="Z75" t="s" s="2">
         <v>607</v>
       </c>
-      <c r="Z75" t="s" s="2">
+      <c r="AA75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF75" t="s" s="2">
         <v>608</v>
-      </c>
-      <c r="AA75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF75" t="s" s="2">
-        <v>609</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>83</v>
@@ -12464,10 +12457,10 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -12493,13 +12486,13 @@
         <v>227</v>
       </c>
       <c r="L76" t="s" s="2">
+        <v>610</v>
+      </c>
+      <c r="M76" t="s" s="2">
         <v>611</v>
       </c>
-      <c r="M76" t="s" s="2">
+      <c r="N76" t="s" s="2">
         <v>612</v>
-      </c>
-      <c r="N76" t="s" s="2">
-        <v>613</v>
       </c>
       <c r="O76" s="2"/>
       <c r="P76" t="s" s="2">
@@ -12549,7 +12542,7 @@
         <v>82</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>83</v>
@@ -12567,16 +12560,16 @@
         <v>82</v>
       </c>
       <c r="AL76" t="s" s="2">
+        <v>614</v>
+      </c>
+      <c r="AM76" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN76" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO76" t="s" s="2">
         <v>615</v>
-      </c>
-      <c r="AM76" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN76" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO76" t="s" s="2">
-        <v>616</v>
       </c>
       <c r="AP76" t="s" s="2">
         <v>82</v>
@@ -12593,10 +12586,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -12622,13 +12615,13 @@
         <v>111</v>
       </c>
       <c r="L77" t="s" s="2">
+        <v>617</v>
+      </c>
+      <c r="M77" t="s" s="2">
         <v>618</v>
       </c>
-      <c r="M77" t="s" s="2">
+      <c r="N77" t="s" s="2">
         <v>619</v>
-      </c>
-      <c r="N77" t="s" s="2">
-        <v>620</v>
       </c>
       <c r="O77" s="2"/>
       <c r="P77" t="s" s="2">
@@ -12678,7 +12671,7 @@
         <v>82</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>83</v>
@@ -12722,10 +12715,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -12748,16 +12741,16 @@
         <v>82</v>
       </c>
       <c r="K78" t="s" s="2">
+        <v>622</v>
+      </c>
+      <c r="L78" t="s" s="2">
         <v>623</v>
       </c>
-      <c r="L78" t="s" s="2">
+      <c r="M78" t="s" s="2">
         <v>624</v>
       </c>
-      <c r="M78" t="s" s="2">
+      <c r="N78" t="s" s="2">
         <v>625</v>
-      </c>
-      <c r="N78" t="s" s="2">
-        <v>626</v>
       </c>
       <c r="O78" s="2"/>
       <c r="P78" t="s" s="2">
@@ -12795,10 +12788,10 @@
         <v>82</v>
       </c>
       <c r="AB78" t="s" s="2">
+        <v>626</v>
+      </c>
+      <c r="AC78" t="s" s="2">
         <v>627</v>
-      </c>
-      <c r="AC78" t="s" s="2">
-        <v>628</v>
       </c>
       <c r="AD78" t="s" s="2">
         <v>82</v>
@@ -12807,7 +12800,7 @@
         <v>124</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>83</v>
@@ -12825,39 +12818,39 @@
         <v>82</v>
       </c>
       <c r="AL78" t="s" s="2">
+        <v>628</v>
+      </c>
+      <c r="AM78" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN78" t="s" s="2">
         <v>629</v>
       </c>
-      <c r="AM78" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN78" t="s" s="2">
+      <c r="AO78" t="s" s="2">
         <v>630</v>
       </c>
-      <c r="AO78" t="s" s="2">
+      <c r="AP78" t="s" s="2">
         <v>631</v>
       </c>
-      <c r="AP78" t="s" s="2">
+      <c r="AQ78" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR78" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AS78" t="s" s="2">
         <v>632</v>
-      </c>
-      <c r="AQ78" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR78" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AS78" t="s" s="2">
-        <v>633</v>
       </c>
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
+        <v>633</v>
+      </c>
+      <c r="B79" t="s" s="2">
+        <v>621</v>
+      </c>
+      <c r="C79" t="s" s="2">
         <v>634</v>
-      </c>
-      <c r="B79" t="s" s="2">
-        <v>622</v>
-      </c>
-      <c r="C79" t="s" s="2">
-        <v>635</v>
       </c>
       <c r="D79" t="s" s="2">
         <v>82</v>
@@ -12879,16 +12872,16 @@
         <v>82</v>
       </c>
       <c r="K79" t="s" s="2">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="M79" t="s" s="2">
+        <v>624</v>
+      </c>
+      <c r="N79" t="s" s="2">
         <v>625</v>
-      </c>
-      <c r="N79" t="s" s="2">
-        <v>626</v>
       </c>
       <c r="O79" s="2"/>
       <c r="P79" t="s" s="2">
@@ -12938,7 +12931,7 @@
         <v>82</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>83</v>
@@ -12956,36 +12949,36 @@
         <v>82</v>
       </c>
       <c r="AL79" t="s" s="2">
+        <v>628</v>
+      </c>
+      <c r="AM79" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN79" t="s" s="2">
         <v>629</v>
       </c>
-      <c r="AM79" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN79" t="s" s="2">
+      <c r="AO79" t="s" s="2">
         <v>630</v>
       </c>
-      <c r="AO79" t="s" s="2">
+      <c r="AP79" t="s" s="2">
         <v>631</v>
       </c>
-      <c r="AP79" t="s" s="2">
+      <c r="AQ79" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR79" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AS79" t="s" s="2">
         <v>632</v>
-      </c>
-      <c r="AQ79" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR79" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AS79" t="s" s="2">
-        <v>633</v>
       </c>
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
+        <v>636</v>
+      </c>
+      <c r="B80" t="s" s="2">
         <v>637</v>
-      </c>
-      <c r="B80" t="s" s="2">
-        <v>638</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -13109,10 +13102,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
+        <v>638</v>
+      </c>
+      <c r="B81" t="s" s="2">
         <v>639</v>
-      </c>
-      <c r="B81" t="s" s="2">
-        <v>640</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -13238,10 +13231,10 @@
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
+        <v>640</v>
+      </c>
+      <c r="B82" t="s" s="2">
         <v>641</v>
-      </c>
-      <c r="B82" t="s" s="2">
-        <v>642</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -13267,13 +13260,13 @@
         <v>111</v>
       </c>
       <c r="L82" t="s" s="2">
+        <v>596</v>
+      </c>
+      <c r="M82" t="s" s="2">
         <v>597</v>
       </c>
-      <c r="M82" t="s" s="2">
+      <c r="N82" t="s" s="2">
         <v>598</v>
-      </c>
-      <c r="N82" t="s" s="2">
-        <v>599</v>
       </c>
       <c r="O82" s="2"/>
       <c r="P82" t="s" s="2">
@@ -13323,16 +13316,16 @@
         <v>82</v>
       </c>
       <c r="AF82" t="s" s="2">
+        <v>599</v>
+      </c>
+      <c r="AG82" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH82" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI82" t="s" s="2">
         <v>600</v>
-      </c>
-      <c r="AG82" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH82" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI82" t="s" s="2">
-        <v>601</v>
       </c>
       <c r="AJ82" t="s" s="2">
         <v>109</v>
@@ -13367,10 +13360,10 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
+        <v>642</v>
+      </c>
+      <c r="B83" t="s" s="2">
         <v>643</v>
-      </c>
-      <c r="B83" t="s" s="2">
-        <v>644</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -13396,13 +13389,13 @@
         <v>140</v>
       </c>
       <c r="L83" t="s" s="2">
+        <v>603</v>
+      </c>
+      <c r="M83" t="s" s="2">
         <v>604</v>
       </c>
-      <c r="M83" t="s" s="2">
+      <c r="N83" t="s" s="2">
         <v>605</v>
-      </c>
-      <c r="N83" t="s" s="2">
-        <v>606</v>
       </c>
       <c r="O83" s="2"/>
       <c r="P83" t="s" s="2">
@@ -13431,28 +13424,28 @@
         <v>157</v>
       </c>
       <c r="Y83" t="s" s="2">
+        <v>606</v>
+      </c>
+      <c r="Z83" t="s" s="2">
         <v>607</v>
       </c>
-      <c r="Z83" t="s" s="2">
+      <c r="AA83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF83" t="s" s="2">
         <v>608</v>
-      </c>
-      <c r="AA83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF83" t="s" s="2">
-        <v>609</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>83</v>
@@ -13496,10 +13489,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
+        <v>644</v>
+      </c>
+      <c r="B84" t="s" s="2">
         <v>645</v>
-      </c>
-      <c r="B84" t="s" s="2">
-        <v>646</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -13525,13 +13518,13 @@
         <v>227</v>
       </c>
       <c r="L84" t="s" s="2">
+        <v>610</v>
+      </c>
+      <c r="M84" t="s" s="2">
         <v>611</v>
       </c>
-      <c r="M84" t="s" s="2">
+      <c r="N84" t="s" s="2">
         <v>612</v>
-      </c>
-      <c r="N84" t="s" s="2">
-        <v>613</v>
       </c>
       <c r="O84" s="2"/>
       <c r="P84" t="s" s="2">
@@ -13581,7 +13574,7 @@
         <v>82</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>83</v>
@@ -13608,7 +13601,7 @@
         <v>82</v>
       </c>
       <c r="AO84" t="s" s="2">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="AP84" t="s" s="2">
         <v>82</v>
@@ -13625,10 +13618,10 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
+        <v>646</v>
+      </c>
+      <c r="B85" t="s" s="2">
         <v>647</v>
-      </c>
-      <c r="B85" t="s" s="2">
-        <v>648</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -13752,10 +13745,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
+        <v>648</v>
+      </c>
+      <c r="B86" t="s" s="2">
         <v>649</v>
-      </c>
-      <c r="B86" t="s" s="2">
-        <v>650</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -13881,10 +13874,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
+        <v>650</v>
+      </c>
+      <c r="B87" t="s" s="2">
         <v>651</v>
-      </c>
-      <c r="B87" t="s" s="2">
-        <v>652</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -13910,16 +13903,16 @@
         <v>175</v>
       </c>
       <c r="L87" t="s" s="2">
+        <v>652</v>
+      </c>
+      <c r="M87" t="s" s="2">
         <v>653</v>
       </c>
-      <c r="M87" t="s" s="2">
+      <c r="N87" t="s" s="2">
         <v>654</v>
       </c>
-      <c r="N87" t="s" s="2">
+      <c r="O87" t="s" s="2">
         <v>655</v>
-      </c>
-      <c r="O87" t="s" s="2">
-        <v>656</v>
       </c>
       <c r="P87" t="s" s="2">
         <v>82</v>
@@ -13947,28 +13940,28 @@
         <v>242</v>
       </c>
       <c r="Y87" t="s" s="2">
+        <v>656</v>
+      </c>
+      <c r="Z87" t="s" s="2">
         <v>657</v>
       </c>
-      <c r="Z87" t="s" s="2">
+      <c r="AA87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF87" t="s" s="2">
         <v>658</v>
-      </c>
-      <c r="AA87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF87" t="s" s="2">
-        <v>659</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>83</v>
@@ -13995,7 +13988,7 @@
         <v>82</v>
       </c>
       <c r="AO87" t="s" s="2">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="AP87" t="s" s="2">
         <v>82</v>
@@ -14012,10 +14005,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
+        <v>660</v>
+      </c>
+      <c r="B88" t="s" s="2">
         <v>661</v>
-      </c>
-      <c r="B88" t="s" s="2">
-        <v>662</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -14041,16 +14034,16 @@
         <v>259</v>
       </c>
       <c r="L88" t="s" s="2">
+        <v>662</v>
+      </c>
+      <c r="M88" t="s" s="2">
         <v>663</v>
       </c>
-      <c r="M88" t="s" s="2">
+      <c r="N88" t="s" s="2">
         <v>664</v>
       </c>
-      <c r="N88" t="s" s="2">
+      <c r="O88" t="s" s="2">
         <v>665</v>
-      </c>
-      <c r="O88" t="s" s="2">
-        <v>666</v>
       </c>
       <c r="P88" t="s" s="2">
         <v>82</v>
@@ -14078,28 +14071,28 @@
         <v>157</v>
       </c>
       <c r="Y88" t="s" s="2">
+        <v>666</v>
+      </c>
+      <c r="Z88" t="s" s="2">
         <v>667</v>
       </c>
-      <c r="Z88" t="s" s="2">
+      <c r="AA88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF88" t="s" s="2">
         <v>668</v>
-      </c>
-      <c r="AA88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF88" t="s" s="2">
-        <v>669</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>83</v>
@@ -14126,7 +14119,7 @@
         <v>82</v>
       </c>
       <c r="AO88" t="s" s="2">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="AP88" t="s" s="2">
         <v>82</v>
@@ -14135,7 +14128,7 @@
         <v>82</v>
       </c>
       <c r="AR88" t="s" s="2">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="AS88" t="s" s="2">
         <v>82</v>
@@ -14143,10 +14136,10 @@
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
+        <v>670</v>
+      </c>
+      <c r="B89" t="s" s="2">
         <v>671</v>
-      </c>
-      <c r="B89" t="s" s="2">
-        <v>672</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -14270,10 +14263,10 @@
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
+        <v>672</v>
+      </c>
+      <c r="B90" t="s" s="2">
         <v>673</v>
-      </c>
-      <c r="B90" t="s" s="2">
-        <v>674</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -14399,10 +14392,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
+        <v>674</v>
+      </c>
+      <c r="B91" t="s" s="2">
         <v>675</v>
-      </c>
-      <c r="B91" t="s" s="2">
-        <v>676</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -14428,16 +14421,16 @@
         <v>153</v>
       </c>
       <c r="L91" t="s" s="2">
+        <v>676</v>
+      </c>
+      <c r="M91" t="s" s="2">
         <v>677</v>
       </c>
-      <c r="M91" t="s" s="2">
+      <c r="N91" t="s" s="2">
         <v>678</v>
       </c>
-      <c r="N91" t="s" s="2">
+      <c r="O91" t="s" s="2">
         <v>679</v>
-      </c>
-      <c r="O91" t="s" s="2">
-        <v>680</v>
       </c>
       <c r="P91" t="s" s="2">
         <v>82</v>
@@ -14486,7 +14479,7 @@
         <v>82</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>83</v>
@@ -14513,16 +14506,16 @@
         <v>82</v>
       </c>
       <c r="AO91" t="s" s="2">
+        <v>681</v>
+      </c>
+      <c r="AP91" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ91" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR91" t="s" s="2">
         <v>682</v>
-      </c>
-      <c r="AP91" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ91" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR91" t="s" s="2">
-        <v>683</v>
       </c>
       <c r="AS91" t="s" s="2">
         <v>82</v>
@@ -14530,10 +14523,10 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
+        <v>683</v>
+      </c>
+      <c r="B92" t="s" s="2">
         <v>684</v>
-      </c>
-      <c r="B92" t="s" s="2">
-        <v>685</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -14657,10 +14650,10 @@
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
+        <v>685</v>
+      </c>
+      <c r="B93" t="s" s="2">
         <v>686</v>
-      </c>
-      <c r="B93" t="s" s="2">
-        <v>687</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -14786,10 +14779,10 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
+        <v>687</v>
+      </c>
+      <c r="B94" t="s" s="2">
         <v>688</v>
-      </c>
-      <c r="B94" t="s" s="2">
-        <v>689</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -14815,16 +14808,16 @@
         <v>140</v>
       </c>
       <c r="L94" t="s" s="2">
+        <v>689</v>
+      </c>
+      <c r="M94" t="s" s="2">
         <v>690</v>
       </c>
-      <c r="M94" t="s" s="2">
+      <c r="N94" t="s" s="2">
         <v>691</v>
       </c>
-      <c r="N94" t="s" s="2">
+      <c r="O94" t="s" s="2">
         <v>692</v>
-      </c>
-      <c r="O94" t="s" s="2">
-        <v>693</v>
       </c>
       <c r="P94" t="s" s="2">
         <v>82</v>
@@ -14834,46 +14827,46 @@
         <v>82</v>
       </c>
       <c r="S94" t="s" s="2">
+        <v>693</v>
+      </c>
+      <c r="T94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF94" t="s" s="2">
         <v>694</v>
-      </c>
-      <c r="T94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF94" t="s" s="2">
-        <v>695</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>83</v>
@@ -14900,16 +14893,16 @@
         <v>82</v>
       </c>
       <c r="AO94" t="s" s="2">
+        <v>695</v>
+      </c>
+      <c r="AP94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR94" t="s" s="2">
         <v>696</v>
-      </c>
-      <c r="AP94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR94" t="s" s="2">
-        <v>697</v>
       </c>
       <c r="AS94" t="s" s="2">
         <v>82</v>
@@ -14917,10 +14910,10 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
+        <v>697</v>
+      </c>
+      <c r="B95" t="s" s="2">
         <v>698</v>
-      </c>
-      <c r="B95" t="s" s="2">
-        <v>699</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -14946,13 +14939,13 @@
         <v>111</v>
       </c>
       <c r="L95" t="s" s="2">
+        <v>699</v>
+      </c>
+      <c r="M95" t="s" s="2">
         <v>700</v>
       </c>
-      <c r="M95" t="s" s="2">
+      <c r="N95" t="s" s="2">
         <v>701</v>
-      </c>
-      <c r="N95" t="s" s="2">
-        <v>702</v>
       </c>
       <c r="O95" s="2"/>
       <c r="P95" t="s" s="2">
@@ -15002,7 +14995,7 @@
         <v>82</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>83</v>
@@ -15029,16 +15022,16 @@
         <v>82</v>
       </c>
       <c r="AO95" t="s" s="2">
+        <v>703</v>
+      </c>
+      <c r="AP95" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ95" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR95" t="s" s="2">
         <v>704</v>
-      </c>
-      <c r="AP95" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ95" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR95" t="s" s="2">
-        <v>705</v>
       </c>
       <c r="AS95" t="s" s="2">
         <v>82</v>
@@ -15046,10 +15039,10 @@
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
+        <v>705</v>
+      </c>
+      <c r="B96" t="s" s="2">
         <v>706</v>
-      </c>
-      <c r="B96" t="s" s="2">
-        <v>707</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -15075,14 +15068,14 @@
         <v>175</v>
       </c>
       <c r="L96" t="s" s="2">
+        <v>707</v>
+      </c>
+      <c r="M96" t="s" s="2">
         <v>708</v>
-      </c>
-      <c r="M96" t="s" s="2">
-        <v>709</v>
       </c>
       <c r="N96" s="2"/>
       <c r="O96" t="s" s="2">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="P96" t="s" s="2">
         <v>82</v>
@@ -15131,7 +15124,7 @@
         <v>82</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>83</v>
@@ -15167,7 +15160,7 @@
         <v>82</v>
       </c>
       <c r="AR96" t="s" s="2">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="AS96" t="s" s="2">
         <v>82</v>
@@ -15175,10 +15168,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
+        <v>712</v>
+      </c>
+      <c r="B97" t="s" s="2">
         <v>713</v>
-      </c>
-      <c r="B97" t="s" s="2">
-        <v>714</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -15204,14 +15197,14 @@
         <v>111</v>
       </c>
       <c r="L97" t="s" s="2">
+        <v>714</v>
+      </c>
+      <c r="M97" t="s" s="2">
         <v>715</v>
-      </c>
-      <c r="M97" t="s" s="2">
-        <v>716</v>
       </c>
       <c r="N97" s="2"/>
       <c r="O97" t="s" s="2">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="P97" t="s" s="2">
         <v>82</v>
@@ -15260,7 +15253,7 @@
         <v>82</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>83</v>
@@ -15287,16 +15280,16 @@
         <v>82</v>
       </c>
       <c r="AO97" t="s" s="2">
+        <v>718</v>
+      </c>
+      <c r="AP97" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ97" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR97" t="s" s="2">
         <v>719</v>
-      </c>
-      <c r="AP97" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ97" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR97" t="s" s="2">
-        <v>720</v>
       </c>
       <c r="AS97" t="s" s="2">
         <v>82</v>
@@ -15304,10 +15297,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
+        <v>720</v>
+      </c>
+      <c r="B98" t="s" s="2">
         <v>721</v>
-      </c>
-      <c r="B98" t="s" s="2">
-        <v>722</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -15330,19 +15323,19 @@
         <v>98</v>
       </c>
       <c r="K98" t="s" s="2">
+        <v>722</v>
+      </c>
+      <c r="L98" t="s" s="2">
         <v>723</v>
       </c>
-      <c r="L98" t="s" s="2">
+      <c r="M98" t="s" s="2">
         <v>724</v>
       </c>
-      <c r="M98" t="s" s="2">
+      <c r="N98" t="s" s="2">
         <v>725</v>
       </c>
-      <c r="N98" t="s" s="2">
+      <c r="O98" t="s" s="2">
         <v>726</v>
-      </c>
-      <c r="O98" t="s" s="2">
-        <v>727</v>
       </c>
       <c r="P98" t="s" s="2">
         <v>82</v>
@@ -15391,7 +15384,7 @@
         <v>82</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>83</v>
@@ -15418,16 +15411,16 @@
         <v>82</v>
       </c>
       <c r="AO98" t="s" s="2">
+        <v>728</v>
+      </c>
+      <c r="AP98" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ98" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR98" t="s" s="2">
         <v>729</v>
-      </c>
-      <c r="AP98" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ98" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR98" t="s" s="2">
-        <v>730</v>
       </c>
       <c r="AS98" t="s" s="2">
         <v>82</v>
@@ -15435,10 +15428,10 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
+        <v>730</v>
+      </c>
+      <c r="B99" t="s" s="2">
         <v>731</v>
-      </c>
-      <c r="B99" t="s" s="2">
-        <v>732</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -15464,16 +15457,16 @@
         <v>111</v>
       </c>
       <c r="L99" t="s" s="2">
+        <v>732</v>
+      </c>
+      <c r="M99" t="s" s="2">
         <v>733</v>
       </c>
-      <c r="M99" t="s" s="2">
+      <c r="N99" t="s" s="2">
         <v>734</v>
       </c>
-      <c r="N99" t="s" s="2">
+      <c r="O99" t="s" s="2">
         <v>735</v>
-      </c>
-      <c r="O99" t="s" s="2">
-        <v>736</v>
       </c>
       <c r="P99" t="s" s="2">
         <v>82</v>
@@ -15522,7 +15515,7 @@
         <v>82</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>83</v>
@@ -15549,16 +15542,16 @@
         <v>82</v>
       </c>
       <c r="AO99" t="s" s="2">
+        <v>737</v>
+      </c>
+      <c r="AP99" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ99" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR99" t="s" s="2">
         <v>738</v>
-      </c>
-      <c r="AP99" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ99" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR99" t="s" s="2">
-        <v>739</v>
       </c>
       <c r="AS99" t="s" s="2">
         <v>82</v>
@@ -15566,10 +15559,10 @@
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
+        <v>739</v>
+      </c>
+      <c r="B100" t="s" s="2">
         <v>740</v>
-      </c>
-      <c r="B100" t="s" s="2">
-        <v>741</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -15595,16 +15588,16 @@
         <v>140</v>
       </c>
       <c r="L100" t="s" s="2">
+        <v>741</v>
+      </c>
+      <c r="M100" t="s" s="2">
         <v>742</v>
       </c>
-      <c r="M100" t="s" s="2">
+      <c r="N100" t="s" s="2">
         <v>743</v>
       </c>
-      <c r="N100" t="s" s="2">
+      <c r="O100" t="s" s="2">
         <v>744</v>
-      </c>
-      <c r="O100" t="s" s="2">
-        <v>745</v>
       </c>
       <c r="P100" t="s" s="2">
         <v>82</v>
@@ -15617,43 +15610,43 @@
         <v>82</v>
       </c>
       <c r="T100" t="s" s="2">
+        <v>745</v>
+      </c>
+      <c r="U100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF100" t="s" s="2">
         <v>746</v>
-      </c>
-      <c r="U100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF100" t="s" s="2">
-        <v>747</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>83</v>
@@ -15680,16 +15673,16 @@
         <v>82</v>
       </c>
       <c r="AO100" t="s" s="2">
+        <v>747</v>
+      </c>
+      <c r="AP100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR100" t="s" s="2">
         <v>748</v>
-      </c>
-      <c r="AP100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR100" t="s" s="2">
-        <v>749</v>
       </c>
       <c r="AS100" t="s" s="2">
         <v>82</v>
@@ -15697,10 +15690,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
+        <v>749</v>
+      </c>
+      <c r="B101" t="s" s="2">
         <v>750</v>
-      </c>
-      <c r="B101" t="s" s="2">
-        <v>751</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -15726,13 +15719,13 @@
         <v>111</v>
       </c>
       <c r="L101" t="s" s="2">
+        <v>751</v>
+      </c>
+      <c r="M101" t="s" s="2">
         <v>752</v>
       </c>
-      <c r="M101" t="s" s="2">
+      <c r="N101" t="s" s="2">
         <v>753</v>
-      </c>
-      <c r="N101" t="s" s="2">
-        <v>754</v>
       </c>
       <c r="O101" s="2"/>
       <c r="P101" t="s" s="2">
@@ -15746,43 +15739,43 @@
         <v>82</v>
       </c>
       <c r="T101" t="s" s="2">
+        <v>754</v>
+      </c>
+      <c r="U101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF101" t="s" s="2">
         <v>755</v>
-      </c>
-      <c r="U101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF101" t="s" s="2">
-        <v>756</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>83</v>
@@ -15809,16 +15802,16 @@
         <v>82</v>
       </c>
       <c r="AO101" t="s" s="2">
+        <v>756</v>
+      </c>
+      <c r="AP101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR101" t="s" s="2">
         <v>757</v>
-      </c>
-      <c r="AP101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR101" t="s" s="2">
-        <v>758</v>
       </c>
       <c r="AS101" t="s" s="2">
         <v>82</v>
@@ -15826,10 +15819,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
+        <v>758</v>
+      </c>
+      <c r="B102" t="s" s="2">
         <v>759</v>
-      </c>
-      <c r="B102" t="s" s="2">
-        <v>760</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -15852,13 +15845,13 @@
         <v>98</v>
       </c>
       <c r="K102" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="L102" t="s" s="2">
+        <v>760</v>
+      </c>
+      <c r="M102" t="s" s="2">
         <v>761</v>
-      </c>
-      <c r="M102" t="s" s="2">
-        <v>762</v>
       </c>
       <c r="N102" s="2"/>
       <c r="O102" s="2"/>
@@ -15909,7 +15902,7 @@
         <v>82</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>83</v>
@@ -15936,16 +15929,16 @@
         <v>82</v>
       </c>
       <c r="AO102" t="s" s="2">
+        <v>763</v>
+      </c>
+      <c r="AP102" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ102" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR102" t="s" s="2">
         <v>764</v>
-      </c>
-      <c r="AP102" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ102" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR102" t="s" s="2">
-        <v>765</v>
       </c>
       <c r="AS102" t="s" s="2">
         <v>82</v>
@@ -15953,10 +15946,10 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
+        <v>765</v>
+      </c>
+      <c r="B103" t="s" s="2">
         <v>766</v>
-      </c>
-      <c r="B103" t="s" s="2">
-        <v>767</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -15982,13 +15975,13 @@
         <v>333</v>
       </c>
       <c r="L103" t="s" s="2">
+        <v>767</v>
+      </c>
+      <c r="M103" t="s" s="2">
         <v>768</v>
       </c>
-      <c r="M103" t="s" s="2">
+      <c r="N103" t="s" s="2">
         <v>769</v>
-      </c>
-      <c r="N103" t="s" s="2">
-        <v>770</v>
       </c>
       <c r="O103" s="2"/>
       <c r="P103" t="s" s="2">
@@ -16038,7 +16031,7 @@
         <v>82</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>83</v>
@@ -16065,16 +16058,16 @@
         <v>82</v>
       </c>
       <c r="AO103" t="s" s="2">
+        <v>771</v>
+      </c>
+      <c r="AP103" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ103" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR103" t="s" s="2">
         <v>772</v>
-      </c>
-      <c r="AP103" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ103" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR103" t="s" s="2">
-        <v>773</v>
       </c>
       <c r="AS103" t="s" s="2">
         <v>82</v>
@@ -16082,10 +16075,10 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
+        <v>773</v>
+      </c>
+      <c r="B104" t="s" s="2">
         <v>774</v>
-      </c>
-      <c r="B104" t="s" s="2">
-        <v>775</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -16111,13 +16104,13 @@
         <v>111</v>
       </c>
       <c r="L104" t="s" s="2">
+        <v>617</v>
+      </c>
+      <c r="M104" t="s" s="2">
         <v>618</v>
       </c>
-      <c r="M104" t="s" s="2">
+      <c r="N104" t="s" s="2">
         <v>619</v>
-      </c>
-      <c r="N104" t="s" s="2">
-        <v>620</v>
       </c>
       <c r="O104" s="2"/>
       <c r="P104" t="s" s="2">
@@ -16167,7 +16160,7 @@
         <v>82</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>83</v>

</xml_diff>

<commit_message>
Documenter la valeur par défaut N sur securityLabel[confidentiality]
Ajoute une définition précisant qu'en l'absence d'information de
confidentialité, N (Normal) doit être utilisé par défaut, en
cohérence avec la pratique déjà en vigueur pour les documents CDA. 494105c0849e2a897d857cc26c40253453dbdcd6
</commit_message>
<xml_diff>
--- a/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4295" uniqueCount="775">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4295" uniqueCount="776">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-06T13:40:23+00:00</t>
+    <t>2026-08-06T13:54:33+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1279,6 +1279,9 @@
   </si>
   <si>
     <t>Niveau de confidentialité standard du document (Normal, Restreint, Très restreint).</t>
+  </si>
+  <si>
+    <t>En l'absence d'information de confidentialité disponible, la valeur par défaut à utiliser est N (Normal), conformément à ce qui est déjà pratiqué aujourd'hui pour les documents CDA.</t>
   </si>
   <si>
     <t>http://terminology.hl7.org/ValueSet/v3-ConfidentialityClassification</t>
@@ -7855,7 +7858,7 @@
         <v>402</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>389</v>
+        <v>403</v>
       </c>
       <c r="N40" t="s" s="2">
         <v>390</v>
@@ -7890,7 +7893,7 @@
       </c>
       <c r="Y40" s="2"/>
       <c r="Z40" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="AA40" t="s" s="2">
         <v>82</v>
@@ -7952,13 +7955,13 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B41" t="s" s="2">
         <v>387</v>
       </c>
       <c r="C41" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D41" t="s" s="2">
         <v>82</v>
@@ -7983,7 +7986,7 @@
         <v>259</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="M41" t="s" s="2">
         <v>389</v>
@@ -8021,7 +8024,7 @@
       </c>
       <c r="Y41" s="2"/>
       <c r="Z41" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AA41" t="s" s="2">
         <v>82</v>
@@ -8083,10 +8086,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -8112,10 +8115,10 @@
         <v>341</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -8166,7 +8169,7 @@
         <v>82</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>97</v>
@@ -8190,10 +8193,10 @@
         <v>82</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="AO42" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="AP42" t="s" s="2">
         <v>82</v>
@@ -8210,10 +8213,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -8337,10 +8340,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -8466,10 +8469,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -8597,10 +8600,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -8623,13 +8626,13 @@
         <v>98</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -8680,7 +8683,7 @@
         <v>82</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>97</v>
@@ -8704,30 +8707,30 @@
         <v>82</v>
       </c>
       <c r="AN46" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="AO46" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="AP46" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="AQ46" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AR46" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="AS46" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -8851,10 +8854,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -8980,10 +8983,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -9009,14 +9012,14 @@
         <v>175</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="P49" t="s" s="2">
         <v>82</v>
@@ -9029,7 +9032,7 @@
         <v>82</v>
       </c>
       <c r="T49" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="U49" t="s" s="2">
         <v>82</v>
@@ -9044,10 +9047,10 @@
         <v>242</v>
       </c>
       <c r="Y49" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="Z49" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="AA49" t="s" s="2">
         <v>82</v>
@@ -9065,7 +9068,7 @@
         <v>82</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>83</v>
@@ -9083,7 +9086,7 @@
         <v>82</v>
       </c>
       <c r="AL49" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="AM49" t="s" s="2">
         <v>82</v>
@@ -9092,7 +9095,7 @@
         <v>82</v>
       </c>
       <c r="AO49" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="AP49" t="s" s="2">
         <v>82</v>
@@ -9101,7 +9104,7 @@
         <v>82</v>
       </c>
       <c r="AR49" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="AS49" t="s" s="2">
         <v>82</v>
@@ -9109,10 +9112,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -9138,14 +9141,14 @@
         <v>175</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="P50" t="s" s="2">
         <v>82</v>
@@ -9158,7 +9161,7 @@
         <v>82</v>
       </c>
       <c r="T50" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="U50" t="s" s="2">
         <v>82</v>
@@ -9194,7 +9197,7 @@
         <v>82</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>83</v>
@@ -9209,10 +9212,10 @@
         <v>109</v>
       </c>
       <c r="AK50" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="AL50" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="AM50" t="s" s="2">
         <v>82</v>
@@ -9221,7 +9224,7 @@
         <v>82</v>
       </c>
       <c r="AO50" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="AP50" t="s" s="2">
         <v>82</v>
@@ -9238,10 +9241,10 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -9264,19 +9267,19 @@
         <v>82</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="N51" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="O51" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="P51" t="s" s="2">
         <v>82</v>
@@ -9325,7 +9328,7 @@
         <v>82</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>83</v>
@@ -9352,7 +9355,7 @@
         <v>82</v>
       </c>
       <c r="AO51" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="AP51" t="s" s="2">
         <v>82</v>
@@ -9361,7 +9364,7 @@
         <v>82</v>
       </c>
       <c r="AR51" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="AS51" t="s" s="2">
         <v>82</v>
@@ -9369,10 +9372,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -9395,19 +9398,19 @@
         <v>98</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="N52" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="O52" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="P52" t="s" s="2">
         <v>82</v>
@@ -9420,7 +9423,7 @@
         <v>82</v>
       </c>
       <c r="T52" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="U52" t="s" s="2">
         <v>82</v>
@@ -9456,7 +9459,7 @@
         <v>82</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>83</v>
@@ -9468,13 +9471,13 @@
         <v>82</v>
       </c>
       <c r="AJ52" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="AK52" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="AL52" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="AM52" t="s" s="2">
         <v>82</v>
@@ -9483,7 +9486,7 @@
         <v>82</v>
       </c>
       <c r="AO52" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="AP52" t="s" s="2">
         <v>82</v>
@@ -9492,7 +9495,7 @@
         <v>82</v>
       </c>
       <c r="AR52" t="s" s="2">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="AS52" t="s" s="2">
         <v>82</v>
@@ -9500,10 +9503,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -9526,19 +9529,19 @@
         <v>98</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="N53" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="O53" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="P53" t="s" s="2">
         <v>82</v>
@@ -9587,7 +9590,7 @@
         <v>82</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>83</v>
@@ -9605,7 +9608,7 @@
         <v>82</v>
       </c>
       <c r="AL53" t="s" s="2">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="AM53" t="s" s="2">
         <v>82</v>
@@ -9614,7 +9617,7 @@
         <v>82</v>
       </c>
       <c r="AO53" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="AP53" t="s" s="2">
         <v>82</v>
@@ -9631,10 +9634,10 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -9657,19 +9660,19 @@
         <v>98</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="N54" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="O54" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="P54" t="s" s="2">
         <v>82</v>
@@ -9718,7 +9721,7 @@
         <v>82</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>83</v>
@@ -9736,7 +9739,7 @@
         <v>82</v>
       </c>
       <c r="AL54" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="AM54" t="s" s="2">
         <v>82</v>
@@ -9745,7 +9748,7 @@
         <v>82</v>
       </c>
       <c r="AO54" t="s" s="2">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="AP54" t="s" s="2">
         <v>82</v>
@@ -9762,10 +9765,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -9791,14 +9794,14 @@
         <v>111</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" t="s" s="2">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="P55" t="s" s="2">
         <v>82</v>
@@ -9811,7 +9814,7 @@
         <v>82</v>
       </c>
       <c r="T55" t="s" s="2">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="U55" t="s" s="2">
         <v>82</v>
@@ -9847,7 +9850,7 @@
         <v>82</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>83</v>
@@ -9862,10 +9865,10 @@
         <v>109</v>
       </c>
       <c r="AK55" t="s" s="2">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="AL55" t="s" s="2">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="AM55" t="s" s="2">
         <v>82</v>
@@ -9874,7 +9877,7 @@
         <v>82</v>
       </c>
       <c r="AO55" t="s" s="2">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="AP55" t="s" s="2">
         <v>82</v>
@@ -9891,10 +9894,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -9917,17 +9920,17 @@
         <v>98</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" t="s" s="2">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="P56" t="s" s="2">
         <v>82</v>
@@ -9976,7 +9979,7 @@
         <v>82</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>83</v>
@@ -9991,10 +9994,10 @@
         <v>109</v>
       </c>
       <c r="AK56" t="s" s="2">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="AL56" t="s" s="2">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="AM56" t="s" s="2">
         <v>82</v>
@@ -10003,7 +10006,7 @@
         <v>82</v>
       </c>
       <c r="AO56" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="AP56" t="s" s="2">
         <v>82</v>
@@ -10020,10 +10023,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -10049,13 +10052,13 @@
         <v>153</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="N57" t="s" s="2">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="O57" s="2"/>
       <c r="P57" t="s" s="2">
@@ -10085,7 +10088,7 @@
       </c>
       <c r="Y57" s="2"/>
       <c r="Z57" t="s" s="2">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="AA57" t="s" s="2">
         <v>82</v>
@@ -10103,7 +10106,7 @@
         <v>82</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>83</v>
@@ -10115,42 +10118,42 @@
         <v>82</v>
       </c>
       <c r="AJ57" t="s" s="2">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="AK57" t="s" s="2">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="AL57" t="s" s="2">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="AM57" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN57" t="s" s="2">
+        <v>511</v>
+      </c>
+      <c r="AO57" t="s" s="2">
+        <v>413</v>
+      </c>
+      <c r="AP57" t="s" s="2">
+        <v>512</v>
+      </c>
+      <c r="AQ57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AS57" t="s" s="2">
         <v>510</v>
-      </c>
-      <c r="AO57" t="s" s="2">
-        <v>412</v>
-      </c>
-      <c r="AP57" t="s" s="2">
-        <v>511</v>
-      </c>
-      <c r="AQ57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AS57" t="s" s="2">
-        <v>509</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -10176,13 +10179,13 @@
         <v>341</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="N58" t="s" s="2">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
@@ -10232,7 +10235,7 @@
         <v>82</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>83</v>
@@ -10259,7 +10262,7 @@
         <v>82</v>
       </c>
       <c r="AO58" t="s" s="2">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="AP58" t="s" s="2">
         <v>82</v>
@@ -10276,10 +10279,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -10403,10 +10406,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -10532,10 +10535,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -10663,10 +10666,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -10689,13 +10692,13 @@
         <v>82</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -10746,7 +10749,7 @@
         <v>82</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>83</v>
@@ -10764,22 +10767,22 @@
         <v>82</v>
       </c>
       <c r="AL62" t="s" s="2">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="AM62" t="s" s="2">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="AN62" t="s" s="2">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AO62" t="s" s="2">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="AP62" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AQ62" t="s" s="2">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="AR62" t="s" s="2">
         <v>82</v>
@@ -10790,10 +10793,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -10819,13 +10822,13 @@
         <v>259</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="N63" t="s" s="2">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="O63" s="2"/>
       <c r="P63" t="s" s="2">
@@ -10854,10 +10857,10 @@
         <v>165</v>
       </c>
       <c r="Y63" t="s" s="2">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="Z63" t="s" s="2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="AA63" t="s" s="2">
         <v>82</v>
@@ -10875,7 +10878,7 @@
         <v>82</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>83</v>
@@ -10887,42 +10890,42 @@
         <v>82</v>
       </c>
       <c r="AJ63" t="s" s="2">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="AK63" t="s" s="2">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="AL63" t="s" s="2">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="AM63" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN63" t="s" s="2">
+        <v>539</v>
+      </c>
+      <c r="AO63" t="s" s="2">
+        <v>540</v>
+      </c>
+      <c r="AP63" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ63" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR63" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AS63" t="s" s="2">
         <v>538</v>
-      </c>
-      <c r="AO63" t="s" s="2">
-        <v>539</v>
-      </c>
-      <c r="AP63" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ63" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR63" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AS63" t="s" s="2">
-        <v>537</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -10945,13 +10948,13 @@
         <v>98</v>
       </c>
       <c r="K64" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
@@ -11002,7 +11005,7 @@
         <v>82</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>83</v>
@@ -11026,13 +11029,13 @@
         <v>82</v>
       </c>
       <c r="AN64" t="s" s="2">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="AO64" t="s" s="2">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="AP64" t="s" s="2">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="AQ64" t="s" s="2">
         <v>82</v>
@@ -11041,15 +11044,15 @@
         <v>82</v>
       </c>
       <c r="AS64" t="s" s="2">
-        <v>547</v>
+        <v>548</v>
       </c>
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -11173,10 +11176,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -11302,10 +11305,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -11328,16 +11331,16 @@
         <v>98</v>
       </c>
       <c r="K67" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="L67" t="s" s="2">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="M67" t="s" s="2">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="N67" t="s" s="2">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="O67" s="2"/>
       <c r="P67" t="s" s="2">
@@ -11387,7 +11390,7 @@
         <v>82</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>83</v>
@@ -11396,16 +11399,16 @@
         <v>97</v>
       </c>
       <c r="AI67" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="AJ67" t="s" s="2">
         <v>109</v>
       </c>
       <c r="AK67" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="AL67" t="s" s="2">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="AM67" t="s" s="2">
         <v>82</v>
@@ -11414,7 +11417,7 @@
         <v>82</v>
       </c>
       <c r="AO67" t="s" s="2">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="AP67" t="s" s="2">
         <v>82</v>
@@ -11423,7 +11426,7 @@
         <v>82</v>
       </c>
       <c r="AR67" t="s" s="2">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="AS67" t="s" s="2">
         <v>82</v>
@@ -11431,10 +11434,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -11457,23 +11460,23 @@
         <v>98</v>
       </c>
       <c r="K68" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="L68" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="M68" t="s" s="2">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="N68" t="s" s="2">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="O68" s="2"/>
       <c r="P68" t="s" s="2">
         <v>82</v>
       </c>
       <c r="Q68" t="s" s="2">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="R68" t="s" s="2">
         <v>82</v>
@@ -11518,7 +11521,7 @@
         <v>82</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>83</v>
@@ -11527,16 +11530,16 @@
         <v>97</v>
       </c>
       <c r="AI68" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="AJ68" t="s" s="2">
         <v>109</v>
       </c>
       <c r="AK68" t="s" s="2">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="AL68" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="AM68" t="s" s="2">
         <v>82</v>
@@ -11545,7 +11548,7 @@
         <v>82</v>
       </c>
       <c r="AO68" t="s" s="2">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="AP68" t="s" s="2">
         <v>82</v>
@@ -11554,7 +11557,7 @@
         <v>82</v>
       </c>
       <c r="AR68" t="s" s="2">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="AS68" t="s" s="2">
         <v>82</v>
@@ -11562,10 +11565,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -11591,10 +11594,10 @@
         <v>259</v>
       </c>
       <c r="L69" t="s" s="2">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="M69" t="s" s="2">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
@@ -11625,7 +11628,7 @@
       </c>
       <c r="Y69" s="2"/>
       <c r="Z69" t="s" s="2">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="AA69" t="s" s="2">
         <v>82</v>
@@ -11643,7 +11646,7 @@
         <v>82</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>83</v>
@@ -11655,42 +11658,42 @@
         <v>82</v>
       </c>
       <c r="AJ69" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="AK69" t="s" s="2">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="AL69" t="s" s="2">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="AM69" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN69" t="s" s="2">
+        <v>578</v>
+      </c>
+      <c r="AO69" t="s" s="2">
+        <v>579</v>
+      </c>
+      <c r="AP69" t="s" s="2">
+        <v>580</v>
+      </c>
+      <c r="AQ69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AS69" t="s" s="2">
         <v>577</v>
-      </c>
-      <c r="AO69" t="s" s="2">
-        <v>578</v>
-      </c>
-      <c r="AP69" t="s" s="2">
-        <v>579</v>
-      </c>
-      <c r="AQ69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AS69" t="s" s="2">
-        <v>576</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -11716,16 +11719,16 @@
         <v>259</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="N70" t="s" s="2">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="O70" t="s" s="2">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="P70" t="s" s="2">
         <v>82</v>
@@ -11754,7 +11757,7 @@
       </c>
       <c r="Y70" s="2"/>
       <c r="Z70" t="s" s="2">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="AA70" t="s" s="2">
         <v>82</v>
@@ -11772,7 +11775,7 @@
         <v>82</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>83</v>
@@ -11784,26 +11787,26 @@
         <v>82</v>
       </c>
       <c r="AJ70" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="AK70" t="s" s="2">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="AL70" t="s" s="2">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="AM70" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN70" t="s" s="2">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="AO70" t="s" s="2">
+        <v>579</v>
+      </c>
+      <c r="AP70" t="s" s="2">
         <v>578</v>
       </c>
-      <c r="AP70" t="s" s="2">
-        <v>577</v>
-      </c>
       <c r="AQ70" t="s" s="2">
         <v>82</v>
       </c>
@@ -11811,15 +11814,15 @@
         <v>82</v>
       </c>
       <c r="AS70" t="s" s="2">
-        <v>587</v>
+        <v>588</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -11842,13 +11845,13 @@
         <v>82</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
@@ -11899,7 +11902,7 @@
         <v>82</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>83</v>
@@ -11938,15 +11941,15 @@
         <v>82</v>
       </c>
       <c r="AS71" t="s" s="2">
-        <v>592</v>
+        <v>593</v>
       </c>
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -12070,10 +12073,10 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -12199,10 +12202,10 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -12228,13 +12231,13 @@
         <v>111</v>
       </c>
       <c r="L74" t="s" s="2">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="M74" t="s" s="2">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="N74" t="s" s="2">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="O74" s="2"/>
       <c r="P74" t="s" s="2">
@@ -12284,7 +12287,7 @@
         <v>82</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>83</v>
@@ -12293,7 +12296,7 @@
         <v>97</v>
       </c>
       <c r="AI74" t="s" s="2">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="AJ74" t="s" s="2">
         <v>109</v>
@@ -12302,7 +12305,7 @@
         <v>82</v>
       </c>
       <c r="AL74" t="s" s="2">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="AM74" t="s" s="2">
         <v>82</v>
@@ -12328,10 +12331,10 @@
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -12357,13 +12360,13 @@
         <v>140</v>
       </c>
       <c r="L75" t="s" s="2">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="M75" t="s" s="2">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="N75" t="s" s="2">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="O75" s="2"/>
       <c r="P75" t="s" s="2">
@@ -12392,10 +12395,10 @@
         <v>157</v>
       </c>
       <c r="Y75" t="s" s="2">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="Z75" t="s" s="2">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="AA75" t="s" s="2">
         <v>82</v>
@@ -12413,7 +12416,7 @@
         <v>82</v>
       </c>
       <c r="AF75" t="s" s="2">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>83</v>
@@ -12457,10 +12460,10 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -12486,13 +12489,13 @@
         <v>227</v>
       </c>
       <c r="L76" t="s" s="2">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="M76" t="s" s="2">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="N76" t="s" s="2">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="O76" s="2"/>
       <c r="P76" t="s" s="2">
@@ -12542,7 +12545,7 @@
         <v>82</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>83</v>
@@ -12560,7 +12563,7 @@
         <v>82</v>
       </c>
       <c r="AL76" t="s" s="2">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="AM76" t="s" s="2">
         <v>82</v>
@@ -12569,7 +12572,7 @@
         <v>82</v>
       </c>
       <c r="AO76" t="s" s="2">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="AP76" t="s" s="2">
         <v>82</v>
@@ -12586,10 +12589,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -12615,13 +12618,13 @@
         <v>111</v>
       </c>
       <c r="L77" t="s" s="2">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="M77" t="s" s="2">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="N77" t="s" s="2">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="O77" s="2"/>
       <c r="P77" t="s" s="2">
@@ -12671,7 +12674,7 @@
         <v>82</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>83</v>
@@ -12715,10 +12718,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -12741,16 +12744,16 @@
         <v>82</v>
       </c>
       <c r="K78" t="s" s="2">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="L78" t="s" s="2">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="M78" t="s" s="2">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="N78" t="s" s="2">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="O78" s="2"/>
       <c r="P78" t="s" s="2">
@@ -12788,10 +12791,10 @@
         <v>82</v>
       </c>
       <c r="AB78" t="s" s="2">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="AC78" t="s" s="2">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="AD78" t="s" s="2">
         <v>82</v>
@@ -12800,7 +12803,7 @@
         <v>124</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>83</v>
@@ -12818,19 +12821,19 @@
         <v>82</v>
       </c>
       <c r="AL78" t="s" s="2">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="AM78" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN78" t="s" s="2">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="AO78" t="s" s="2">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="AP78" t="s" s="2">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="AQ78" t="s" s="2">
         <v>82</v>
@@ -12839,18 +12842,18 @@
         <v>82</v>
       </c>
       <c r="AS78" t="s" s="2">
-        <v>632</v>
+        <v>633</v>
       </c>
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C79" t="s" s="2">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="D79" t="s" s="2">
         <v>82</v>
@@ -12872,16 +12875,16 @@
         <v>82</v>
       </c>
       <c r="K79" t="s" s="2">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="M79" t="s" s="2">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="N79" t="s" s="2">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="O79" s="2"/>
       <c r="P79" t="s" s="2">
@@ -12931,7 +12934,7 @@
         <v>82</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>83</v>
@@ -12949,19 +12952,19 @@
         <v>82</v>
       </c>
       <c r="AL79" t="s" s="2">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="AM79" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN79" t="s" s="2">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="AO79" t="s" s="2">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="AP79" t="s" s="2">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="AQ79" t="s" s="2">
         <v>82</v>
@@ -12970,15 +12973,15 @@
         <v>82</v>
       </c>
       <c r="AS79" t="s" s="2">
-        <v>632</v>
+        <v>633</v>
       </c>
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -13102,10 +13105,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -13231,10 +13234,10 @@
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -13260,13 +13263,13 @@
         <v>111</v>
       </c>
       <c r="L82" t="s" s="2">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="M82" t="s" s="2">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="N82" t="s" s="2">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="O82" s="2"/>
       <c r="P82" t="s" s="2">
@@ -13316,7 +13319,7 @@
         <v>82</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>83</v>
@@ -13325,7 +13328,7 @@
         <v>97</v>
       </c>
       <c r="AI82" t="s" s="2">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="AJ82" t="s" s="2">
         <v>109</v>
@@ -13360,10 +13363,10 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -13389,13 +13392,13 @@
         <v>140</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="N83" t="s" s="2">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="O83" s="2"/>
       <c r="P83" t="s" s="2">
@@ -13424,10 +13427,10 @@
         <v>157</v>
       </c>
       <c r="Y83" t="s" s="2">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="Z83" t="s" s="2">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="AA83" t="s" s="2">
         <v>82</v>
@@ -13445,7 +13448,7 @@
         <v>82</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>83</v>
@@ -13489,10 +13492,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -13518,13 +13521,13 @@
         <v>227</v>
       </c>
       <c r="L84" t="s" s="2">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="M84" t="s" s="2">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="N84" t="s" s="2">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="O84" s="2"/>
       <c r="P84" t="s" s="2">
@@ -13574,7 +13577,7 @@
         <v>82</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>83</v>
@@ -13601,7 +13604,7 @@
         <v>82</v>
       </c>
       <c r="AO84" t="s" s="2">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="AP84" t="s" s="2">
         <v>82</v>
@@ -13618,10 +13621,10 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -13745,10 +13748,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -13874,10 +13877,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -13903,16 +13906,16 @@
         <v>175</v>
       </c>
       <c r="L87" t="s" s="2">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="M87" t="s" s="2">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="N87" t="s" s="2">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="O87" t="s" s="2">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="P87" t="s" s="2">
         <v>82</v>
@@ -13940,10 +13943,10 @@
         <v>242</v>
       </c>
       <c r="Y87" t="s" s="2">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="Z87" t="s" s="2">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="AA87" t="s" s="2">
         <v>82</v>
@@ -13961,7 +13964,7 @@
         <v>82</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>83</v>
@@ -13988,7 +13991,7 @@
         <v>82</v>
       </c>
       <c r="AO87" t="s" s="2">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="AP87" t="s" s="2">
         <v>82</v>
@@ -14005,10 +14008,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -14034,16 +14037,16 @@
         <v>259</v>
       </c>
       <c r="L88" t="s" s="2">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="M88" t="s" s="2">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="N88" t="s" s="2">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="O88" t="s" s="2">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="P88" t="s" s="2">
         <v>82</v>
@@ -14071,10 +14074,10 @@
         <v>157</v>
       </c>
       <c r="Y88" t="s" s="2">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="Z88" t="s" s="2">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="AA88" t="s" s="2">
         <v>82</v>
@@ -14092,7 +14095,7 @@
         <v>82</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>83</v>
@@ -14119,7 +14122,7 @@
         <v>82</v>
       </c>
       <c r="AO88" t="s" s="2">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="AP88" t="s" s="2">
         <v>82</v>
@@ -14128,7 +14131,7 @@
         <v>82</v>
       </c>
       <c r="AR88" t="s" s="2">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="AS88" t="s" s="2">
         <v>82</v>
@@ -14136,10 +14139,10 @@
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -14263,10 +14266,10 @@
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -14392,10 +14395,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -14421,16 +14424,16 @@
         <v>153</v>
       </c>
       <c r="L91" t="s" s="2">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="M91" t="s" s="2">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="N91" t="s" s="2">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="O91" t="s" s="2">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="P91" t="s" s="2">
         <v>82</v>
@@ -14479,7 +14482,7 @@
         <v>82</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>83</v>
@@ -14506,7 +14509,7 @@
         <v>82</v>
       </c>
       <c r="AO91" t="s" s="2">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="AP91" t="s" s="2">
         <v>82</v>
@@ -14515,7 +14518,7 @@
         <v>82</v>
       </c>
       <c r="AR91" t="s" s="2">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="AS91" t="s" s="2">
         <v>82</v>
@@ -14523,10 +14526,10 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -14650,10 +14653,10 @@
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -14779,10 +14782,10 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -14808,16 +14811,16 @@
         <v>140</v>
       </c>
       <c r="L94" t="s" s="2">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="M94" t="s" s="2">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="N94" t="s" s="2">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="O94" t="s" s="2">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="P94" t="s" s="2">
         <v>82</v>
@@ -14827,7 +14830,7 @@
         <v>82</v>
       </c>
       <c r="S94" t="s" s="2">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="T94" t="s" s="2">
         <v>82</v>
@@ -14866,7 +14869,7 @@
         <v>82</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>83</v>
@@ -14893,7 +14896,7 @@
         <v>82</v>
       </c>
       <c r="AO94" t="s" s="2">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="AP94" t="s" s="2">
         <v>82</v>
@@ -14902,7 +14905,7 @@
         <v>82</v>
       </c>
       <c r="AR94" t="s" s="2">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="AS94" t="s" s="2">
         <v>82</v>
@@ -14910,10 +14913,10 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -14939,13 +14942,13 @@
         <v>111</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="N95" t="s" s="2">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="O95" s="2"/>
       <c r="P95" t="s" s="2">
@@ -14995,7 +14998,7 @@
         <v>82</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>83</v>
@@ -15022,7 +15025,7 @@
         <v>82</v>
       </c>
       <c r="AO95" t="s" s="2">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="AP95" t="s" s="2">
         <v>82</v>
@@ -15031,7 +15034,7 @@
         <v>82</v>
       </c>
       <c r="AR95" t="s" s="2">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="AS95" t="s" s="2">
         <v>82</v>
@@ -15039,10 +15042,10 @@
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -15068,14 +15071,14 @@
         <v>175</v>
       </c>
       <c r="L96" t="s" s="2">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="M96" t="s" s="2">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="N96" s="2"/>
       <c r="O96" t="s" s="2">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="P96" t="s" s="2">
         <v>82</v>
@@ -15124,7 +15127,7 @@
         <v>82</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>83</v>
@@ -15160,7 +15163,7 @@
         <v>82</v>
       </c>
       <c r="AR96" t="s" s="2">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="AS96" t="s" s="2">
         <v>82</v>
@@ -15168,10 +15171,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -15197,14 +15200,14 @@
         <v>111</v>
       </c>
       <c r="L97" t="s" s="2">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="M97" t="s" s="2">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="N97" s="2"/>
       <c r="O97" t="s" s="2">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="P97" t="s" s="2">
         <v>82</v>
@@ -15253,7 +15256,7 @@
         <v>82</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>83</v>
@@ -15280,7 +15283,7 @@
         <v>82</v>
       </c>
       <c r="AO97" t="s" s="2">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="AP97" t="s" s="2">
         <v>82</v>
@@ -15289,7 +15292,7 @@
         <v>82</v>
       </c>
       <c r="AR97" t="s" s="2">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="AS97" t="s" s="2">
         <v>82</v>
@@ -15297,10 +15300,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -15323,19 +15326,19 @@
         <v>98</v>
       </c>
       <c r="K98" t="s" s="2">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="L98" t="s" s="2">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="M98" t="s" s="2">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="N98" t="s" s="2">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="O98" t="s" s="2">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="P98" t="s" s="2">
         <v>82</v>
@@ -15384,7 +15387,7 @@
         <v>82</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>83</v>
@@ -15411,7 +15414,7 @@
         <v>82</v>
       </c>
       <c r="AO98" t="s" s="2">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="AP98" t="s" s="2">
         <v>82</v>
@@ -15420,7 +15423,7 @@
         <v>82</v>
       </c>
       <c r="AR98" t="s" s="2">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="AS98" t="s" s="2">
         <v>82</v>
@@ -15428,10 +15431,10 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -15457,16 +15460,16 @@
         <v>111</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="M99" t="s" s="2">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="N99" t="s" s="2">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="O99" t="s" s="2">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="P99" t="s" s="2">
         <v>82</v>
@@ -15515,7 +15518,7 @@
         <v>82</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>83</v>
@@ -15542,7 +15545,7 @@
         <v>82</v>
       </c>
       <c r="AO99" t="s" s="2">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="AP99" t="s" s="2">
         <v>82</v>
@@ -15551,7 +15554,7 @@
         <v>82</v>
       </c>
       <c r="AR99" t="s" s="2">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="AS99" t="s" s="2">
         <v>82</v>
@@ -15559,10 +15562,10 @@
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -15588,16 +15591,16 @@
         <v>140</v>
       </c>
       <c r="L100" t="s" s="2">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="M100" t="s" s="2">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="N100" t="s" s="2">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="O100" t="s" s="2">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="P100" t="s" s="2">
         <v>82</v>
@@ -15610,7 +15613,7 @@
         <v>82</v>
       </c>
       <c r="T100" t="s" s="2">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="U100" t="s" s="2">
         <v>82</v>
@@ -15646,7 +15649,7 @@
         <v>82</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>83</v>
@@ -15673,7 +15676,7 @@
         <v>82</v>
       </c>
       <c r="AO100" t="s" s="2">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="AP100" t="s" s="2">
         <v>82</v>
@@ -15682,7 +15685,7 @@
         <v>82</v>
       </c>
       <c r="AR100" t="s" s="2">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="AS100" t="s" s="2">
         <v>82</v>
@@ -15690,10 +15693,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -15719,13 +15722,13 @@
         <v>111</v>
       </c>
       <c r="L101" t="s" s="2">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="M101" t="s" s="2">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="N101" t="s" s="2">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="O101" s="2"/>
       <c r="P101" t="s" s="2">
@@ -15739,7 +15742,7 @@
         <v>82</v>
       </c>
       <c r="T101" t="s" s="2">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="U101" t="s" s="2">
         <v>82</v>
@@ -15775,7 +15778,7 @@
         <v>82</v>
       </c>
       <c r="AF101" t="s" s="2">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>83</v>
@@ -15802,7 +15805,7 @@
         <v>82</v>
       </c>
       <c r="AO101" t="s" s="2">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="AP101" t="s" s="2">
         <v>82</v>
@@ -15811,7 +15814,7 @@
         <v>82</v>
       </c>
       <c r="AR101" t="s" s="2">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="AS101" t="s" s="2">
         <v>82</v>
@@ -15819,10 +15822,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -15845,13 +15848,13 @@
         <v>98</v>
       </c>
       <c r="K102" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="L102" t="s" s="2">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="M102" t="s" s="2">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="N102" s="2"/>
       <c r="O102" s="2"/>
@@ -15902,7 +15905,7 @@
         <v>82</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>83</v>
@@ -15929,7 +15932,7 @@
         <v>82</v>
       </c>
       <c r="AO102" t="s" s="2">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="AP102" t="s" s="2">
         <v>82</v>
@@ -15938,7 +15941,7 @@
         <v>82</v>
       </c>
       <c r="AR102" t="s" s="2">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="AS102" t="s" s="2">
         <v>82</v>
@@ -15946,10 +15949,10 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -15975,13 +15978,13 @@
         <v>333</v>
       </c>
       <c r="L103" t="s" s="2">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="M103" t="s" s="2">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="N103" t="s" s="2">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="O103" s="2"/>
       <c r="P103" t="s" s="2">
@@ -16031,7 +16034,7 @@
         <v>82</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>83</v>
@@ -16058,7 +16061,7 @@
         <v>82</v>
       </c>
       <c r="AO103" t="s" s="2">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="AP103" t="s" s="2">
         <v>82</v>
@@ -16067,7 +16070,7 @@
         <v>82</v>
       </c>
       <c r="AR103" t="s" s="2">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="AS103" t="s" s="2">
         <v>82</v>
@@ -16075,10 +16078,10 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -16104,13 +16107,13 @@
         <v>111</v>
       </c>
       <c r="L104" t="s" s="2">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="M104" t="s" s="2">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="N104" t="s" s="2">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="O104" s="2"/>
       <c r="P104" t="s" s="2">
@@ -16160,7 +16163,7 @@
         <v>82</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>83</v>

</xml_diff>

<commit_message>
Fusionner short/definition et signaler les valeurs additionnelles (U/L/M)
Déplace le texte sur la valeur par défaut N dans ^short plutôt que
^definition. Ajoute "..." après Normal/Restreint/Très restreint car
le ValueSet v3-ConfidentialityClassification porte 6 codes (U, L, M,
N, R, V), pas seulement les 3 codes NRV historiques. 1118db45e68cfd47ae1c22a66518fe53fc3667ec
</commit_message>
<xml_diff>
--- a/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4295" uniqueCount="776">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4295" uniqueCount="775">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-06T13:54:33+00:00</t>
+    <t>2026-08-06T13:55:54+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1278,10 +1278,7 @@
     <t>confidentiality</t>
   </si>
   <si>
-    <t>Niveau de confidentialité standard du document (Normal, Restreint, Très restreint).</t>
-  </si>
-  <si>
-    <t>En l'absence d'information de confidentialité disponible, la valeur par défaut à utiliser est N (Normal), conformément à ce qui est déjà pratiqué aujourd'hui pour les documents CDA.</t>
+    <t>Niveau de confidentialité standard du document (Normal, Restreint, Très restreint, ...). En l'absence d'information de confidentialité disponible, la valeur par défaut à utiliser est N (Normal), conformément à ce qui est déjà pratiqué aujourd'hui pour les documents CDA.</t>
   </si>
   <si>
     <t>http://terminology.hl7.org/ValueSet/v3-ConfidentialityClassification</t>
@@ -7858,7 +7855,7 @@
         <v>402</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>403</v>
+        <v>389</v>
       </c>
       <c r="N40" t="s" s="2">
         <v>390</v>
@@ -7893,7 +7890,7 @@
       </c>
       <c r="Y40" s="2"/>
       <c r="Z40" t="s" s="2">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="AA40" t="s" s="2">
         <v>82</v>
@@ -7955,13 +7952,13 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B41" t="s" s="2">
         <v>387</v>
       </c>
       <c r="C41" t="s" s="2">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D41" t="s" s="2">
         <v>82</v>
@@ -7986,7 +7983,7 @@
         <v>259</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="M41" t="s" s="2">
         <v>389</v>
@@ -8024,7 +8021,7 @@
       </c>
       <c r="Y41" s="2"/>
       <c r="Z41" t="s" s="2">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="AA41" t="s" s="2">
         <v>82</v>
@@ -8086,10 +8083,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -8115,10 +8112,10 @@
         <v>341</v>
       </c>
       <c r="L42" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="M42" t="s" s="2">
         <v>410</v>
-      </c>
-      <c r="M42" t="s" s="2">
-        <v>411</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -8169,7 +8166,7 @@
         <v>82</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>97</v>
@@ -8193,10 +8190,10 @@
         <v>82</v>
       </c>
       <c r="AN42" t="s" s="2">
+        <v>411</v>
+      </c>
+      <c r="AO42" t="s" s="2">
         <v>412</v>
-      </c>
-      <c r="AO42" t="s" s="2">
-        <v>413</v>
       </c>
       <c r="AP42" t="s" s="2">
         <v>82</v>
@@ -8213,10 +8210,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -8340,10 +8337,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -8469,10 +8466,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -8600,10 +8597,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -8626,13 +8623,13 @@
         <v>98</v>
       </c>
       <c r="K46" t="s" s="2">
+        <v>417</v>
+      </c>
+      <c r="L46" t="s" s="2">
         <v>418</v>
       </c>
-      <c r="L46" t="s" s="2">
+      <c r="M46" t="s" s="2">
         <v>419</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>420</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -8683,7 +8680,7 @@
         <v>82</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>97</v>
@@ -8707,30 +8704,30 @@
         <v>82</v>
       </c>
       <c r="AN46" t="s" s="2">
+        <v>420</v>
+      </c>
+      <c r="AO46" t="s" s="2">
+        <v>412</v>
+      </c>
+      <c r="AP46" t="s" s="2">
         <v>421</v>
       </c>
-      <c r="AO46" t="s" s="2">
-        <v>413</v>
-      </c>
-      <c r="AP46" t="s" s="2">
+      <c r="AQ46" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR46" t="s" s="2">
         <v>422</v>
       </c>
-      <c r="AQ46" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR46" t="s" s="2">
+      <c r="AS46" t="s" s="2">
         <v>423</v>
-      </c>
-      <c r="AS46" t="s" s="2">
-        <v>424</v>
       </c>
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -8854,10 +8851,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -8983,10 +8980,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -9012,14 +9009,14 @@
         <v>175</v>
       </c>
       <c r="L49" t="s" s="2">
+        <v>427</v>
+      </c>
+      <c r="M49" t="s" s="2">
         <v>428</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>429</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" t="s" s="2">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="P49" t="s" s="2">
         <v>82</v>
@@ -9032,7 +9029,7 @@
         <v>82</v>
       </c>
       <c r="T49" t="s" s="2">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="U49" t="s" s="2">
         <v>82</v>
@@ -9047,28 +9044,28 @@
         <v>242</v>
       </c>
       <c r="Y49" t="s" s="2">
+        <v>431</v>
+      </c>
+      <c r="Z49" t="s" s="2">
         <v>432</v>
       </c>
-      <c r="Z49" t="s" s="2">
+      <c r="AA49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF49" t="s" s="2">
         <v>433</v>
-      </c>
-      <c r="AA49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF49" t="s" s="2">
-        <v>434</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>83</v>
@@ -9086,25 +9083,25 @@
         <v>82</v>
       </c>
       <c r="AL49" t="s" s="2">
+        <v>434</v>
+      </c>
+      <c r="AM49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO49" t="s" s="2">
         <v>435</v>
       </c>
-      <c r="AM49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO49" t="s" s="2">
+      <c r="AP49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ49" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR49" t="s" s="2">
         <v>436</v>
-      </c>
-      <c r="AP49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ49" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR49" t="s" s="2">
-        <v>437</v>
       </c>
       <c r="AS49" t="s" s="2">
         <v>82</v>
@@ -9112,10 +9109,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -9141,14 +9138,14 @@
         <v>175</v>
       </c>
       <c r="L50" t="s" s="2">
+        <v>438</v>
+      </c>
+      <c r="M50" t="s" s="2">
         <v>439</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>440</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" t="s" s="2">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="P50" t="s" s="2">
         <v>82</v>
@@ -9161,7 +9158,7 @@
         <v>82</v>
       </c>
       <c r="T50" t="s" s="2">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="U50" t="s" s="2">
         <v>82</v>
@@ -9197,7 +9194,7 @@
         <v>82</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>83</v>
@@ -9212,19 +9209,19 @@
         <v>109</v>
       </c>
       <c r="AK50" t="s" s="2">
+        <v>443</v>
+      </c>
+      <c r="AL50" t="s" s="2">
         <v>444</v>
       </c>
-      <c r="AL50" t="s" s="2">
+      <c r="AM50" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN50" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO50" t="s" s="2">
         <v>445</v>
-      </c>
-      <c r="AM50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN50" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO50" t="s" s="2">
-        <v>446</v>
       </c>
       <c r="AP50" t="s" s="2">
         <v>82</v>
@@ -9241,10 +9238,10 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -9267,19 +9264,19 @@
         <v>82</v>
       </c>
       <c r="K51" t="s" s="2">
+        <v>447</v>
+      </c>
+      <c r="L51" t="s" s="2">
         <v>448</v>
       </c>
-      <c r="L51" t="s" s="2">
+      <c r="M51" t="s" s="2">
         <v>449</v>
       </c>
-      <c r="M51" t="s" s="2">
+      <c r="N51" t="s" s="2">
         <v>450</v>
       </c>
-      <c r="N51" t="s" s="2">
+      <c r="O51" t="s" s="2">
         <v>451</v>
-      </c>
-      <c r="O51" t="s" s="2">
-        <v>452</v>
       </c>
       <c r="P51" t="s" s="2">
         <v>82</v>
@@ -9328,7 +9325,7 @@
         <v>82</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>83</v>
@@ -9355,16 +9352,16 @@
         <v>82</v>
       </c>
       <c r="AO51" t="s" s="2">
+        <v>453</v>
+      </c>
+      <c r="AP51" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ51" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR51" t="s" s="2">
         <v>454</v>
-      </c>
-      <c r="AP51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ51" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR51" t="s" s="2">
-        <v>455</v>
       </c>
       <c r="AS51" t="s" s="2">
         <v>82</v>
@@ -9372,10 +9369,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -9398,19 +9395,19 @@
         <v>98</v>
       </c>
       <c r="K52" t="s" s="2">
+        <v>456</v>
+      </c>
+      <c r="L52" t="s" s="2">
         <v>457</v>
       </c>
-      <c r="L52" t="s" s="2">
+      <c r="M52" t="s" s="2">
         <v>458</v>
       </c>
-      <c r="M52" t="s" s="2">
+      <c r="N52" t="s" s="2">
         <v>459</v>
       </c>
-      <c r="N52" t="s" s="2">
+      <c r="O52" t="s" s="2">
         <v>460</v>
-      </c>
-      <c r="O52" t="s" s="2">
-        <v>461</v>
       </c>
       <c r="P52" t="s" s="2">
         <v>82</v>
@@ -9423,79 +9420,79 @@
         <v>82</v>
       </c>
       <c r="T52" t="s" s="2">
+        <v>461</v>
+      </c>
+      <c r="U52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF52" t="s" s="2">
         <v>462</v>
       </c>
-      <c r="U52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF52" t="s" s="2">
+      <c r="AG52" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH52" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ52" t="s" s="2">
         <v>463</v>
       </c>
-      <c r="AG52" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH52" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ52" t="s" s="2">
+      <c r="AK52" t="s" s="2">
         <v>464</v>
       </c>
-      <c r="AK52" t="s" s="2">
+      <c r="AL52" t="s" s="2">
         <v>465</v>
       </c>
-      <c r="AL52" t="s" s="2">
+      <c r="AM52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO52" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="AM52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO52" t="s" s="2">
+      <c r="AP52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ52" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR52" t="s" s="2">
         <v>467</v>
-      </c>
-      <c r="AP52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ52" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR52" t="s" s="2">
-        <v>468</v>
       </c>
       <c r="AS52" t="s" s="2">
         <v>82</v>
@@ -9503,10 +9500,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -9529,19 +9526,19 @@
         <v>98</v>
       </c>
       <c r="K53" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="L53" t="s" s="2">
         <v>470</v>
       </c>
-      <c r="L53" t="s" s="2">
+      <c r="M53" t="s" s="2">
         <v>471</v>
       </c>
-      <c r="M53" t="s" s="2">
+      <c r="N53" t="s" s="2">
         <v>472</v>
       </c>
-      <c r="N53" t="s" s="2">
+      <c r="O53" t="s" s="2">
         <v>473</v>
-      </c>
-      <c r="O53" t="s" s="2">
-        <v>474</v>
       </c>
       <c r="P53" t="s" s="2">
         <v>82</v>
@@ -9590,7 +9587,7 @@
         <v>82</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>83</v>
@@ -9608,16 +9605,16 @@
         <v>82</v>
       </c>
       <c r="AL53" t="s" s="2">
+        <v>475</v>
+      </c>
+      <c r="AM53" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN53" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO53" t="s" s="2">
         <v>476</v>
-      </c>
-      <c r="AM53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN53" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO53" t="s" s="2">
-        <v>477</v>
       </c>
       <c r="AP53" t="s" s="2">
         <v>82</v>
@@ -9634,10 +9631,10 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -9660,19 +9657,19 @@
         <v>98</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="L54" t="s" s="2">
+        <v>478</v>
+      </c>
+      <c r="M54" t="s" s="2">
         <v>479</v>
       </c>
-      <c r="M54" t="s" s="2">
+      <c r="N54" t="s" s="2">
         <v>480</v>
       </c>
-      <c r="N54" t="s" s="2">
+      <c r="O54" t="s" s="2">
         <v>481</v>
-      </c>
-      <c r="O54" t="s" s="2">
-        <v>482</v>
       </c>
       <c r="P54" t="s" s="2">
         <v>82</v>
@@ -9721,7 +9718,7 @@
         <v>82</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>83</v>
@@ -9739,16 +9736,16 @@
         <v>82</v>
       </c>
       <c r="AL54" t="s" s="2">
+        <v>483</v>
+      </c>
+      <c r="AM54" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN54" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO54" t="s" s="2">
         <v>484</v>
-      </c>
-      <c r="AM54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN54" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO54" t="s" s="2">
-        <v>485</v>
       </c>
       <c r="AP54" t="s" s="2">
         <v>82</v>
@@ -9765,10 +9762,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -9794,14 +9791,14 @@
         <v>111</v>
       </c>
       <c r="L55" t="s" s="2">
+        <v>486</v>
+      </c>
+      <c r="M55" t="s" s="2">
         <v>487</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>488</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" t="s" s="2">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="P55" t="s" s="2">
         <v>82</v>
@@ -9814,43 +9811,43 @@
         <v>82</v>
       </c>
       <c r="T55" t="s" s="2">
+        <v>489</v>
+      </c>
+      <c r="U55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF55" t="s" s="2">
         <v>490</v>
-      </c>
-      <c r="U55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF55" t="s" s="2">
-        <v>491</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>83</v>
@@ -9865,19 +9862,19 @@
         <v>109</v>
       </c>
       <c r="AK55" t="s" s="2">
+        <v>491</v>
+      </c>
+      <c r="AL55" t="s" s="2">
         <v>492</v>
       </c>
-      <c r="AL55" t="s" s="2">
+      <c r="AM55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN55" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO55" t="s" s="2">
         <v>493</v>
-      </c>
-      <c r="AM55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN55" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO55" t="s" s="2">
-        <v>494</v>
       </c>
       <c r="AP55" t="s" s="2">
         <v>82</v>
@@ -9894,10 +9891,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -9920,17 +9917,17 @@
         <v>98</v>
       </c>
       <c r="K56" t="s" s="2">
+        <v>495</v>
+      </c>
+      <c r="L56" t="s" s="2">
         <v>496</v>
       </c>
-      <c r="L56" t="s" s="2">
+      <c r="M56" t="s" s="2">
         <v>497</v>
-      </c>
-      <c r="M56" t="s" s="2">
-        <v>498</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" t="s" s="2">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="P56" t="s" s="2">
         <v>82</v>
@@ -9979,7 +9976,7 @@
         <v>82</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>83</v>
@@ -9994,11 +9991,11 @@
         <v>109</v>
       </c>
       <c r="AK56" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="AL56" t="s" s="2">
         <v>501</v>
       </c>
-      <c r="AL56" t="s" s="2">
-        <v>502</v>
-      </c>
       <c r="AM56" t="s" s="2">
         <v>82</v>
       </c>
@@ -10006,7 +10003,7 @@
         <v>82</v>
       </c>
       <c r="AO56" t="s" s="2">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="AP56" t="s" s="2">
         <v>82</v>
@@ -10023,10 +10020,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -10052,13 +10049,13 @@
         <v>153</v>
       </c>
       <c r="L57" t="s" s="2">
+        <v>503</v>
+      </c>
+      <c r="M57" t="s" s="2">
         <v>504</v>
       </c>
-      <c r="M57" t="s" s="2">
+      <c r="N57" t="s" s="2">
         <v>505</v>
-      </c>
-      <c r="N57" t="s" s="2">
-        <v>506</v>
       </c>
       <c r="O57" s="2"/>
       <c r="P57" t="s" s="2">
@@ -10088,56 +10085,56 @@
       </c>
       <c r="Y57" s="2"/>
       <c r="Z57" t="s" s="2">
+        <v>506</v>
+      </c>
+      <c r="AA57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF57" t="s" s="2">
+        <v>502</v>
+      </c>
+      <c r="AG57" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH57" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ57" t="s" s="2">
         <v>507</v>
       </c>
-      <c r="AA57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF57" t="s" s="2">
-        <v>503</v>
-      </c>
-      <c r="AG57" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH57" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ57" t="s" s="2">
+      <c r="AK57" t="s" s="2">
         <v>508</v>
       </c>
-      <c r="AK57" t="s" s="2">
+      <c r="AL57" t="s" s="2">
         <v>509</v>
       </c>
-      <c r="AL57" t="s" s="2">
+      <c r="AM57" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN57" t="s" s="2">
         <v>510</v>
       </c>
-      <c r="AM57" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN57" t="s" s="2">
+      <c r="AO57" t="s" s="2">
+        <v>412</v>
+      </c>
+      <c r="AP57" t="s" s="2">
         <v>511</v>
       </c>
-      <c r="AO57" t="s" s="2">
-        <v>413</v>
-      </c>
-      <c r="AP57" t="s" s="2">
-        <v>512</v>
-      </c>
       <c r="AQ57" t="s" s="2">
         <v>82</v>
       </c>
@@ -10145,15 +10142,15 @@
         <v>82</v>
       </c>
       <c r="AS57" t="s" s="2">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -10179,13 +10176,13 @@
         <v>341</v>
       </c>
       <c r="L58" t="s" s="2">
+        <v>513</v>
+      </c>
+      <c r="M58" t="s" s="2">
         <v>514</v>
       </c>
-      <c r="M58" t="s" s="2">
+      <c r="N58" t="s" s="2">
         <v>515</v>
-      </c>
-      <c r="N58" t="s" s="2">
-        <v>516</v>
       </c>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
@@ -10235,7 +10232,7 @@
         <v>82</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>83</v>
@@ -10262,7 +10259,7 @@
         <v>82</v>
       </c>
       <c r="AO58" t="s" s="2">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="AP58" t="s" s="2">
         <v>82</v>
@@ -10279,10 +10276,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -10406,10 +10403,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -10535,10 +10532,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -10666,10 +10663,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -10692,13 +10689,13 @@
         <v>82</v>
       </c>
       <c r="K62" t="s" s="2">
+        <v>521</v>
+      </c>
+      <c r="L62" t="s" s="2">
         <v>522</v>
       </c>
-      <c r="L62" t="s" s="2">
+      <c r="M62" t="s" s="2">
         <v>523</v>
-      </c>
-      <c r="M62" t="s" s="2">
-        <v>524</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -10749,7 +10746,7 @@
         <v>82</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>83</v>
@@ -10767,22 +10764,22 @@
         <v>82</v>
       </c>
       <c r="AL62" t="s" s="2">
+        <v>524</v>
+      </c>
+      <c r="AM62" t="s" s="2">
         <v>525</v>
       </c>
-      <c r="AM62" t="s" s="2">
+      <c r="AN62" t="s" s="2">
         <v>526</v>
       </c>
-      <c r="AN62" t="s" s="2">
+      <c r="AO62" t="s" s="2">
         <v>527</v>
       </c>
-      <c r="AO62" t="s" s="2">
+      <c r="AP62" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ62" t="s" s="2">
         <v>528</v>
-      </c>
-      <c r="AP62" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ62" t="s" s="2">
-        <v>529</v>
       </c>
       <c r="AR62" t="s" s="2">
         <v>82</v>
@@ -10793,10 +10790,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -10822,13 +10819,13 @@
         <v>259</v>
       </c>
       <c r="L63" t="s" s="2">
+        <v>530</v>
+      </c>
+      <c r="M63" t="s" s="2">
         <v>531</v>
       </c>
-      <c r="M63" t="s" s="2">
+      <c r="N63" t="s" s="2">
         <v>532</v>
-      </c>
-      <c r="N63" t="s" s="2">
-        <v>533</v>
       </c>
       <c r="O63" s="2"/>
       <c r="P63" t="s" s="2">
@@ -10857,11 +10854,11 @@
         <v>165</v>
       </c>
       <c r="Y63" t="s" s="2">
+        <v>533</v>
+      </c>
+      <c r="Z63" t="s" s="2">
         <v>534</v>
       </c>
-      <c r="Z63" t="s" s="2">
-        <v>535</v>
-      </c>
       <c r="AA63" t="s" s="2">
         <v>82</v>
       </c>
@@ -10878,7 +10875,7 @@
         <v>82</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>83</v>
@@ -10890,23 +10887,23 @@
         <v>82</v>
       </c>
       <c r="AJ63" t="s" s="2">
+        <v>535</v>
+      </c>
+      <c r="AK63" t="s" s="2">
         <v>536</v>
       </c>
-      <c r="AK63" t="s" s="2">
+      <c r="AL63" t="s" s="2">
         <v>537</v>
       </c>
-      <c r="AL63" t="s" s="2">
+      <c r="AM63" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN63" t="s" s="2">
         <v>538</v>
       </c>
-      <c r="AM63" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN63" t="s" s="2">
+      <c r="AO63" t="s" s="2">
         <v>539</v>
       </c>
-      <c r="AO63" t="s" s="2">
-        <v>540</v>
-      </c>
       <c r="AP63" t="s" s="2">
         <v>82</v>
       </c>
@@ -10917,15 +10914,15 @@
         <v>82</v>
       </c>
       <c r="AS63" t="s" s="2">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -10948,13 +10945,13 @@
         <v>98</v>
       </c>
       <c r="K64" t="s" s="2">
+        <v>541</v>
+      </c>
+      <c r="L64" t="s" s="2">
         <v>542</v>
       </c>
-      <c r="L64" t="s" s="2">
+      <c r="M64" t="s" s="2">
         <v>543</v>
-      </c>
-      <c r="M64" t="s" s="2">
-        <v>544</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
@@ -11005,7 +11002,7 @@
         <v>82</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>83</v>
@@ -11029,30 +11026,30 @@
         <v>82</v>
       </c>
       <c r="AN64" t="s" s="2">
+        <v>544</v>
+      </c>
+      <c r="AO64" t="s" s="2">
         <v>545</v>
       </c>
-      <c r="AO64" t="s" s="2">
+      <c r="AP64" t="s" s="2">
         <v>546</v>
       </c>
-      <c r="AP64" t="s" s="2">
+      <c r="AQ64" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR64" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AS64" t="s" s="2">
         <v>547</v>
-      </c>
-      <c r="AQ64" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR64" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AS64" t="s" s="2">
-        <v>548</v>
       </c>
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -11176,10 +11173,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -11305,10 +11302,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -11331,16 +11328,16 @@
         <v>98</v>
       </c>
       <c r="K67" t="s" s="2">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="L67" t="s" s="2">
+        <v>551</v>
+      </c>
+      <c r="M67" t="s" s="2">
         <v>552</v>
       </c>
-      <c r="M67" t="s" s="2">
+      <c r="N67" t="s" s="2">
         <v>553</v>
-      </c>
-      <c r="N67" t="s" s="2">
-        <v>554</v>
       </c>
       <c r="O67" s="2"/>
       <c r="P67" t="s" s="2">
@@ -11390,43 +11387,43 @@
         <v>82</v>
       </c>
       <c r="AF67" t="s" s="2">
+        <v>554</v>
+      </c>
+      <c r="AG67" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH67" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI67" t="s" s="2">
         <v>555</v>
-      </c>
-      <c r="AG67" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH67" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI67" t="s" s="2">
-        <v>556</v>
       </c>
       <c r="AJ67" t="s" s="2">
         <v>109</v>
       </c>
       <c r="AK67" t="s" s="2">
+        <v>556</v>
+      </c>
+      <c r="AL67" t="s" s="2">
         <v>557</v>
       </c>
-      <c r="AL67" t="s" s="2">
+      <c r="AM67" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN67" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO67" t="s" s="2">
         <v>558</v>
       </c>
-      <c r="AM67" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN67" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO67" t="s" s="2">
+      <c r="AP67" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ67" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR67" t="s" s="2">
         <v>559</v>
-      </c>
-      <c r="AP67" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ67" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR67" t="s" s="2">
-        <v>560</v>
       </c>
       <c r="AS67" t="s" s="2">
         <v>82</v>
@@ -11434,10 +11431,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -11460,69 +11457,69 @@
         <v>98</v>
       </c>
       <c r="K68" t="s" s="2">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="L68" t="s" s="2">
+        <v>561</v>
+      </c>
+      <c r="M68" t="s" s="2">
         <v>562</v>
       </c>
-      <c r="M68" t="s" s="2">
+      <c r="N68" t="s" s="2">
         <v>563</v>
-      </c>
-      <c r="N68" t="s" s="2">
-        <v>564</v>
       </c>
       <c r="O68" s="2"/>
       <c r="P68" t="s" s="2">
         <v>82</v>
       </c>
       <c r="Q68" t="s" s="2">
+        <v>564</v>
+      </c>
+      <c r="R68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="S68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="T68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF68" t="s" s="2">
         <v>565</v>
       </c>
-      <c r="R68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF68" t="s" s="2">
-        <v>566</v>
-      </c>
       <c r="AG68" t="s" s="2">
         <v>83</v>
       </c>
@@ -11530,34 +11527,34 @@
         <v>97</v>
       </c>
       <c r="AI68" t="s" s="2">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="AJ68" t="s" s="2">
         <v>109</v>
       </c>
       <c r="AK68" t="s" s="2">
+        <v>566</v>
+      </c>
+      <c r="AL68" t="s" s="2">
         <v>567</v>
       </c>
-      <c r="AL68" t="s" s="2">
+      <c r="AM68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO68" t="s" s="2">
         <v>568</v>
       </c>
-      <c r="AM68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO68" t="s" s="2">
+      <c r="AP68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ68" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR68" t="s" s="2">
         <v>569</v>
-      </c>
-      <c r="AP68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ68" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR68" t="s" s="2">
-        <v>570</v>
       </c>
       <c r="AS68" t="s" s="2">
         <v>82</v>
@@ -11565,10 +11562,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -11594,10 +11591,10 @@
         <v>259</v>
       </c>
       <c r="L69" t="s" s="2">
+        <v>571</v>
+      </c>
+      <c r="M69" t="s" s="2">
         <v>572</v>
-      </c>
-      <c r="M69" t="s" s="2">
-        <v>573</v>
       </c>
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
@@ -11628,56 +11625,56 @@
       </c>
       <c r="Y69" s="2"/>
       <c r="Z69" t="s" s="2">
+        <v>573</v>
+      </c>
+      <c r="AA69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF69" t="s" s="2">
+        <v>570</v>
+      </c>
+      <c r="AG69" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH69" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ69" t="s" s="2">
         <v>574</v>
       </c>
-      <c r="AA69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF69" t="s" s="2">
-        <v>571</v>
-      </c>
-      <c r="AG69" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH69" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ69" t="s" s="2">
+      <c r="AK69" t="s" s="2">
         <v>575</v>
       </c>
-      <c r="AK69" t="s" s="2">
+      <c r="AL69" t="s" s="2">
         <v>576</v>
       </c>
-      <c r="AL69" t="s" s="2">
+      <c r="AM69" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN69" t="s" s="2">
         <v>577</v>
       </c>
-      <c r="AM69" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN69" t="s" s="2">
+      <c r="AO69" t="s" s="2">
         <v>578</v>
       </c>
-      <c r="AO69" t="s" s="2">
+      <c r="AP69" t="s" s="2">
         <v>579</v>
       </c>
-      <c r="AP69" t="s" s="2">
-        <v>580</v>
-      </c>
       <c r="AQ69" t="s" s="2">
         <v>82</v>
       </c>
@@ -11685,15 +11682,15 @@
         <v>82</v>
       </c>
       <c r="AS69" t="s" s="2">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -11719,16 +11716,16 @@
         <v>259</v>
       </c>
       <c r="L70" t="s" s="2">
+        <v>581</v>
+      </c>
+      <c r="M70" t="s" s="2">
         <v>582</v>
       </c>
-      <c r="M70" t="s" s="2">
+      <c r="N70" t="s" s="2">
         <v>583</v>
       </c>
-      <c r="N70" t="s" s="2">
+      <c r="O70" t="s" s="2">
         <v>584</v>
-      </c>
-      <c r="O70" t="s" s="2">
-        <v>585</v>
       </c>
       <c r="P70" t="s" s="2">
         <v>82</v>
@@ -11757,55 +11754,55 @@
       </c>
       <c r="Y70" s="2"/>
       <c r="Z70" t="s" s="2">
+        <v>585</v>
+      </c>
+      <c r="AA70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF70" t="s" s="2">
+        <v>580</v>
+      </c>
+      <c r="AG70" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH70" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI70" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AJ70" t="s" s="2">
+        <v>574</v>
+      </c>
+      <c r="AK70" t="s" s="2">
         <v>586</v>
       </c>
-      <c r="AA70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF70" t="s" s="2">
-        <v>581</v>
-      </c>
-      <c r="AG70" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH70" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI70" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ70" t="s" s="2">
-        <v>575</v>
-      </c>
-      <c r="AK70" t="s" s="2">
+      <c r="AL70" t="s" s="2">
         <v>587</v>
       </c>
-      <c r="AL70" t="s" s="2">
-        <v>588</v>
-      </c>
       <c r="AM70" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AN70" t="s" s="2">
+        <v>577</v>
+      </c>
+      <c r="AO70" t="s" s="2">
         <v>578</v>
       </c>
-      <c r="AO70" t="s" s="2">
-        <v>579</v>
-      </c>
       <c r="AP70" t="s" s="2">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="AQ70" t="s" s="2">
         <v>82</v>
@@ -11814,15 +11811,15 @@
         <v>82</v>
       </c>
       <c r="AS70" t="s" s="2">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -11845,13 +11842,13 @@
         <v>82</v>
       </c>
       <c r="K71" t="s" s="2">
+        <v>589</v>
+      </c>
+      <c r="L71" t="s" s="2">
         <v>590</v>
       </c>
-      <c r="L71" t="s" s="2">
+      <c r="M71" t="s" s="2">
         <v>591</v>
-      </c>
-      <c r="M71" t="s" s="2">
-        <v>592</v>
       </c>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
@@ -11902,7 +11899,7 @@
         <v>82</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>83</v>
@@ -11941,15 +11938,15 @@
         <v>82</v>
       </c>
       <c r="AS71" t="s" s="2">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -12073,10 +12070,10 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -12202,10 +12199,10 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -12231,13 +12228,13 @@
         <v>111</v>
       </c>
       <c r="L74" t="s" s="2">
+        <v>596</v>
+      </c>
+      <c r="M74" t="s" s="2">
         <v>597</v>
       </c>
-      <c r="M74" t="s" s="2">
+      <c r="N74" t="s" s="2">
         <v>598</v>
-      </c>
-      <c r="N74" t="s" s="2">
-        <v>599</v>
       </c>
       <c r="O74" s="2"/>
       <c r="P74" t="s" s="2">
@@ -12287,16 +12284,16 @@
         <v>82</v>
       </c>
       <c r="AF74" t="s" s="2">
+        <v>599</v>
+      </c>
+      <c r="AG74" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH74" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI74" t="s" s="2">
         <v>600</v>
-      </c>
-      <c r="AG74" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH74" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI74" t="s" s="2">
-        <v>601</v>
       </c>
       <c r="AJ74" t="s" s="2">
         <v>109</v>
@@ -12305,7 +12302,7 @@
         <v>82</v>
       </c>
       <c r="AL74" t="s" s="2">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="AM74" t="s" s="2">
         <v>82</v>
@@ -12331,10 +12328,10 @@
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -12360,13 +12357,13 @@
         <v>140</v>
       </c>
       <c r="L75" t="s" s="2">
+        <v>603</v>
+      </c>
+      <c r="M75" t="s" s="2">
         <v>604</v>
       </c>
-      <c r="M75" t="s" s="2">
+      <c r="N75" t="s" s="2">
         <v>605</v>
-      </c>
-      <c r="N75" t="s" s="2">
-        <v>606</v>
       </c>
       <c r="O75" s="2"/>
       <c r="P75" t="s" s="2">
@@ -12395,28 +12392,28 @@
         <v>157</v>
       </c>
       <c r="Y75" t="s" s="2">
+        <v>606</v>
+      </c>
+      <c r="Z75" t="s" s="2">
         <v>607</v>
       </c>
-      <c r="Z75" t="s" s="2">
+      <c r="AA75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE75" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF75" t="s" s="2">
         <v>608</v>
-      </c>
-      <c r="AA75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE75" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF75" t="s" s="2">
-        <v>609</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>83</v>
@@ -12460,10 +12457,10 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -12489,13 +12486,13 @@
         <v>227</v>
       </c>
       <c r="L76" t="s" s="2">
+        <v>610</v>
+      </c>
+      <c r="M76" t="s" s="2">
         <v>611</v>
       </c>
-      <c r="M76" t="s" s="2">
+      <c r="N76" t="s" s="2">
         <v>612</v>
-      </c>
-      <c r="N76" t="s" s="2">
-        <v>613</v>
       </c>
       <c r="O76" s="2"/>
       <c r="P76" t="s" s="2">
@@ -12545,7 +12542,7 @@
         <v>82</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>83</v>
@@ -12563,16 +12560,16 @@
         <v>82</v>
       </c>
       <c r="AL76" t="s" s="2">
+        <v>614</v>
+      </c>
+      <c r="AM76" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN76" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AO76" t="s" s="2">
         <v>615</v>
-      </c>
-      <c r="AM76" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN76" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO76" t="s" s="2">
-        <v>616</v>
       </c>
       <c r="AP76" t="s" s="2">
         <v>82</v>
@@ -12589,10 +12586,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -12618,13 +12615,13 @@
         <v>111</v>
       </c>
       <c r="L77" t="s" s="2">
+        <v>617</v>
+      </c>
+      <c r="M77" t="s" s="2">
         <v>618</v>
       </c>
-      <c r="M77" t="s" s="2">
+      <c r="N77" t="s" s="2">
         <v>619</v>
-      </c>
-      <c r="N77" t="s" s="2">
-        <v>620</v>
       </c>
       <c r="O77" s="2"/>
       <c r="P77" t="s" s="2">
@@ -12674,7 +12671,7 @@
         <v>82</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>83</v>
@@ -12718,10 +12715,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -12744,16 +12741,16 @@
         <v>82</v>
       </c>
       <c r="K78" t="s" s="2">
+        <v>622</v>
+      </c>
+      <c r="L78" t="s" s="2">
         <v>623</v>
       </c>
-      <c r="L78" t="s" s="2">
+      <c r="M78" t="s" s="2">
         <v>624</v>
       </c>
-      <c r="M78" t="s" s="2">
+      <c r="N78" t="s" s="2">
         <v>625</v>
-      </c>
-      <c r="N78" t="s" s="2">
-        <v>626</v>
       </c>
       <c r="O78" s="2"/>
       <c r="P78" t="s" s="2">
@@ -12791,10 +12788,10 @@
         <v>82</v>
       </c>
       <c r="AB78" t="s" s="2">
+        <v>626</v>
+      </c>
+      <c r="AC78" t="s" s="2">
         <v>627</v>
-      </c>
-      <c r="AC78" t="s" s="2">
-        <v>628</v>
       </c>
       <c r="AD78" t="s" s="2">
         <v>82</v>
@@ -12803,7 +12800,7 @@
         <v>124</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>83</v>
@@ -12821,39 +12818,39 @@
         <v>82</v>
       </c>
       <c r="AL78" t="s" s="2">
+        <v>628</v>
+      </c>
+      <c r="AM78" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN78" t="s" s="2">
         <v>629</v>
       </c>
-      <c r="AM78" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN78" t="s" s="2">
+      <c r="AO78" t="s" s="2">
         <v>630</v>
       </c>
-      <c r="AO78" t="s" s="2">
+      <c r="AP78" t="s" s="2">
         <v>631</v>
       </c>
-      <c r="AP78" t="s" s="2">
+      <c r="AQ78" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR78" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AS78" t="s" s="2">
         <v>632</v>
-      </c>
-      <c r="AQ78" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR78" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AS78" t="s" s="2">
-        <v>633</v>
       </c>
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
+        <v>633</v>
+      </c>
+      <c r="B79" t="s" s="2">
+        <v>621</v>
+      </c>
+      <c r="C79" t="s" s="2">
         <v>634</v>
-      </c>
-      <c r="B79" t="s" s="2">
-        <v>622</v>
-      </c>
-      <c r="C79" t="s" s="2">
-        <v>635</v>
       </c>
       <c r="D79" t="s" s="2">
         <v>82</v>
@@ -12875,16 +12872,16 @@
         <v>82</v>
       </c>
       <c r="K79" t="s" s="2">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="M79" t="s" s="2">
+        <v>624</v>
+      </c>
+      <c r="N79" t="s" s="2">
         <v>625</v>
-      </c>
-      <c r="N79" t="s" s="2">
-        <v>626</v>
       </c>
       <c r="O79" s="2"/>
       <c r="P79" t="s" s="2">
@@ -12934,7 +12931,7 @@
         <v>82</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>83</v>
@@ -12952,36 +12949,36 @@
         <v>82</v>
       </c>
       <c r="AL79" t="s" s="2">
+        <v>628</v>
+      </c>
+      <c r="AM79" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AN79" t="s" s="2">
         <v>629</v>
       </c>
-      <c r="AM79" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN79" t="s" s="2">
+      <c r="AO79" t="s" s="2">
         <v>630</v>
       </c>
-      <c r="AO79" t="s" s="2">
+      <c r="AP79" t="s" s="2">
         <v>631</v>
       </c>
-      <c r="AP79" t="s" s="2">
+      <c r="AQ79" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR79" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AS79" t="s" s="2">
         <v>632</v>
-      </c>
-      <c r="AQ79" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR79" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AS79" t="s" s="2">
-        <v>633</v>
       </c>
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
+        <v>636</v>
+      </c>
+      <c r="B80" t="s" s="2">
         <v>637</v>
-      </c>
-      <c r="B80" t="s" s="2">
-        <v>638</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -13105,10 +13102,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
+        <v>638</v>
+      </c>
+      <c r="B81" t="s" s="2">
         <v>639</v>
-      </c>
-      <c r="B81" t="s" s="2">
-        <v>640</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -13234,10 +13231,10 @@
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
+        <v>640</v>
+      </c>
+      <c r="B82" t="s" s="2">
         <v>641</v>
-      </c>
-      <c r="B82" t="s" s="2">
-        <v>642</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -13263,13 +13260,13 @@
         <v>111</v>
       </c>
       <c r="L82" t="s" s="2">
+        <v>596</v>
+      </c>
+      <c r="M82" t="s" s="2">
         <v>597</v>
       </c>
-      <c r="M82" t="s" s="2">
+      <c r="N82" t="s" s="2">
         <v>598</v>
-      </c>
-      <c r="N82" t="s" s="2">
-        <v>599</v>
       </c>
       <c r="O82" s="2"/>
       <c r="P82" t="s" s="2">
@@ -13319,16 +13316,16 @@
         <v>82</v>
       </c>
       <c r="AF82" t="s" s="2">
+        <v>599</v>
+      </c>
+      <c r="AG82" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH82" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AI82" t="s" s="2">
         <v>600</v>
-      </c>
-      <c r="AG82" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AH82" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AI82" t="s" s="2">
-        <v>601</v>
       </c>
       <c r="AJ82" t="s" s="2">
         <v>109</v>
@@ -13363,10 +13360,10 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
+        <v>642</v>
+      </c>
+      <c r="B83" t="s" s="2">
         <v>643</v>
-      </c>
-      <c r="B83" t="s" s="2">
-        <v>644</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -13392,13 +13389,13 @@
         <v>140</v>
       </c>
       <c r="L83" t="s" s="2">
+        <v>603</v>
+      </c>
+      <c r="M83" t="s" s="2">
         <v>604</v>
       </c>
-      <c r="M83" t="s" s="2">
+      <c r="N83" t="s" s="2">
         <v>605</v>
-      </c>
-      <c r="N83" t="s" s="2">
-        <v>606</v>
       </c>
       <c r="O83" s="2"/>
       <c r="P83" t="s" s="2">
@@ -13427,28 +13424,28 @@
         <v>157</v>
       </c>
       <c r="Y83" t="s" s="2">
+        <v>606</v>
+      </c>
+      <c r="Z83" t="s" s="2">
         <v>607</v>
       </c>
-      <c r="Z83" t="s" s="2">
+      <c r="AA83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE83" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF83" t="s" s="2">
         <v>608</v>
-      </c>
-      <c r="AA83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE83" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF83" t="s" s="2">
-        <v>609</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>83</v>
@@ -13492,10 +13489,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
+        <v>644</v>
+      </c>
+      <c r="B84" t="s" s="2">
         <v>645</v>
-      </c>
-      <c r="B84" t="s" s="2">
-        <v>646</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -13521,13 +13518,13 @@
         <v>227</v>
       </c>
       <c r="L84" t="s" s="2">
+        <v>610</v>
+      </c>
+      <c r="M84" t="s" s="2">
         <v>611</v>
       </c>
-      <c r="M84" t="s" s="2">
+      <c r="N84" t="s" s="2">
         <v>612</v>
-      </c>
-      <c r="N84" t="s" s="2">
-        <v>613</v>
       </c>
       <c r="O84" s="2"/>
       <c r="P84" t="s" s="2">
@@ -13577,7 +13574,7 @@
         <v>82</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>83</v>
@@ -13604,7 +13601,7 @@
         <v>82</v>
       </c>
       <c r="AO84" t="s" s="2">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="AP84" t="s" s="2">
         <v>82</v>
@@ -13621,10 +13618,10 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
+        <v>646</v>
+      </c>
+      <c r="B85" t="s" s="2">
         <v>647</v>
-      </c>
-      <c r="B85" t="s" s="2">
-        <v>648</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -13748,10 +13745,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
+        <v>648</v>
+      </c>
+      <c r="B86" t="s" s="2">
         <v>649</v>
-      </c>
-      <c r="B86" t="s" s="2">
-        <v>650</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -13877,10 +13874,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
+        <v>650</v>
+      </c>
+      <c r="B87" t="s" s="2">
         <v>651</v>
-      </c>
-      <c r="B87" t="s" s="2">
-        <v>652</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -13906,16 +13903,16 @@
         <v>175</v>
       </c>
       <c r="L87" t="s" s="2">
+        <v>652</v>
+      </c>
+      <c r="M87" t="s" s="2">
         <v>653</v>
       </c>
-      <c r="M87" t="s" s="2">
+      <c r="N87" t="s" s="2">
         <v>654</v>
       </c>
-      <c r="N87" t="s" s="2">
+      <c r="O87" t="s" s="2">
         <v>655</v>
-      </c>
-      <c r="O87" t="s" s="2">
-        <v>656</v>
       </c>
       <c r="P87" t="s" s="2">
         <v>82</v>
@@ -13943,28 +13940,28 @@
         <v>242</v>
       </c>
       <c r="Y87" t="s" s="2">
+        <v>656</v>
+      </c>
+      <c r="Z87" t="s" s="2">
         <v>657</v>
       </c>
-      <c r="Z87" t="s" s="2">
+      <c r="AA87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE87" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF87" t="s" s="2">
         <v>658</v>
-      </c>
-      <c r="AA87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE87" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF87" t="s" s="2">
-        <v>659</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>83</v>
@@ -13991,7 +13988,7 @@
         <v>82</v>
       </c>
       <c r="AO87" t="s" s="2">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="AP87" t="s" s="2">
         <v>82</v>
@@ -14008,10 +14005,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
+        <v>660</v>
+      </c>
+      <c r="B88" t="s" s="2">
         <v>661</v>
-      </c>
-      <c r="B88" t="s" s="2">
-        <v>662</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -14037,16 +14034,16 @@
         <v>259</v>
       </c>
       <c r="L88" t="s" s="2">
+        <v>662</v>
+      </c>
+      <c r="M88" t="s" s="2">
         <v>663</v>
       </c>
-      <c r="M88" t="s" s="2">
+      <c r="N88" t="s" s="2">
         <v>664</v>
       </c>
-      <c r="N88" t="s" s="2">
+      <c r="O88" t="s" s="2">
         <v>665</v>
-      </c>
-      <c r="O88" t="s" s="2">
-        <v>666</v>
       </c>
       <c r="P88" t="s" s="2">
         <v>82</v>
@@ -14074,28 +14071,28 @@
         <v>157</v>
       </c>
       <c r="Y88" t="s" s="2">
+        <v>666</v>
+      </c>
+      <c r="Z88" t="s" s="2">
         <v>667</v>
       </c>
-      <c r="Z88" t="s" s="2">
+      <c r="AA88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE88" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF88" t="s" s="2">
         <v>668</v>
-      </c>
-      <c r="AA88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF88" t="s" s="2">
-        <v>669</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>83</v>
@@ -14122,7 +14119,7 @@
         <v>82</v>
       </c>
       <c r="AO88" t="s" s="2">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="AP88" t="s" s="2">
         <v>82</v>
@@ -14131,7 +14128,7 @@
         <v>82</v>
       </c>
       <c r="AR88" t="s" s="2">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="AS88" t="s" s="2">
         <v>82</v>
@@ -14139,10 +14136,10 @@
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
+        <v>670</v>
+      </c>
+      <c r="B89" t="s" s="2">
         <v>671</v>
-      </c>
-      <c r="B89" t="s" s="2">
-        <v>672</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -14266,10 +14263,10 @@
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
+        <v>672</v>
+      </c>
+      <c r="B90" t="s" s="2">
         <v>673</v>
-      </c>
-      <c r="B90" t="s" s="2">
-        <v>674</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -14395,10 +14392,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
+        <v>674</v>
+      </c>
+      <c r="B91" t="s" s="2">
         <v>675</v>
-      </c>
-      <c r="B91" t="s" s="2">
-        <v>676</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -14424,16 +14421,16 @@
         <v>153</v>
       </c>
       <c r="L91" t="s" s="2">
+        <v>676</v>
+      </c>
+      <c r="M91" t="s" s="2">
         <v>677</v>
       </c>
-      <c r="M91" t="s" s="2">
+      <c r="N91" t="s" s="2">
         <v>678</v>
       </c>
-      <c r="N91" t="s" s="2">
+      <c r="O91" t="s" s="2">
         <v>679</v>
-      </c>
-      <c r="O91" t="s" s="2">
-        <v>680</v>
       </c>
       <c r="P91" t="s" s="2">
         <v>82</v>
@@ -14482,7 +14479,7 @@
         <v>82</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>83</v>
@@ -14509,16 +14506,16 @@
         <v>82</v>
       </c>
       <c r="AO91" t="s" s="2">
+        <v>681</v>
+      </c>
+      <c r="AP91" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ91" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR91" t="s" s="2">
         <v>682</v>
-      </c>
-      <c r="AP91" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ91" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR91" t="s" s="2">
-        <v>683</v>
       </c>
       <c r="AS91" t="s" s="2">
         <v>82</v>
@@ -14526,10 +14523,10 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
+        <v>683</v>
+      </c>
+      <c r="B92" t="s" s="2">
         <v>684</v>
-      </c>
-      <c r="B92" t="s" s="2">
-        <v>685</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -14653,10 +14650,10 @@
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
+        <v>685</v>
+      </c>
+      <c r="B93" t="s" s="2">
         <v>686</v>
-      </c>
-      <c r="B93" t="s" s="2">
-        <v>687</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -14782,10 +14779,10 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
+        <v>687</v>
+      </c>
+      <c r="B94" t="s" s="2">
         <v>688</v>
-      </c>
-      <c r="B94" t="s" s="2">
-        <v>689</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -14811,16 +14808,16 @@
         <v>140</v>
       </c>
       <c r="L94" t="s" s="2">
+        <v>689</v>
+      </c>
+      <c r="M94" t="s" s="2">
         <v>690</v>
       </c>
-      <c r="M94" t="s" s="2">
+      <c r="N94" t="s" s="2">
         <v>691</v>
       </c>
-      <c r="N94" t="s" s="2">
+      <c r="O94" t="s" s="2">
         <v>692</v>
-      </c>
-      <c r="O94" t="s" s="2">
-        <v>693</v>
       </c>
       <c r="P94" t="s" s="2">
         <v>82</v>
@@ -14830,46 +14827,46 @@
         <v>82</v>
       </c>
       <c r="S94" t="s" s="2">
+        <v>693</v>
+      </c>
+      <c r="T94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="U94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF94" t="s" s="2">
         <v>694</v>
-      </c>
-      <c r="T94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF94" t="s" s="2">
-        <v>695</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>83</v>
@@ -14896,16 +14893,16 @@
         <v>82</v>
       </c>
       <c r="AO94" t="s" s="2">
+        <v>695</v>
+      </c>
+      <c r="AP94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ94" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR94" t="s" s="2">
         <v>696</v>
-      </c>
-      <c r="AP94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ94" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR94" t="s" s="2">
-        <v>697</v>
       </c>
       <c r="AS94" t="s" s="2">
         <v>82</v>
@@ -14913,10 +14910,10 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
+        <v>697</v>
+      </c>
+      <c r="B95" t="s" s="2">
         <v>698</v>
-      </c>
-      <c r="B95" t="s" s="2">
-        <v>699</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -14942,13 +14939,13 @@
         <v>111</v>
       </c>
       <c r="L95" t="s" s="2">
+        <v>699</v>
+      </c>
+      <c r="M95" t="s" s="2">
         <v>700</v>
       </c>
-      <c r="M95" t="s" s="2">
+      <c r="N95" t="s" s="2">
         <v>701</v>
-      </c>
-      <c r="N95" t="s" s="2">
-        <v>702</v>
       </c>
       <c r="O95" s="2"/>
       <c r="P95" t="s" s="2">
@@ -14998,7 +14995,7 @@
         <v>82</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>83</v>
@@ -15025,16 +15022,16 @@
         <v>82</v>
       </c>
       <c r="AO95" t="s" s="2">
+        <v>703</v>
+      </c>
+      <c r="AP95" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ95" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR95" t="s" s="2">
         <v>704</v>
-      </c>
-      <c r="AP95" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ95" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR95" t="s" s="2">
-        <v>705</v>
       </c>
       <c r="AS95" t="s" s="2">
         <v>82</v>
@@ -15042,10 +15039,10 @@
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
+        <v>705</v>
+      </c>
+      <c r="B96" t="s" s="2">
         <v>706</v>
-      </c>
-      <c r="B96" t="s" s="2">
-        <v>707</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -15071,14 +15068,14 @@
         <v>175</v>
       </c>
       <c r="L96" t="s" s="2">
+        <v>707</v>
+      </c>
+      <c r="M96" t="s" s="2">
         <v>708</v>
-      </c>
-      <c r="M96" t="s" s="2">
-        <v>709</v>
       </c>
       <c r="N96" s="2"/>
       <c r="O96" t="s" s="2">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="P96" t="s" s="2">
         <v>82</v>
@@ -15127,7 +15124,7 @@
         <v>82</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>83</v>
@@ -15163,7 +15160,7 @@
         <v>82</v>
       </c>
       <c r="AR96" t="s" s="2">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="AS96" t="s" s="2">
         <v>82</v>
@@ -15171,10 +15168,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
+        <v>712</v>
+      </c>
+      <c r="B97" t="s" s="2">
         <v>713</v>
-      </c>
-      <c r="B97" t="s" s="2">
-        <v>714</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -15200,14 +15197,14 @@
         <v>111</v>
       </c>
       <c r="L97" t="s" s="2">
+        <v>714</v>
+      </c>
+      <c r="M97" t="s" s="2">
         <v>715</v>
-      </c>
-      <c r="M97" t="s" s="2">
-        <v>716</v>
       </c>
       <c r="N97" s="2"/>
       <c r="O97" t="s" s="2">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="P97" t="s" s="2">
         <v>82</v>
@@ -15256,7 +15253,7 @@
         <v>82</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>83</v>
@@ -15283,16 +15280,16 @@
         <v>82</v>
       </c>
       <c r="AO97" t="s" s="2">
+        <v>718</v>
+      </c>
+      <c r="AP97" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ97" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR97" t="s" s="2">
         <v>719</v>
-      </c>
-      <c r="AP97" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ97" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR97" t="s" s="2">
-        <v>720</v>
       </c>
       <c r="AS97" t="s" s="2">
         <v>82</v>
@@ -15300,10 +15297,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
+        <v>720</v>
+      </c>
+      <c r="B98" t="s" s="2">
         <v>721</v>
-      </c>
-      <c r="B98" t="s" s="2">
-        <v>722</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -15326,19 +15323,19 @@
         <v>98</v>
       </c>
       <c r="K98" t="s" s="2">
+        <v>722</v>
+      </c>
+      <c r="L98" t="s" s="2">
         <v>723</v>
       </c>
-      <c r="L98" t="s" s="2">
+      <c r="M98" t="s" s="2">
         <v>724</v>
       </c>
-      <c r="M98" t="s" s="2">
+      <c r="N98" t="s" s="2">
         <v>725</v>
       </c>
-      <c r="N98" t="s" s="2">
+      <c r="O98" t="s" s="2">
         <v>726</v>
-      </c>
-      <c r="O98" t="s" s="2">
-        <v>727</v>
       </c>
       <c r="P98" t="s" s="2">
         <v>82</v>
@@ -15387,7 +15384,7 @@
         <v>82</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>83</v>
@@ -15414,16 +15411,16 @@
         <v>82</v>
       </c>
       <c r="AO98" t="s" s="2">
+        <v>728</v>
+      </c>
+      <c r="AP98" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ98" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR98" t="s" s="2">
         <v>729</v>
-      </c>
-      <c r="AP98" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ98" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR98" t="s" s="2">
-        <v>730</v>
       </c>
       <c r="AS98" t="s" s="2">
         <v>82</v>
@@ -15431,10 +15428,10 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
+        <v>730</v>
+      </c>
+      <c r="B99" t="s" s="2">
         <v>731</v>
-      </c>
-      <c r="B99" t="s" s="2">
-        <v>732</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -15460,16 +15457,16 @@
         <v>111</v>
       </c>
       <c r="L99" t="s" s="2">
+        <v>732</v>
+      </c>
+      <c r="M99" t="s" s="2">
         <v>733</v>
       </c>
-      <c r="M99" t="s" s="2">
+      <c r="N99" t="s" s="2">
         <v>734</v>
       </c>
-      <c r="N99" t="s" s="2">
+      <c r="O99" t="s" s="2">
         <v>735</v>
-      </c>
-      <c r="O99" t="s" s="2">
-        <v>736</v>
       </c>
       <c r="P99" t="s" s="2">
         <v>82</v>
@@ -15518,7 +15515,7 @@
         <v>82</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>83</v>
@@ -15545,16 +15542,16 @@
         <v>82</v>
       </c>
       <c r="AO99" t="s" s="2">
+        <v>737</v>
+      </c>
+      <c r="AP99" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ99" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR99" t="s" s="2">
         <v>738</v>
-      </c>
-      <c r="AP99" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ99" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR99" t="s" s="2">
-        <v>739</v>
       </c>
       <c r="AS99" t="s" s="2">
         <v>82</v>
@@ -15562,10 +15559,10 @@
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
+        <v>739</v>
+      </c>
+      <c r="B100" t="s" s="2">
         <v>740</v>
-      </c>
-      <c r="B100" t="s" s="2">
-        <v>741</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -15591,16 +15588,16 @@
         <v>140</v>
       </c>
       <c r="L100" t="s" s="2">
+        <v>741</v>
+      </c>
+      <c r="M100" t="s" s="2">
         <v>742</v>
       </c>
-      <c r="M100" t="s" s="2">
+      <c r="N100" t="s" s="2">
         <v>743</v>
       </c>
-      <c r="N100" t="s" s="2">
+      <c r="O100" t="s" s="2">
         <v>744</v>
-      </c>
-      <c r="O100" t="s" s="2">
-        <v>745</v>
       </c>
       <c r="P100" t="s" s="2">
         <v>82</v>
@@ -15613,43 +15610,43 @@
         <v>82</v>
       </c>
       <c r="T100" t="s" s="2">
+        <v>745</v>
+      </c>
+      <c r="U100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF100" t="s" s="2">
         <v>746</v>
-      </c>
-      <c r="U100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF100" t="s" s="2">
-        <v>747</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>83</v>
@@ -15676,16 +15673,16 @@
         <v>82</v>
       </c>
       <c r="AO100" t="s" s="2">
+        <v>747</v>
+      </c>
+      <c r="AP100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ100" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR100" t="s" s="2">
         <v>748</v>
-      </c>
-      <c r="AP100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ100" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR100" t="s" s="2">
-        <v>749</v>
       </c>
       <c r="AS100" t="s" s="2">
         <v>82</v>
@@ -15693,10 +15690,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
+        <v>749</v>
+      </c>
+      <c r="B101" t="s" s="2">
         <v>750</v>
-      </c>
-      <c r="B101" t="s" s="2">
-        <v>751</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -15722,13 +15719,13 @@
         <v>111</v>
       </c>
       <c r="L101" t="s" s="2">
+        <v>751</v>
+      </c>
+      <c r="M101" t="s" s="2">
         <v>752</v>
       </c>
-      <c r="M101" t="s" s="2">
+      <c r="N101" t="s" s="2">
         <v>753</v>
-      </c>
-      <c r="N101" t="s" s="2">
-        <v>754</v>
       </c>
       <c r="O101" s="2"/>
       <c r="P101" t="s" s="2">
@@ -15742,43 +15739,43 @@
         <v>82</v>
       </c>
       <c r="T101" t="s" s="2">
+        <v>754</v>
+      </c>
+      <c r="U101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="V101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="W101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="X101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Y101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="Z101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AA101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AB101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AC101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AD101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AE101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AF101" t="s" s="2">
         <v>755</v>
-      </c>
-      <c r="U101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF101" t="s" s="2">
-        <v>756</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>83</v>
@@ -15805,16 +15802,16 @@
         <v>82</v>
       </c>
       <c r="AO101" t="s" s="2">
+        <v>756</v>
+      </c>
+      <c r="AP101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ101" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR101" t="s" s="2">
         <v>757</v>
-      </c>
-      <c r="AP101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ101" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR101" t="s" s="2">
-        <v>758</v>
       </c>
       <c r="AS101" t="s" s="2">
         <v>82</v>
@@ -15822,10 +15819,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
+        <v>758</v>
+      </c>
+      <c r="B102" t="s" s="2">
         <v>759</v>
-      </c>
-      <c r="B102" t="s" s="2">
-        <v>760</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -15848,13 +15845,13 @@
         <v>98</v>
       </c>
       <c r="K102" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="L102" t="s" s="2">
+        <v>760</v>
+      </c>
+      <c r="M102" t="s" s="2">
         <v>761</v>
-      </c>
-      <c r="M102" t="s" s="2">
-        <v>762</v>
       </c>
       <c r="N102" s="2"/>
       <c r="O102" s="2"/>
@@ -15905,7 +15902,7 @@
         <v>82</v>
       </c>
       <c r="AF102" t="s" s="2">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="AG102" t="s" s="2">
         <v>83</v>
@@ -15932,16 +15929,16 @@
         <v>82</v>
       </c>
       <c r="AO102" t="s" s="2">
+        <v>763</v>
+      </c>
+      <c r="AP102" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ102" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR102" t="s" s="2">
         <v>764</v>
-      </c>
-      <c r="AP102" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ102" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR102" t="s" s="2">
-        <v>765</v>
       </c>
       <c r="AS102" t="s" s="2">
         <v>82</v>
@@ -15949,10 +15946,10 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
+        <v>765</v>
+      </c>
+      <c r="B103" t="s" s="2">
         <v>766</v>
-      </c>
-      <c r="B103" t="s" s="2">
-        <v>767</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -15978,13 +15975,13 @@
         <v>333</v>
       </c>
       <c r="L103" t="s" s="2">
+        <v>767</v>
+      </c>
+      <c r="M103" t="s" s="2">
         <v>768</v>
       </c>
-      <c r="M103" t="s" s="2">
+      <c r="N103" t="s" s="2">
         <v>769</v>
-      </c>
-      <c r="N103" t="s" s="2">
-        <v>770</v>
       </c>
       <c r="O103" s="2"/>
       <c r="P103" t="s" s="2">
@@ -16034,7 +16031,7 @@
         <v>82</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>83</v>
@@ -16061,16 +16058,16 @@
         <v>82</v>
       </c>
       <c r="AO103" t="s" s="2">
+        <v>771</v>
+      </c>
+      <c r="AP103" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AQ103" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AR103" t="s" s="2">
         <v>772</v>
-      </c>
-      <c r="AP103" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AQ103" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AR103" t="s" s="2">
-        <v>773</v>
       </c>
       <c r="AS103" t="s" s="2">
         <v>82</v>
@@ -16078,10 +16075,10 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
+        <v>773</v>
+      </c>
+      <c r="B104" t="s" s="2">
         <v>774</v>
-      </c>
-      <c r="B104" t="s" s="2">
-        <v>775</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -16107,13 +16104,13 @@
         <v>111</v>
       </c>
       <c r="L104" t="s" s="2">
+        <v>617</v>
+      </c>
+      <c r="M104" t="s" s="2">
         <v>618</v>
       </c>
-      <c r="M104" t="s" s="2">
+      <c r="N104" t="s" s="2">
         <v>619</v>
-      </c>
-      <c r="N104" t="s" s="2">
-        <v>620</v>
       </c>
       <c r="O104" s="2"/>
       <c r="P104" t="s" s="2">
@@ -16163,7 +16160,7 @@
         <v>82</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>83</v>

</xml_diff>

<commit_message>
Apply suggestion from @aperie07
Co-authored-by: aperie07 <99648638+aperie07@users.noreply.github.com> e3b314c48d7355ff5e36530b7a2a59fa8ddc7de9
</commit_message>
<xml_diff>
--- a/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/nr-securitylabel-slicing-123/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-06T14:05:46+00:00</t>
+    <t>2026-08-06T14:06:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1251,7 +1251,7 @@
 </t>
   </si>
   <si>
-    <t>Slice sur securityLabel pour distinguer le niveau de confidentialité (NRV) du statut de visibilité complémentaire (TRE A07) : chaque slice est discriminée par son required binding sur un ValueSet fermé (v3-ConfidentialityClassification pour confidentiality, JDV_J110-StatutVisibiliteDocument-CISIS pour visibilityStatus)</t>
+    <t>Slice sur securityLabel pour distinguer le niveau de confidentialité (U, L, M, N, R, V) du statut de visibilité (MASQUE_PS, INVISIBLE_PATIENT, etc...) : chaque slice est discriminée par son required binding sur un ValueSet fermé (v3-ConfidentialityClassification pour confidentiality, JDV_J110-StatutVisibiliteDocument-CISIS pour visibilityStatus)</t>
   </si>
   <si>
     <t>niveauConfidentialite : [0..*] code</t>
@@ -2780,7 +2780,7 @@
     <col min="26" max="26" width="102.93359375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
-    <col min="29" max="29" width="249.46875" customWidth="true" bestFit="true"/>
+    <col min="29" max="29" width="255.0" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="32" max="32" width="37.78125" customWidth="true" bestFit="true" hidden="true"/>

</xml_diff>